<commit_message>
Final renaming in templates
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11008"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\ahernandez\repos\aspect\api\templates\xpert_site_summary_report\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_and_site_summary_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1FC26ABA-9387-4DD5-8D3D-A94150437884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D72F13-2304-2E48-B9C1-2B12DDAA6C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="760" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Xpert Site Summary Report" sheetId="1" r:id="rId1"/>
-    <sheet name="Xpert Site Inventory" sheetId="2" r:id="rId2"/>
-    <sheet name="Xpert Site Errors by Device" sheetId="3" r:id="rId3"/>
+    <sheet name="Device and Site Summary Report" sheetId="1" r:id="rId1"/>
+    <sheet name="Device and Site Inventory" sheetId="2" r:id="rId2"/>
+    <sheet name="Errors by Device" sheetId="3" r:id="rId3"/>
     <sheet name="Error Codes" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -371,15 +371,6 @@
     <t>Last Result Update</t>
   </si>
   <si>
-    <t>Xpert Site Summary Report</t>
-  </si>
-  <si>
-    <t>Xpert Site Inventory</t>
-  </si>
-  <si>
-    <t>Xpert Site Errors by Devices</t>
-  </si>
-  <si>
     <r>
       <t xml:space="preserve">Note:
 </t>
@@ -398,6 +389,15 @@
   </si>
   <si>
     <t>Note: this report only includes the consumables that were sometime tracked on the sites</t>
+  </si>
+  <si>
+    <t>Device and Site Summary Report</t>
+  </si>
+  <si>
+    <t>Device and Site Inventory</t>
+  </si>
+  <si>
+    <t>Errors by Device</t>
   </si>
 </sst>
 </file>
@@ -575,6 +575,9 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -585,9 +588,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -972,88 +972,88 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:T11"/>
-  <sheetFormatPr defaultColWidth="11.125" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="15.125" customWidth="1"/>
-    <col min="5" max="5" width="31.125" customWidth="1"/>
+    <col min="4" max="4" width="15.1640625" customWidth="1"/>
+    <col min="5" max="5" width="31.1640625" customWidth="1"/>
     <col min="6" max="9" width="19" customWidth="1"/>
-    <col min="10" max="10" width="14.625" style="3" customWidth="1"/>
-    <col min="11" max="11" width="14.375" style="4" customWidth="1"/>
-    <col min="12" max="14" width="14.375" style="3" customWidth="1"/>
-    <col min="15" max="15" width="13.125" style="3" customWidth="1"/>
+    <col min="10" max="10" width="14.6640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="14.33203125" style="4" customWidth="1"/>
+    <col min="12" max="14" width="14.33203125" style="3" customWidth="1"/>
+    <col min="15" max="15" width="13.1640625" style="3" customWidth="1"/>
     <col min="16" max="16" width="10.5" style="3" customWidth="1"/>
-    <col min="17" max="17" width="18.125" style="3" customWidth="1"/>
+    <col min="17" max="17" width="18.1640625" style="3" customWidth="1"/>
     <col min="18" max="18" width="11" style="4" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="1015" max="1024" width="9.125" customWidth="1"/>
+    <col min="1015" max="1024" width="9.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
     </row>
-    <row r="2" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="F2" s="28"/>
-      <c r="G2" s="28"/>
+      <c r="E2" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
       <c r="H2" s="22"/>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
       <c r="C3" s="23"/>
       <c r="D3" s="23"/>
-      <c r="E3" s="28"/>
-      <c r="F3" s="28"/>
-      <c r="G3" s="28"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
       <c r="H3" s="22"/>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="28"/>
-      <c r="F4" s="28"/>
-      <c r="G4" s="28"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="24"/>
       <c r="H4" s="22"/>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="17" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="28"/>
-      <c r="F5" s="28"/>
-      <c r="G5" s="28"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
       <c r="H5" s="22"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="28"/>
-      <c r="F6" s="28"/>
-      <c r="G6" s="28"/>
-    </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="E6" s="24"/>
+      <c r="F6" s="24"/>
+      <c r="G6" s="24"/>
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="6"/>
     </row>
-    <row r="8" spans="1:20" s="10" customFormat="1" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" s="10" customFormat="1" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>6</v>
       </c>
@@ -1115,7 +1115,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>25</v>
       </c>
@@ -1177,7 +1177,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A11" s="16"/>
       <c r="B11" s="16"/>
       <c r="C11" s="16"/>
@@ -1201,68 +1201,68 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H9"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="21.625" customWidth="1"/>
-    <col min="2" max="2" width="17.375" customWidth="1"/>
-    <col min="3" max="3" width="21.75" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="27.375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.6640625" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" customWidth="1"/>
+    <col min="3" max="3" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.1640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="24" t="s">
-        <v>114</v>
-      </c>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-    </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C2" s="25" t="s">
+        <v>111</v>
+      </c>
+      <c r="D2" s="25"/>
+      <c r="E2" s="25"/>
+      <c r="F2" s="25"/>
+      <c r="G2" s="25"/>
+    </row>
+    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
       <c r="C6" s="7"/>
       <c r="D6" s="6"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>5</v>
       </c>
       <c r="C7" s="7"/>
       <c r="D7" s="6"/>
     </row>
-    <row r="8" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="8" t="s">
         <v>45</v>
       </c>
@@ -1288,7 +1288,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
       <c r="A9" s="11" t="s">
         <v>53</v>
       </c>
@@ -1326,46 +1326,46 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L10"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="33.125" customWidth="1"/>
-    <col min="2" max="9" width="8.625" style="3" customWidth="1"/>
-    <col min="10" max="10" width="12.125" style="3" customWidth="1"/>
-    <col min="11" max="11" width="14.125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="33.1640625" customWidth="1"/>
+    <col min="2" max="9" width="8.6640625" style="3" customWidth="1"/>
+    <col min="10" max="10" width="12.1640625" style="3" customWidth="1"/>
+    <col min="11" max="11" width="14.1640625" style="3" customWidth="1"/>
     <col min="12" max="12" width="15.5" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:12" ht="17" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
         <v>5</v>
       </c>
@@ -1373,30 +1373,30 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="25" t="s">
+    <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="27" t="s">
         <v>61</v>
       </c>
-      <c r="C8" s="26"/>
-      <c r="D8" s="26"/>
-      <c r="E8" s="26"/>
-      <c r="F8" s="26"/>
-      <c r="G8" s="26"/>
-      <c r="H8" s="26"/>
-      <c r="I8" s="26"/>
-      <c r="J8" s="26"/>
-      <c r="K8" s="27" t="s">
+      <c r="C8" s="27"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="27"/>
+      <c r="G8" s="27"/>
+      <c r="H8" s="27"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="28" t="s">
         <v>62</v>
       </c>
-      <c r="L8" s="27" t="s">
+      <c r="L8" s="28" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="25"/>
+    <row r="9" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="26"/>
       <c r="B9" s="1">
         <v>5011</v>
       </c>
@@ -1424,10 +1424,10 @@
       <c r="J9" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="K9" s="27"/>
-      <c r="L9" s="27"/>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="K9" s="28"/>
+      <c r="L9" s="28"/>
+    </row>
+    <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="2" t="s">
         <v>65</v>
       </c>
@@ -1481,14 +1481,14 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.125" customWidth="1"/>
-    <col min="2" max="2" width="39.125" customWidth="1"/>
-    <col min="3" max="3" width="100.625" customWidth="1"/>
+    <col min="1" max="1" width="5.1640625" customWidth="1"/>
+    <col min="2" max="2" width="39.1640625" customWidth="1"/>
+    <col min="3" max="3" width="100.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="16" t="s">
         <v>76</v>
       </c>
@@ -1499,7 +1499,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="19">
         <v>1001</v>
       </c>
@@ -1510,7 +1510,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="19">
         <v>1002</v>
       </c>
@@ -1521,7 +1521,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="19">
         <v>1004</v>
       </c>
@@ -1532,7 +1532,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="19">
         <v>1005</v>
       </c>
@@ -1543,7 +1543,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="19">
         <v>1006</v>
       </c>
@@ -1554,7 +1554,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="19">
         <v>1007</v>
       </c>
@@ -1565,7 +1565,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="19">
         <v>1017</v>
       </c>
@@ -1576,7 +1576,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="19">
         <v>1018</v>
       </c>
@@ -1587,7 +1587,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="19">
         <v>2003</v>
       </c>
@@ -1598,7 +1598,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="19">
         <v>2005</v>
       </c>
@@ -1609,7 +1609,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="19">
         <v>2008</v>
       </c>
@@ -1620,7 +1620,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="19">
         <v>2009</v>
       </c>
@@ -1631,7 +1631,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="19">
         <v>2011</v>
       </c>
@@ -1642,7 +1642,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="19">
         <v>2014</v>
       </c>
@@ -1653,7 +1653,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="19">
         <v>2016</v>
       </c>
@@ -1664,7 +1664,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="19">
         <v>2018</v>
       </c>
@@ -1675,7 +1675,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="19">
         <v>2022</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="19">
         <v>2025</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="19">
         <v>2032</v>
       </c>
@@ -1708,7 +1708,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="19">
         <v>2034</v>
       </c>
@@ -1719,7 +1719,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="19">
         <v>2037</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="19">
         <v>4010</v>
       </c>
@@ -1741,7 +1741,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="19">
         <v>4017</v>
       </c>
@@ -1752,7 +1752,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="19">
         <v>5006</v>
       </c>
@@ -1763,7 +1763,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="19">
         <v>5007</v>
       </c>
@@ -1774,7 +1774,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="19">
         <v>5011</v>
       </c>

</xml_diff>

<commit_message>
removed a genXpert text from the report templates
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_and_site_summary_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D72F13-2304-2E48-B9C1-2B12DDAA6C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60241C67-1345-9C46-B5F5-0C29D521269B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="760" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4360" yWindow="760" windowWidth="29040" windowHeight="16440" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Device and Site Summary Report" sheetId="1" r:id="rId1"/>
@@ -371,6 +371,18 @@
     <t>Last Result Update</t>
   </si>
   <si>
+    <t>Note: this report only includes the consumables that were sometime tracked on the sites</t>
+  </si>
+  <si>
+    <t>Device and Site Summary Report</t>
+  </si>
+  <si>
+    <t>Device and Site Inventory</t>
+  </si>
+  <si>
+    <t>Errors by Device</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Note:
 </t>
@@ -384,20 +396,8 @@
         <family val="2"/>
         <charset val="1"/>
       </rPr>
-      <t>The result categories are represented by all the possible result combinations that GeneXpert sends to Aspect. For example, MTB Detected does not include MTB Detected Rif Detected, as they are considered different results</t>
+      <t>The result categories are represented by all the possible result combinations that the device sends to Aspect. For example, MTB Detected does not include MTB Detected Rif Detected, as they are considered different results</t>
     </r>
-  </si>
-  <si>
-    <t>Note: this report only includes the consumables that were sometime tracked on the sites</t>
-  </si>
-  <si>
-    <t>Device and Site Summary Report</t>
-  </si>
-  <si>
-    <t>Device and Site Inventory</t>
-  </si>
-  <si>
-    <t>Errors by Device</t>
   </si>
 </sst>
 </file>
@@ -991,7 +991,7 @@
   <sheetData>
     <row r="1" spans="1:20" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1003,7 +1003,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="F2" s="24"/>
       <c r="G2" s="24"/>
@@ -1215,7 +1215,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="17" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1226,7 +1226,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D2" s="25"/>
       <c r="E2" s="25"/>
@@ -1337,7 +1337,7 @@
   <sheetData>
     <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
[feat/ASP-6682-Device-and-Site-Summary-Report-Request-for-an-additional-sheet] fix: fixed default 0s and sheet
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -5873,7 +5873,7 @@
       <c r="A10" s="22" t="s">
         <v>90</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="32" t="s">
         <v>91</v>
       </c>
       <c r="C10" s="2" t="s">
@@ -5885,16 +5885,16 @@
       <c r="E10" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="F10" s="2" t="str">
-        <f>IF(C10=0,0,D10/C10)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G10" s="32" t="s">
+      <c r="F10" s="2">
+        <f>IFERROR(IF(A10="No data","",IF(C10=0,0,D10/C10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="33" t="str">
-        <f>IF(B10=0,0,G10/B10)</f>
-        <v>#VALUE!</v>
+      <c r="H10" s="33">
+        <f> IFERROR(IF(A10="No data","",IF(B10&lt;&gt;0, G10/B10, 0)),0)</f>
+        <v>0</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>95</v>
@@ -5902,25 +5902,25 @@
       <c r="J10" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="K10" s="2" t="str">
-        <f>U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L10" s="2" t="str">
-        <f>IF(G10=0,0,I10/G10)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="M10" s="2" t="str">
-        <f>IF(G10=0,0,J10/G10)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="N10" s="2" t="str">
-        <f>IF(D10=0,0,I10/D10)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="O10" s="2" t="str">
-        <f>IF(G10=0,0,K10/G10)</f>
-        <v>#VALUE!</v>
+      <c r="K10" s="2">
+        <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
+        <v>0</v>
+      </c>
+      <c r="L10" s="2">
+        <f>IFERROR(IF(A10="No data","",IF(G10=0,0,I10/G10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="2">
+        <f>IFERROR(IF(A10="No data","",IF(G10=0,0,J10/G10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="N10" s="2">
+        <f>IFERROR(IF(A10="No data","",IF(D10=0,0,I10/D10)),0)</f>
+        <v>0</v>
+      </c>
+      <c r="O10" s="2">
+        <f>IFERROR(IF(A10="No data","",IF(G10=0,0,K10/G10)),0)</f>
+        <v>0</v>
       </c>
       <c r="P10" s="2" t="s">
         <v>97</v>
@@ -5931,9 +5931,9 @@
       <c r="R10" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="S10" s="2" t="str">
-        <f>IF(I10=0,0,R10/I10)</f>
-        <v>#VALUE!</v>
+      <c r="S10" s="2">
+        <f>IFERROR(IF(A10="No data","",IF(I10=0,0,R10/I10)),0)</f>
+        <v>0</v>
       </c>
       <c r="T10" s="2" t="s">
         <v>100</v>
@@ -5968,9 +5968,9 @@
       <c r="AD10" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="AE10" s="2" t="str">
-        <f>U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10</f>
-        <v>#VALUE!</v>
+      <c r="AE10" s="2">
+        <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="11" ht="15.75" customHeight="1">

</xml_diff>

<commit_message>
[feat/ASP-6682-Device-and-Site-Summary-Report-Request-for-an-additional-sheet] fix: added extra columns for No result and added Trace detected for
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="203" uniqueCount="148">
   <si>
     <t>Device and Site Summary Report</t>
   </si>
@@ -302,7 +302,10 @@
     <t>Type of error</t>
   </si>
   <si>
-    <t>Invalid results</t>
+    <t>Invalid Results</t>
+  </si>
+  <si>
+    <t>No Results</t>
   </si>
   <si>
     <t>Total errors, invalid results, no results</t>
@@ -372,6 +375,9 @@
   </si>
   <si>
     <t>&lt;invalidResults&gt;</t>
+  </si>
+  <si>
+    <t>&lt;noResults&gt;</t>
   </si>
   <si>
     <t>Errors by Device</t>
@@ -643,7 +649,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -714,20 +720,23 @@
     <xf borderId="6" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="8" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="2" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center"/>
+    <xf borderId="4" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -5475,7 +5484,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="33.11"/>
     <col customWidth="1" min="2" max="2" width="8.56"/>
-    <col customWidth="1" min="3" max="3" width="9.89"/>
+    <col customWidth="1" min="3" max="3" width="12.67"/>
     <col customWidth="1" min="4" max="4" width="7.33"/>
     <col customWidth="1" min="5" max="5" width="12.44"/>
     <col customWidth="1" min="6" max="6" width="13.44"/>
@@ -5492,8 +5501,8 @@
     <col customWidth="1" min="18" max="20" width="12.56"/>
     <col customWidth="1" min="21" max="28" width="8.67"/>
     <col customWidth="1" min="29" max="29" width="12.11"/>
-    <col customWidth="1" min="30" max="30" width="14.11"/>
-    <col customWidth="1" min="31" max="31" width="15.44"/>
+    <col customWidth="1" min="30" max="31" width="14.11"/>
+    <col customWidth="1" min="32" max="32" width="15.44"/>
   </cols>
   <sheetData>
     <row r="1" ht="21.75" customHeight="1">
@@ -5530,6 +5539,7 @@
       <c r="AC1" s="2"/>
       <c r="AD1" s="2"/>
       <c r="AE1" s="2"/>
+      <c r="AF1" s="2"/>
     </row>
     <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="4" t="s">
@@ -5565,6 +5575,7 @@
       <c r="AC2" s="2"/>
       <c r="AD2" s="2"/>
       <c r="AE2" s="2"/>
+      <c r="AF2" s="2"/>
     </row>
     <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="4" t="s">
@@ -5600,6 +5611,7 @@
       <c r="AC3" s="2"/>
       <c r="AD3" s="2"/>
       <c r="AE3" s="2"/>
+      <c r="AF3" s="2"/>
     </row>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="22" t="s">
@@ -5635,6 +5647,7 @@
       <c r="AC4" s="2"/>
       <c r="AD4" s="2"/>
       <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
     </row>
     <row r="5" ht="15.75" customHeight="1">
       <c r="A5" s="22"/>
@@ -5668,6 +5681,7 @@
       <c r="AC5" s="2"/>
       <c r="AD5" s="2"/>
       <c r="AE5" s="2"/>
+      <c r="AF5" s="2"/>
     </row>
     <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="4"/>
@@ -5701,6 +5715,7 @@
       <c r="AC6" s="2"/>
       <c r="AD6" s="2"/>
       <c r="AE6" s="2"/>
+      <c r="AF6" s="2"/>
     </row>
     <row r="7" ht="15.75" customHeight="1">
       <c r="A7" s="23" t="s">
@@ -5738,6 +5753,7 @@
       <c r="AC7" s="2"/>
       <c r="AD7" s="2"/>
       <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
       <c r="A8" s="24" t="s">
@@ -5816,6 +5832,9 @@
       </c>
       <c r="AE8" s="29" t="s">
         <v>88</v>
+      </c>
+      <c r="AF8" s="24" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1">
@@ -5864,26 +5883,27 @@
         <v>2022.0</v>
       </c>
       <c r="AC9" s="31" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AD9" s="30"/>
       <c r="AE9" s="30"/>
+      <c r="AF9" s="30"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="22" t="s">
-        <v>90</v>
-      </c>
-      <c r="B10" s="32" t="s">
         <v>91</v>
       </c>
+      <c r="B10" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="C10" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F10" s="2">
         <f>IFERROR(IF(A10="No data","",IF(C10=0,0,D10/C10)),0)</f>
@@ -5892,18 +5912,18 @@
       <c r="G10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="33">
+      <c r="H10" s="32">
         <f> IFERROR(IF(A10="No data","",IF(B10&lt;&gt;0, G10/B10, 0)),0)</f>
         <v>0</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="K10" s="2">
-        <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
+        <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10+AE10),0)</f>
         <v>0</v>
       </c>
       <c r="L10" s="2">
@@ -5923,53 +5943,56 @@
         <v>0</v>
       </c>
       <c r="P10" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="Q10" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="R10" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="S10" s="2">
         <f>IFERROR(IF(A10="No data","",IF(I10=0,0,R10/I10)),0)</f>
         <v>0</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="V10" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="W10" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="X10" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="Y10" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="Z10" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="AA10" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="AB10" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AC10" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="AD10" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="AE10" s="2">
-        <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
+        <v>111</v>
+      </c>
+      <c r="AE10" s="33" t="s">
+        <v>112</v>
+      </c>
+      <c r="AF10" s="2">
+        <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10+AE10),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -6004,6 +6027,7 @@
       <c r="AC11" s="2"/>
       <c r="AD11" s="2"/>
       <c r="AE11" s="2"/>
+      <c r="AF11" s="2"/>
     </row>
     <row r="12" ht="15.75" customHeight="1">
       <c r="B12" s="2"/>
@@ -6036,6 +6060,7 @@
       <c r="AC12" s="2"/>
       <c r="AD12" s="2"/>
       <c r="AE12" s="2"/>
+      <c r="AF12" s="2"/>
     </row>
     <row r="13" ht="15.75" customHeight="1">
       <c r="B13" s="2"/>
@@ -6068,6 +6093,7 @@
       <c r="AC13" s="2"/>
       <c r="AD13" s="2"/>
       <c r="AE13" s="2"/>
+      <c r="AF13" s="2"/>
     </row>
     <row r="14" ht="15.75" customHeight="1">
       <c r="B14" s="2"/>
@@ -6100,6 +6126,7 @@
       <c r="AC14" s="2"/>
       <c r="AD14" s="2"/>
       <c r="AE14" s="2"/>
+      <c r="AF14" s="2"/>
     </row>
     <row r="15" ht="15.75" customHeight="1">
       <c r="B15" s="2"/>
@@ -6132,6 +6159,7 @@
       <c r="AC15" s="2"/>
       <c r="AD15" s="2"/>
       <c r="AE15" s="2"/>
+      <c r="AF15" s="2"/>
     </row>
     <row r="16" ht="15.75" customHeight="1">
       <c r="B16" s="2"/>
@@ -6164,6 +6192,7 @@
       <c r="AC16" s="2"/>
       <c r="AD16" s="2"/>
       <c r="AE16" s="2"/>
+      <c r="AF16" s="2"/>
     </row>
     <row r="17" ht="15.75" customHeight="1">
       <c r="B17" s="2"/>
@@ -6196,6 +6225,7 @@
       <c r="AC17" s="2"/>
       <c r="AD17" s="2"/>
       <c r="AE17" s="2"/>
+      <c r="AF17" s="2"/>
     </row>
     <row r="18" ht="15.75" customHeight="1">
       <c r="B18" s="2"/>
@@ -6228,6 +6258,7 @@
       <c r="AC18" s="2"/>
       <c r="AD18" s="2"/>
       <c r="AE18" s="2"/>
+      <c r="AF18" s="2"/>
     </row>
     <row r="19" ht="15.75" customHeight="1">
       <c r="B19" s="2"/>
@@ -6260,6 +6291,7 @@
       <c r="AC19" s="2"/>
       <c r="AD19" s="2"/>
       <c r="AE19" s="2"/>
+      <c r="AF19" s="2"/>
     </row>
     <row r="20" ht="15.75" customHeight="1">
       <c r="B20" s="2"/>
@@ -6292,6 +6324,7 @@
       <c r="AC20" s="2"/>
       <c r="AD20" s="2"/>
       <c r="AE20" s="2"/>
+      <c r="AF20" s="2"/>
     </row>
     <row r="21" ht="15.75" customHeight="1">
       <c r="B21" s="2"/>
@@ -6324,6 +6357,7 @@
       <c r="AC21" s="2"/>
       <c r="AD21" s="2"/>
       <c r="AE21" s="2"/>
+      <c r="AF21" s="2"/>
     </row>
     <row r="22" ht="15.75" customHeight="1">
       <c r="B22" s="2"/>
@@ -6356,6 +6390,7 @@
       <c r="AC22" s="2"/>
       <c r="AD22" s="2"/>
       <c r="AE22" s="2"/>
+      <c r="AF22" s="2"/>
     </row>
     <row r="23" ht="15.75" customHeight="1">
       <c r="B23" s="2"/>
@@ -6388,6 +6423,7 @@
       <c r="AC23" s="2"/>
       <c r="AD23" s="2"/>
       <c r="AE23" s="2"/>
+      <c r="AF23" s="2"/>
     </row>
     <row r="24" ht="15.75" customHeight="1">
       <c r="B24" s="2"/>
@@ -6420,6 +6456,7 @@
       <c r="AC24" s="2"/>
       <c r="AD24" s="2"/>
       <c r="AE24" s="2"/>
+      <c r="AF24" s="2"/>
     </row>
     <row r="25" ht="15.75" customHeight="1">
       <c r="B25" s="2"/>
@@ -6452,6 +6489,7 @@
       <c r="AC25" s="2"/>
       <c r="AD25" s="2"/>
       <c r="AE25" s="2"/>
+      <c r="AF25" s="2"/>
     </row>
     <row r="26" ht="15.75" customHeight="1">
       <c r="B26" s="2"/>
@@ -6484,6 +6522,7 @@
       <c r="AC26" s="2"/>
       <c r="AD26" s="2"/>
       <c r="AE26" s="2"/>
+      <c r="AF26" s="2"/>
     </row>
     <row r="27" ht="15.75" customHeight="1">
       <c r="B27" s="2"/>
@@ -6516,6 +6555,7 @@
       <c r="AC27" s="2"/>
       <c r="AD27" s="2"/>
       <c r="AE27" s="2"/>
+      <c r="AF27" s="2"/>
     </row>
     <row r="28" ht="15.75" customHeight="1">
       <c r="B28" s="2"/>
@@ -6548,6 +6588,7 @@
       <c r="AC28" s="2"/>
       <c r="AD28" s="2"/>
       <c r="AE28" s="2"/>
+      <c r="AF28" s="2"/>
     </row>
     <row r="29" ht="15.75" customHeight="1">
       <c r="B29" s="2"/>
@@ -6580,6 +6621,7 @@
       <c r="AC29" s="2"/>
       <c r="AD29" s="2"/>
       <c r="AE29" s="2"/>
+      <c r="AF29" s="2"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="B30" s="2"/>
@@ -6612,6 +6654,7 @@
       <c r="AC30" s="2"/>
       <c r="AD30" s="2"/>
       <c r="AE30" s="2"/>
+      <c r="AF30" s="2"/>
     </row>
     <row r="31" ht="15.75" customHeight="1">
       <c r="B31" s="2"/>
@@ -6644,6 +6687,7 @@
       <c r="AC31" s="2"/>
       <c r="AD31" s="2"/>
       <c r="AE31" s="2"/>
+      <c r="AF31" s="2"/>
     </row>
     <row r="32" ht="15.75" customHeight="1">
       <c r="B32" s="2"/>
@@ -6676,6 +6720,7 @@
       <c r="AC32" s="2"/>
       <c r="AD32" s="2"/>
       <c r="AE32" s="2"/>
+      <c r="AF32" s="2"/>
     </row>
     <row r="33" ht="15.75" customHeight="1">
       <c r="B33" s="2"/>
@@ -6708,6 +6753,7 @@
       <c r="AC33" s="2"/>
       <c r="AD33" s="2"/>
       <c r="AE33" s="2"/>
+      <c r="AF33" s="2"/>
     </row>
     <row r="34" ht="15.75" customHeight="1">
       <c r="B34" s="2"/>
@@ -6740,6 +6786,7 @@
       <c r="AC34" s="2"/>
       <c r="AD34" s="2"/>
       <c r="AE34" s="2"/>
+      <c r="AF34" s="2"/>
     </row>
     <row r="35" ht="15.75" customHeight="1">
       <c r="B35" s="2"/>
@@ -6772,6 +6819,7 @@
       <c r="AC35" s="2"/>
       <c r="AD35" s="2"/>
       <c r="AE35" s="2"/>
+      <c r="AF35" s="2"/>
     </row>
     <row r="36" ht="15.75" customHeight="1">
       <c r="B36" s="2"/>
@@ -6804,6 +6852,7 @@
       <c r="AC36" s="2"/>
       <c r="AD36" s="2"/>
       <c r="AE36" s="2"/>
+      <c r="AF36" s="2"/>
     </row>
     <row r="37" ht="15.75" customHeight="1">
       <c r="B37" s="2"/>
@@ -6836,6 +6885,7 @@
       <c r="AC37" s="2"/>
       <c r="AD37" s="2"/>
       <c r="AE37" s="2"/>
+      <c r="AF37" s="2"/>
     </row>
     <row r="38" ht="15.75" customHeight="1">
       <c r="B38" s="2"/>
@@ -6868,6 +6918,7 @@
       <c r="AC38" s="2"/>
       <c r="AD38" s="2"/>
       <c r="AE38" s="2"/>
+      <c r="AF38" s="2"/>
     </row>
     <row r="39" ht="15.75" customHeight="1">
       <c r="B39" s="2"/>
@@ -6900,6 +6951,7 @@
       <c r="AC39" s="2"/>
       <c r="AD39" s="2"/>
       <c r="AE39" s="2"/>
+      <c r="AF39" s="2"/>
     </row>
     <row r="40" ht="15.75" customHeight="1">
       <c r="B40" s="2"/>
@@ -6932,6 +6984,7 @@
       <c r="AC40" s="2"/>
       <c r="AD40" s="2"/>
       <c r="AE40" s="2"/>
+      <c r="AF40" s="2"/>
     </row>
     <row r="41" ht="15.75" customHeight="1">
       <c r="B41" s="2"/>
@@ -6964,6 +7017,7 @@
       <c r="AC41" s="2"/>
       <c r="AD41" s="2"/>
       <c r="AE41" s="2"/>
+      <c r="AF41" s="2"/>
     </row>
     <row r="42" ht="15.75" customHeight="1">
       <c r="B42" s="2"/>
@@ -6996,6 +7050,7 @@
       <c r="AC42" s="2"/>
       <c r="AD42" s="2"/>
       <c r="AE42" s="2"/>
+      <c r="AF42" s="2"/>
     </row>
     <row r="43" ht="15.75" customHeight="1">
       <c r="B43" s="2"/>
@@ -7028,6 +7083,7 @@
       <c r="AC43" s="2"/>
       <c r="AD43" s="2"/>
       <c r="AE43" s="2"/>
+      <c r="AF43" s="2"/>
     </row>
     <row r="44" ht="15.75" customHeight="1">
       <c r="B44" s="2"/>
@@ -7060,6 +7116,7 @@
       <c r="AC44" s="2"/>
       <c r="AD44" s="2"/>
       <c r="AE44" s="2"/>
+      <c r="AF44" s="2"/>
     </row>
     <row r="45" ht="15.75" customHeight="1">
       <c r="B45" s="2"/>
@@ -7092,6 +7149,7 @@
       <c r="AC45" s="2"/>
       <c r="AD45" s="2"/>
       <c r="AE45" s="2"/>
+      <c r="AF45" s="2"/>
     </row>
     <row r="46" ht="15.75" customHeight="1">
       <c r="B46" s="2"/>
@@ -7124,6 +7182,7 @@
       <c r="AC46" s="2"/>
       <c r="AD46" s="2"/>
       <c r="AE46" s="2"/>
+      <c r="AF46" s="2"/>
     </row>
     <row r="47" ht="15.75" customHeight="1">
       <c r="B47" s="2"/>
@@ -7156,6 +7215,7 @@
       <c r="AC47" s="2"/>
       <c r="AD47" s="2"/>
       <c r="AE47" s="2"/>
+      <c r="AF47" s="2"/>
     </row>
     <row r="48" ht="15.75" customHeight="1">
       <c r="B48" s="2"/>
@@ -7188,6 +7248,7 @@
       <c r="AC48" s="2"/>
       <c r="AD48" s="2"/>
       <c r="AE48" s="2"/>
+      <c r="AF48" s="2"/>
     </row>
     <row r="49" ht="15.75" customHeight="1">
       <c r="B49" s="2"/>
@@ -7220,6 +7281,7 @@
       <c r="AC49" s="2"/>
       <c r="AD49" s="2"/>
       <c r="AE49" s="2"/>
+      <c r="AF49" s="2"/>
     </row>
     <row r="50" ht="15.75" customHeight="1">
       <c r="B50" s="2"/>
@@ -7252,6 +7314,7 @@
       <c r="AC50" s="2"/>
       <c r="AD50" s="2"/>
       <c r="AE50" s="2"/>
+      <c r="AF50" s="2"/>
     </row>
     <row r="51" ht="15.75" customHeight="1">
       <c r="B51" s="2"/>
@@ -7284,6 +7347,7 @@
       <c r="AC51" s="2"/>
       <c r="AD51" s="2"/>
       <c r="AE51" s="2"/>
+      <c r="AF51" s="2"/>
     </row>
     <row r="52" ht="15.75" customHeight="1">
       <c r="B52" s="2"/>
@@ -7316,6 +7380,7 @@
       <c r="AC52" s="2"/>
       <c r="AD52" s="2"/>
       <c r="AE52" s="2"/>
+      <c r="AF52" s="2"/>
     </row>
     <row r="53" ht="15.75" customHeight="1">
       <c r="B53" s="2"/>
@@ -7348,6 +7413,7 @@
       <c r="AC53" s="2"/>
       <c r="AD53" s="2"/>
       <c r="AE53" s="2"/>
+      <c r="AF53" s="2"/>
     </row>
     <row r="54" ht="15.75" customHeight="1">
       <c r="B54" s="2"/>
@@ -7380,6 +7446,7 @@
       <c r="AC54" s="2"/>
       <c r="AD54" s="2"/>
       <c r="AE54" s="2"/>
+      <c r="AF54" s="2"/>
     </row>
     <row r="55" ht="15.75" customHeight="1">
       <c r="B55" s="2"/>
@@ -7412,6 +7479,7 @@
       <c r="AC55" s="2"/>
       <c r="AD55" s="2"/>
       <c r="AE55" s="2"/>
+      <c r="AF55" s="2"/>
     </row>
     <row r="56" ht="15.75" customHeight="1">
       <c r="B56" s="2"/>
@@ -7444,6 +7512,7 @@
       <c r="AC56" s="2"/>
       <c r="AD56" s="2"/>
       <c r="AE56" s="2"/>
+      <c r="AF56" s="2"/>
     </row>
     <row r="57" ht="15.75" customHeight="1">
       <c r="B57" s="2"/>
@@ -7476,6 +7545,7 @@
       <c r="AC57" s="2"/>
       <c r="AD57" s="2"/>
       <c r="AE57" s="2"/>
+      <c r="AF57" s="2"/>
     </row>
     <row r="58" ht="15.75" customHeight="1">
       <c r="B58" s="2"/>
@@ -7508,6 +7578,7 @@
       <c r="AC58" s="2"/>
       <c r="AD58" s="2"/>
       <c r="AE58" s="2"/>
+      <c r="AF58" s="2"/>
     </row>
     <row r="59" ht="15.75" customHeight="1">
       <c r="B59" s="2"/>
@@ -7540,6 +7611,7 @@
       <c r="AC59" s="2"/>
       <c r="AD59" s="2"/>
       <c r="AE59" s="2"/>
+      <c r="AF59" s="2"/>
     </row>
     <row r="60" ht="15.75" customHeight="1">
       <c r="B60" s="2"/>
@@ -7572,6 +7644,7 @@
       <c r="AC60" s="2"/>
       <c r="AD60" s="2"/>
       <c r="AE60" s="2"/>
+      <c r="AF60" s="2"/>
     </row>
     <row r="61" ht="15.75" customHeight="1">
       <c r="B61" s="2"/>
@@ -7604,6 +7677,7 @@
       <c r="AC61" s="2"/>
       <c r="AD61" s="2"/>
       <c r="AE61" s="2"/>
+      <c r="AF61" s="2"/>
     </row>
     <row r="62" ht="15.75" customHeight="1">
       <c r="B62" s="2"/>
@@ -7636,6 +7710,7 @@
       <c r="AC62" s="2"/>
       <c r="AD62" s="2"/>
       <c r="AE62" s="2"/>
+      <c r="AF62" s="2"/>
     </row>
     <row r="63" ht="15.75" customHeight="1">
       <c r="B63" s="2"/>
@@ -7668,6 +7743,7 @@
       <c r="AC63" s="2"/>
       <c r="AD63" s="2"/>
       <c r="AE63" s="2"/>
+      <c r="AF63" s="2"/>
     </row>
     <row r="64" ht="15.75" customHeight="1">
       <c r="B64" s="2"/>
@@ -7700,6 +7776,7 @@
       <c r="AC64" s="2"/>
       <c r="AD64" s="2"/>
       <c r="AE64" s="2"/>
+      <c r="AF64" s="2"/>
     </row>
     <row r="65" ht="15.75" customHeight="1">
       <c r="B65" s="2"/>
@@ -7732,6 +7809,7 @@
       <c r="AC65" s="2"/>
       <c r="AD65" s="2"/>
       <c r="AE65" s="2"/>
+      <c r="AF65" s="2"/>
     </row>
     <row r="66" ht="15.75" customHeight="1">
       <c r="B66" s="2"/>
@@ -7764,6 +7842,7 @@
       <c r="AC66" s="2"/>
       <c r="AD66" s="2"/>
       <c r="AE66" s="2"/>
+      <c r="AF66" s="2"/>
     </row>
     <row r="67" ht="15.75" customHeight="1">
       <c r="B67" s="2"/>
@@ -7796,6 +7875,7 @@
       <c r="AC67" s="2"/>
       <c r="AD67" s="2"/>
       <c r="AE67" s="2"/>
+      <c r="AF67" s="2"/>
     </row>
     <row r="68" ht="15.75" customHeight="1">
       <c r="B68" s="2"/>
@@ -7828,6 +7908,7 @@
       <c r="AC68" s="2"/>
       <c r="AD68" s="2"/>
       <c r="AE68" s="2"/>
+      <c r="AF68" s="2"/>
     </row>
     <row r="69" ht="15.75" customHeight="1">
       <c r="B69" s="2"/>
@@ -7860,6 +7941,7 @@
       <c r="AC69" s="2"/>
       <c r="AD69" s="2"/>
       <c r="AE69" s="2"/>
+      <c r="AF69" s="2"/>
     </row>
     <row r="70" ht="15.75" customHeight="1">
       <c r="B70" s="2"/>
@@ -7892,6 +7974,7 @@
       <c r="AC70" s="2"/>
       <c r="AD70" s="2"/>
       <c r="AE70" s="2"/>
+      <c r="AF70" s="2"/>
     </row>
     <row r="71" ht="15.75" customHeight="1">
       <c r="B71" s="2"/>
@@ -7924,6 +8007,7 @@
       <c r="AC71" s="2"/>
       <c r="AD71" s="2"/>
       <c r="AE71" s="2"/>
+      <c r="AF71" s="2"/>
     </row>
     <row r="72" ht="15.75" customHeight="1">
       <c r="B72" s="2"/>
@@ -7956,6 +8040,7 @@
       <c r="AC72" s="2"/>
       <c r="AD72" s="2"/>
       <c r="AE72" s="2"/>
+      <c r="AF72" s="2"/>
     </row>
     <row r="73" ht="15.75" customHeight="1">
       <c r="B73" s="2"/>
@@ -7988,6 +8073,7 @@
       <c r="AC73" s="2"/>
       <c r="AD73" s="2"/>
       <c r="AE73" s="2"/>
+      <c r="AF73" s="2"/>
     </row>
     <row r="74" ht="15.75" customHeight="1">
       <c r="B74" s="2"/>
@@ -8020,6 +8106,7 @@
       <c r="AC74" s="2"/>
       <c r="AD74" s="2"/>
       <c r="AE74" s="2"/>
+      <c r="AF74" s="2"/>
     </row>
     <row r="75" ht="15.75" customHeight="1">
       <c r="B75" s="2"/>
@@ -8052,6 +8139,7 @@
       <c r="AC75" s="2"/>
       <c r="AD75" s="2"/>
       <c r="AE75" s="2"/>
+      <c r="AF75" s="2"/>
     </row>
     <row r="76" ht="15.75" customHeight="1">
       <c r="B76" s="2"/>
@@ -8084,6 +8172,7 @@
       <c r="AC76" s="2"/>
       <c r="AD76" s="2"/>
       <c r="AE76" s="2"/>
+      <c r="AF76" s="2"/>
     </row>
     <row r="77" ht="15.75" customHeight="1">
       <c r="B77" s="2"/>
@@ -8116,6 +8205,7 @@
       <c r="AC77" s="2"/>
       <c r="AD77" s="2"/>
       <c r="AE77" s="2"/>
+      <c r="AF77" s="2"/>
     </row>
     <row r="78" ht="15.75" customHeight="1">
       <c r="B78" s="2"/>
@@ -8148,6 +8238,7 @@
       <c r="AC78" s="2"/>
       <c r="AD78" s="2"/>
       <c r="AE78" s="2"/>
+      <c r="AF78" s="2"/>
     </row>
     <row r="79" ht="15.75" customHeight="1">
       <c r="B79" s="2"/>
@@ -8180,6 +8271,7 @@
       <c r="AC79" s="2"/>
       <c r="AD79" s="2"/>
       <c r="AE79" s="2"/>
+      <c r="AF79" s="2"/>
     </row>
     <row r="80" ht="15.75" customHeight="1">
       <c r="B80" s="2"/>
@@ -8212,6 +8304,7 @@
       <c r="AC80" s="2"/>
       <c r="AD80" s="2"/>
       <c r="AE80" s="2"/>
+      <c r="AF80" s="2"/>
     </row>
     <row r="81" ht="15.75" customHeight="1">
       <c r="B81" s="2"/>
@@ -8244,6 +8337,7 @@
       <c r="AC81" s="2"/>
       <c r="AD81" s="2"/>
       <c r="AE81" s="2"/>
+      <c r="AF81" s="2"/>
     </row>
     <row r="82" ht="15.75" customHeight="1">
       <c r="B82" s="2"/>
@@ -8276,6 +8370,7 @@
       <c r="AC82" s="2"/>
       <c r="AD82" s="2"/>
       <c r="AE82" s="2"/>
+      <c r="AF82" s="2"/>
     </row>
     <row r="83" ht="15.75" customHeight="1">
       <c r="B83" s="2"/>
@@ -8308,6 +8403,7 @@
       <c r="AC83" s="2"/>
       <c r="AD83" s="2"/>
       <c r="AE83" s="2"/>
+      <c r="AF83" s="2"/>
     </row>
     <row r="84" ht="15.75" customHeight="1">
       <c r="B84" s="2"/>
@@ -8340,6 +8436,7 @@
       <c r="AC84" s="2"/>
       <c r="AD84" s="2"/>
       <c r="AE84" s="2"/>
+      <c r="AF84" s="2"/>
     </row>
     <row r="85" ht="15.75" customHeight="1">
       <c r="B85" s="2"/>
@@ -8372,6 +8469,7 @@
       <c r="AC85" s="2"/>
       <c r="AD85" s="2"/>
       <c r="AE85" s="2"/>
+      <c r="AF85" s="2"/>
     </row>
     <row r="86" ht="15.75" customHeight="1">
       <c r="B86" s="2"/>
@@ -8404,6 +8502,7 @@
       <c r="AC86" s="2"/>
       <c r="AD86" s="2"/>
       <c r="AE86" s="2"/>
+      <c r="AF86" s="2"/>
     </row>
     <row r="87" ht="15.75" customHeight="1">
       <c r="B87" s="2"/>
@@ -8436,6 +8535,7 @@
       <c r="AC87" s="2"/>
       <c r="AD87" s="2"/>
       <c r="AE87" s="2"/>
+      <c r="AF87" s="2"/>
     </row>
     <row r="88" ht="15.75" customHeight="1">
       <c r="B88" s="2"/>
@@ -8468,6 +8568,7 @@
       <c r="AC88" s="2"/>
       <c r="AD88" s="2"/>
       <c r="AE88" s="2"/>
+      <c r="AF88" s="2"/>
     </row>
     <row r="89" ht="15.75" customHeight="1">
       <c r="B89" s="2"/>
@@ -8500,6 +8601,7 @@
       <c r="AC89" s="2"/>
       <c r="AD89" s="2"/>
       <c r="AE89" s="2"/>
+      <c r="AF89" s="2"/>
     </row>
     <row r="90" ht="15.75" customHeight="1">
       <c r="B90" s="2"/>
@@ -8532,6 +8634,7 @@
       <c r="AC90" s="2"/>
       <c r="AD90" s="2"/>
       <c r="AE90" s="2"/>
+      <c r="AF90" s="2"/>
     </row>
     <row r="91" ht="15.75" customHeight="1">
       <c r="B91" s="2"/>
@@ -8564,6 +8667,7 @@
       <c r="AC91" s="2"/>
       <c r="AD91" s="2"/>
       <c r="AE91" s="2"/>
+      <c r="AF91" s="2"/>
     </row>
     <row r="92" ht="15.75" customHeight="1">
       <c r="B92" s="2"/>
@@ -8596,6 +8700,7 @@
       <c r="AC92" s="2"/>
       <c r="AD92" s="2"/>
       <c r="AE92" s="2"/>
+      <c r="AF92" s="2"/>
     </row>
     <row r="93" ht="15.75" customHeight="1">
       <c r="B93" s="2"/>
@@ -8628,6 +8733,7 @@
       <c r="AC93" s="2"/>
       <c r="AD93" s="2"/>
       <c r="AE93" s="2"/>
+      <c r="AF93" s="2"/>
     </row>
     <row r="94" ht="15.75" customHeight="1">
       <c r="B94" s="2"/>
@@ -8660,6 +8766,7 @@
       <c r="AC94" s="2"/>
       <c r="AD94" s="2"/>
       <c r="AE94" s="2"/>
+      <c r="AF94" s="2"/>
     </row>
     <row r="95" ht="15.75" customHeight="1">
       <c r="B95" s="2"/>
@@ -8692,6 +8799,7 @@
       <c r="AC95" s="2"/>
       <c r="AD95" s="2"/>
       <c r="AE95" s="2"/>
+      <c r="AF95" s="2"/>
     </row>
     <row r="96" ht="15.75" customHeight="1">
       <c r="B96" s="2"/>
@@ -8724,6 +8832,7 @@
       <c r="AC96" s="2"/>
       <c r="AD96" s="2"/>
       <c r="AE96" s="2"/>
+      <c r="AF96" s="2"/>
     </row>
     <row r="97" ht="15.75" customHeight="1">
       <c r="B97" s="2"/>
@@ -8756,6 +8865,7 @@
       <c r="AC97" s="2"/>
       <c r="AD97" s="2"/>
       <c r="AE97" s="2"/>
+      <c r="AF97" s="2"/>
     </row>
     <row r="98" ht="15.75" customHeight="1">
       <c r="B98" s="2"/>
@@ -8788,6 +8898,7 @@
       <c r="AC98" s="2"/>
       <c r="AD98" s="2"/>
       <c r="AE98" s="2"/>
+      <c r="AF98" s="2"/>
     </row>
     <row r="99" ht="15.75" customHeight="1">
       <c r="B99" s="2"/>
@@ -8820,6 +8931,7 @@
       <c r="AC99" s="2"/>
       <c r="AD99" s="2"/>
       <c r="AE99" s="2"/>
+      <c r="AF99" s="2"/>
     </row>
     <row r="100" ht="15.75" customHeight="1">
       <c r="B100" s="2"/>
@@ -8852,6 +8964,7 @@
       <c r="AC100" s="2"/>
       <c r="AD100" s="2"/>
       <c r="AE100" s="2"/>
+      <c r="AF100" s="2"/>
     </row>
     <row r="101" ht="15.75" customHeight="1">
       <c r="B101" s="2"/>
@@ -8884,6 +8997,7 @@
       <c r="AC101" s="2"/>
       <c r="AD101" s="2"/>
       <c r="AE101" s="2"/>
+      <c r="AF101" s="2"/>
     </row>
     <row r="102" ht="15.75" customHeight="1">
       <c r="B102" s="2"/>
@@ -8916,6 +9030,7 @@
       <c r="AC102" s="2"/>
       <c r="AD102" s="2"/>
       <c r="AE102" s="2"/>
+      <c r="AF102" s="2"/>
     </row>
     <row r="103" ht="15.75" customHeight="1">
       <c r="B103" s="2"/>
@@ -8948,6 +9063,7 @@
       <c r="AC103" s="2"/>
       <c r="AD103" s="2"/>
       <c r="AE103" s="2"/>
+      <c r="AF103" s="2"/>
     </row>
     <row r="104" ht="15.75" customHeight="1">
       <c r="B104" s="2"/>
@@ -8980,6 +9096,7 @@
       <c r="AC104" s="2"/>
       <c r="AD104" s="2"/>
       <c r="AE104" s="2"/>
+      <c r="AF104" s="2"/>
     </row>
     <row r="105" ht="15.75" customHeight="1">
       <c r="B105" s="2"/>
@@ -9012,6 +9129,7 @@
       <c r="AC105" s="2"/>
       <c r="AD105" s="2"/>
       <c r="AE105" s="2"/>
+      <c r="AF105" s="2"/>
     </row>
     <row r="106" ht="15.75" customHeight="1">
       <c r="B106" s="2"/>
@@ -9044,6 +9162,7 @@
       <c r="AC106" s="2"/>
       <c r="AD106" s="2"/>
       <c r="AE106" s="2"/>
+      <c r="AF106" s="2"/>
     </row>
     <row r="107" ht="15.75" customHeight="1">
       <c r="B107" s="2"/>
@@ -9076,6 +9195,7 @@
       <c r="AC107" s="2"/>
       <c r="AD107" s="2"/>
       <c r="AE107" s="2"/>
+      <c r="AF107" s="2"/>
     </row>
     <row r="108" ht="15.75" customHeight="1">
       <c r="B108" s="2"/>
@@ -9108,6 +9228,7 @@
       <c r="AC108" s="2"/>
       <c r="AD108" s="2"/>
       <c r="AE108" s="2"/>
+      <c r="AF108" s="2"/>
     </row>
     <row r="109" ht="15.75" customHeight="1">
       <c r="B109" s="2"/>
@@ -9140,6 +9261,7 @@
       <c r="AC109" s="2"/>
       <c r="AD109" s="2"/>
       <c r="AE109" s="2"/>
+      <c r="AF109" s="2"/>
     </row>
     <row r="110" ht="15.75" customHeight="1">
       <c r="B110" s="2"/>
@@ -9172,6 +9294,7 @@
       <c r="AC110" s="2"/>
       <c r="AD110" s="2"/>
       <c r="AE110" s="2"/>
+      <c r="AF110" s="2"/>
     </row>
     <row r="111" ht="15.75" customHeight="1">
       <c r="B111" s="2"/>
@@ -9204,6 +9327,7 @@
       <c r="AC111" s="2"/>
       <c r="AD111" s="2"/>
       <c r="AE111" s="2"/>
+      <c r="AF111" s="2"/>
     </row>
     <row r="112" ht="15.75" customHeight="1">
       <c r="B112" s="2"/>
@@ -9236,6 +9360,7 @@
       <c r="AC112" s="2"/>
       <c r="AD112" s="2"/>
       <c r="AE112" s="2"/>
+      <c r="AF112" s="2"/>
     </row>
     <row r="113" ht="15.75" customHeight="1">
       <c r="B113" s="2"/>
@@ -9268,6 +9393,7 @@
       <c r="AC113" s="2"/>
       <c r="AD113" s="2"/>
       <c r="AE113" s="2"/>
+      <c r="AF113" s="2"/>
     </row>
     <row r="114" ht="15.75" customHeight="1">
       <c r="B114" s="2"/>
@@ -9300,6 +9426,7 @@
       <c r="AC114" s="2"/>
       <c r="AD114" s="2"/>
       <c r="AE114" s="2"/>
+      <c r="AF114" s="2"/>
     </row>
     <row r="115" ht="15.75" customHeight="1">
       <c r="B115" s="2"/>
@@ -9332,6 +9459,7 @@
       <c r="AC115" s="2"/>
       <c r="AD115" s="2"/>
       <c r="AE115" s="2"/>
+      <c r="AF115" s="2"/>
     </row>
     <row r="116" ht="15.75" customHeight="1">
       <c r="B116" s="2"/>
@@ -9364,6 +9492,7 @@
       <c r="AC116" s="2"/>
       <c r="AD116" s="2"/>
       <c r="AE116" s="2"/>
+      <c r="AF116" s="2"/>
     </row>
     <row r="117" ht="15.75" customHeight="1">
       <c r="B117" s="2"/>
@@ -9396,6 +9525,7 @@
       <c r="AC117" s="2"/>
       <c r="AD117" s="2"/>
       <c r="AE117" s="2"/>
+      <c r="AF117" s="2"/>
     </row>
     <row r="118" ht="15.75" customHeight="1">
       <c r="B118" s="2"/>
@@ -9428,6 +9558,7 @@
       <c r="AC118" s="2"/>
       <c r="AD118" s="2"/>
       <c r="AE118" s="2"/>
+      <c r="AF118" s="2"/>
     </row>
     <row r="119" ht="15.75" customHeight="1">
       <c r="B119" s="2"/>
@@ -9460,6 +9591,7 @@
       <c r="AC119" s="2"/>
       <c r="AD119" s="2"/>
       <c r="AE119" s="2"/>
+      <c r="AF119" s="2"/>
     </row>
     <row r="120" ht="15.75" customHeight="1">
       <c r="B120" s="2"/>
@@ -9492,6 +9624,7 @@
       <c r="AC120" s="2"/>
       <c r="AD120" s="2"/>
       <c r="AE120" s="2"/>
+      <c r="AF120" s="2"/>
     </row>
     <row r="121" ht="15.75" customHeight="1">
       <c r="B121" s="2"/>
@@ -9524,6 +9657,7 @@
       <c r="AC121" s="2"/>
       <c r="AD121" s="2"/>
       <c r="AE121" s="2"/>
+      <c r="AF121" s="2"/>
     </row>
     <row r="122" ht="15.75" customHeight="1">
       <c r="B122" s="2"/>
@@ -9556,6 +9690,7 @@
       <c r="AC122" s="2"/>
       <c r="AD122" s="2"/>
       <c r="AE122" s="2"/>
+      <c r="AF122" s="2"/>
     </row>
     <row r="123" ht="15.75" customHeight="1">
       <c r="B123" s="2"/>
@@ -9588,6 +9723,7 @@
       <c r="AC123" s="2"/>
       <c r="AD123" s="2"/>
       <c r="AE123" s="2"/>
+      <c r="AF123" s="2"/>
     </row>
     <row r="124" ht="15.75" customHeight="1">
       <c r="B124" s="2"/>
@@ -9620,6 +9756,7 @@
       <c r="AC124" s="2"/>
       <c r="AD124" s="2"/>
       <c r="AE124" s="2"/>
+      <c r="AF124" s="2"/>
     </row>
     <row r="125" ht="15.75" customHeight="1">
       <c r="B125" s="2"/>
@@ -9652,6 +9789,7 @@
       <c r="AC125" s="2"/>
       <c r="AD125" s="2"/>
       <c r="AE125" s="2"/>
+      <c r="AF125" s="2"/>
     </row>
     <row r="126" ht="15.75" customHeight="1">
       <c r="B126" s="2"/>
@@ -9684,6 +9822,7 @@
       <c r="AC126" s="2"/>
       <c r="AD126" s="2"/>
       <c r="AE126" s="2"/>
+      <c r="AF126" s="2"/>
     </row>
     <row r="127" ht="15.75" customHeight="1">
       <c r="B127" s="2"/>
@@ -9716,6 +9855,7 @@
       <c r="AC127" s="2"/>
       <c r="AD127" s="2"/>
       <c r="AE127" s="2"/>
+      <c r="AF127" s="2"/>
     </row>
     <row r="128" ht="15.75" customHeight="1">
       <c r="B128" s="2"/>
@@ -9748,6 +9888,7 @@
       <c r="AC128" s="2"/>
       <c r="AD128" s="2"/>
       <c r="AE128" s="2"/>
+      <c r="AF128" s="2"/>
     </row>
     <row r="129" ht="15.75" customHeight="1">
       <c r="B129" s="2"/>
@@ -9780,6 +9921,7 @@
       <c r="AC129" s="2"/>
       <c r="AD129" s="2"/>
       <c r="AE129" s="2"/>
+      <c r="AF129" s="2"/>
     </row>
     <row r="130" ht="15.75" customHeight="1">
       <c r="B130" s="2"/>
@@ -9812,6 +9954,7 @@
       <c r="AC130" s="2"/>
       <c r="AD130" s="2"/>
       <c r="AE130" s="2"/>
+      <c r="AF130" s="2"/>
     </row>
     <row r="131" ht="15.75" customHeight="1">
       <c r="B131" s="2"/>
@@ -9844,6 +9987,7 @@
       <c r="AC131" s="2"/>
       <c r="AD131" s="2"/>
       <c r="AE131" s="2"/>
+      <c r="AF131" s="2"/>
     </row>
     <row r="132" ht="15.75" customHeight="1">
       <c r="B132" s="2"/>
@@ -9876,6 +10020,7 @@
       <c r="AC132" s="2"/>
       <c r="AD132" s="2"/>
       <c r="AE132" s="2"/>
+      <c r="AF132" s="2"/>
     </row>
     <row r="133" ht="15.75" customHeight="1">
       <c r="B133" s="2"/>
@@ -9908,6 +10053,7 @@
       <c r="AC133" s="2"/>
       <c r="AD133" s="2"/>
       <c r="AE133" s="2"/>
+      <c r="AF133" s="2"/>
     </row>
     <row r="134" ht="15.75" customHeight="1">
       <c r="B134" s="2"/>
@@ -9940,6 +10086,7 @@
       <c r="AC134" s="2"/>
       <c r="AD134" s="2"/>
       <c r="AE134" s="2"/>
+      <c r="AF134" s="2"/>
     </row>
     <row r="135" ht="15.75" customHeight="1">
       <c r="B135" s="2"/>
@@ -9972,6 +10119,7 @@
       <c r="AC135" s="2"/>
       <c r="AD135" s="2"/>
       <c r="AE135" s="2"/>
+      <c r="AF135" s="2"/>
     </row>
     <row r="136" ht="15.75" customHeight="1">
       <c r="B136" s="2"/>
@@ -10004,6 +10152,7 @@
       <c r="AC136" s="2"/>
       <c r="AD136" s="2"/>
       <c r="AE136" s="2"/>
+      <c r="AF136" s="2"/>
     </row>
     <row r="137" ht="15.75" customHeight="1">
       <c r="B137" s="2"/>
@@ -10036,6 +10185,7 @@
       <c r="AC137" s="2"/>
       <c r="AD137" s="2"/>
       <c r="AE137" s="2"/>
+      <c r="AF137" s="2"/>
     </row>
     <row r="138" ht="15.75" customHeight="1">
       <c r="B138" s="2"/>
@@ -10068,6 +10218,7 @@
       <c r="AC138" s="2"/>
       <c r="AD138" s="2"/>
       <c r="AE138" s="2"/>
+      <c r="AF138" s="2"/>
     </row>
     <row r="139" ht="15.75" customHeight="1">
       <c r="B139" s="2"/>
@@ -10100,6 +10251,7 @@
       <c r="AC139" s="2"/>
       <c r="AD139" s="2"/>
       <c r="AE139" s="2"/>
+      <c r="AF139" s="2"/>
     </row>
     <row r="140" ht="15.75" customHeight="1">
       <c r="B140" s="2"/>
@@ -10132,6 +10284,7 @@
       <c r="AC140" s="2"/>
       <c r="AD140" s="2"/>
       <c r="AE140" s="2"/>
+      <c r="AF140" s="2"/>
     </row>
     <row r="141" ht="15.75" customHeight="1">
       <c r="B141" s="2"/>
@@ -10164,6 +10317,7 @@
       <c r="AC141" s="2"/>
       <c r="AD141" s="2"/>
       <c r="AE141" s="2"/>
+      <c r="AF141" s="2"/>
     </row>
     <row r="142" ht="15.75" customHeight="1">
       <c r="B142" s="2"/>
@@ -10196,6 +10350,7 @@
       <c r="AC142" s="2"/>
       <c r="AD142" s="2"/>
       <c r="AE142" s="2"/>
+      <c r="AF142" s="2"/>
     </row>
     <row r="143" ht="15.75" customHeight="1">
       <c r="B143" s="2"/>
@@ -10228,6 +10383,7 @@
       <c r="AC143" s="2"/>
       <c r="AD143" s="2"/>
       <c r="AE143" s="2"/>
+      <c r="AF143" s="2"/>
     </row>
     <row r="144" ht="15.75" customHeight="1">
       <c r="B144" s="2"/>
@@ -10260,6 +10416,7 @@
       <c r="AC144" s="2"/>
       <c r="AD144" s="2"/>
       <c r="AE144" s="2"/>
+      <c r="AF144" s="2"/>
     </row>
     <row r="145" ht="15.75" customHeight="1">
       <c r="B145" s="2"/>
@@ -10292,6 +10449,7 @@
       <c r="AC145" s="2"/>
       <c r="AD145" s="2"/>
       <c r="AE145" s="2"/>
+      <c r="AF145" s="2"/>
     </row>
     <row r="146" ht="15.75" customHeight="1">
       <c r="B146" s="2"/>
@@ -10324,6 +10482,7 @@
       <c r="AC146" s="2"/>
       <c r="AD146" s="2"/>
       <c r="AE146" s="2"/>
+      <c r="AF146" s="2"/>
     </row>
     <row r="147" ht="15.75" customHeight="1">
       <c r="B147" s="2"/>
@@ -10356,6 +10515,7 @@
       <c r="AC147" s="2"/>
       <c r="AD147" s="2"/>
       <c r="AE147" s="2"/>
+      <c r="AF147" s="2"/>
     </row>
     <row r="148" ht="15.75" customHeight="1">
       <c r="B148" s="2"/>
@@ -10388,6 +10548,7 @@
       <c r="AC148" s="2"/>
       <c r="AD148" s="2"/>
       <c r="AE148" s="2"/>
+      <c r="AF148" s="2"/>
     </row>
     <row r="149" ht="15.75" customHeight="1">
       <c r="B149" s="2"/>
@@ -10420,6 +10581,7 @@
       <c r="AC149" s="2"/>
       <c r="AD149" s="2"/>
       <c r="AE149" s="2"/>
+      <c r="AF149" s="2"/>
     </row>
     <row r="150" ht="15.75" customHeight="1">
       <c r="B150" s="2"/>
@@ -10452,6 +10614,7 @@
       <c r="AC150" s="2"/>
       <c r="AD150" s="2"/>
       <c r="AE150" s="2"/>
+      <c r="AF150" s="2"/>
     </row>
     <row r="151" ht="15.75" customHeight="1">
       <c r="B151" s="2"/>
@@ -10484,6 +10647,7 @@
       <c r="AC151" s="2"/>
       <c r="AD151" s="2"/>
       <c r="AE151" s="2"/>
+      <c r="AF151" s="2"/>
     </row>
     <row r="152" ht="15.75" customHeight="1">
       <c r="B152" s="2"/>
@@ -10516,6 +10680,7 @@
       <c r="AC152" s="2"/>
       <c r="AD152" s="2"/>
       <c r="AE152" s="2"/>
+      <c r="AF152" s="2"/>
     </row>
     <row r="153" ht="15.75" customHeight="1">
       <c r="B153" s="2"/>
@@ -10548,6 +10713,7 @@
       <c r="AC153" s="2"/>
       <c r="AD153" s="2"/>
       <c r="AE153" s="2"/>
+      <c r="AF153" s="2"/>
     </row>
     <row r="154" ht="15.75" customHeight="1">
       <c r="B154" s="2"/>
@@ -10580,6 +10746,7 @@
       <c r="AC154" s="2"/>
       <c r="AD154" s="2"/>
       <c r="AE154" s="2"/>
+      <c r="AF154" s="2"/>
     </row>
     <row r="155" ht="15.75" customHeight="1">
       <c r="B155" s="2"/>
@@ -10612,6 +10779,7 @@
       <c r="AC155" s="2"/>
       <c r="AD155" s="2"/>
       <c r="AE155" s="2"/>
+      <c r="AF155" s="2"/>
     </row>
     <row r="156" ht="15.75" customHeight="1">
       <c r="B156" s="2"/>
@@ -10644,6 +10812,7 @@
       <c r="AC156" s="2"/>
       <c r="AD156" s="2"/>
       <c r="AE156" s="2"/>
+      <c r="AF156" s="2"/>
     </row>
     <row r="157" ht="15.75" customHeight="1">
       <c r="B157" s="2"/>
@@ -10676,6 +10845,7 @@
       <c r="AC157" s="2"/>
       <c r="AD157" s="2"/>
       <c r="AE157" s="2"/>
+      <c r="AF157" s="2"/>
     </row>
     <row r="158" ht="15.75" customHeight="1">
       <c r="B158" s="2"/>
@@ -10708,6 +10878,7 @@
       <c r="AC158" s="2"/>
       <c r="AD158" s="2"/>
       <c r="AE158" s="2"/>
+      <c r="AF158" s="2"/>
     </row>
     <row r="159" ht="15.75" customHeight="1">
       <c r="B159" s="2"/>
@@ -10740,6 +10911,7 @@
       <c r="AC159" s="2"/>
       <c r="AD159" s="2"/>
       <c r="AE159" s="2"/>
+      <c r="AF159" s="2"/>
     </row>
     <row r="160" ht="15.75" customHeight="1">
       <c r="B160" s="2"/>
@@ -10772,6 +10944,7 @@
       <c r="AC160" s="2"/>
       <c r="AD160" s="2"/>
       <c r="AE160" s="2"/>
+      <c r="AF160" s="2"/>
     </row>
     <row r="161" ht="15.75" customHeight="1">
       <c r="B161" s="2"/>
@@ -10804,6 +10977,7 @@
       <c r="AC161" s="2"/>
       <c r="AD161" s="2"/>
       <c r="AE161" s="2"/>
+      <c r="AF161" s="2"/>
     </row>
     <row r="162" ht="15.75" customHeight="1">
       <c r="B162" s="2"/>
@@ -10836,6 +11010,7 @@
       <c r="AC162" s="2"/>
       <c r="AD162" s="2"/>
       <c r="AE162" s="2"/>
+      <c r="AF162" s="2"/>
     </row>
     <row r="163" ht="15.75" customHeight="1">
       <c r="B163" s="2"/>
@@ -10868,6 +11043,7 @@
       <c r="AC163" s="2"/>
       <c r="AD163" s="2"/>
       <c r="AE163" s="2"/>
+      <c r="AF163" s="2"/>
     </row>
     <row r="164" ht="15.75" customHeight="1">
       <c r="B164" s="2"/>
@@ -10900,6 +11076,7 @@
       <c r="AC164" s="2"/>
       <c r="AD164" s="2"/>
       <c r="AE164" s="2"/>
+      <c r="AF164" s="2"/>
     </row>
     <row r="165" ht="15.75" customHeight="1">
       <c r="B165" s="2"/>
@@ -10932,6 +11109,7 @@
       <c r="AC165" s="2"/>
       <c r="AD165" s="2"/>
       <c r="AE165" s="2"/>
+      <c r="AF165" s="2"/>
     </row>
     <row r="166" ht="15.75" customHeight="1">
       <c r="B166" s="2"/>
@@ -10964,6 +11142,7 @@
       <c r="AC166" s="2"/>
       <c r="AD166" s="2"/>
       <c r="AE166" s="2"/>
+      <c r="AF166" s="2"/>
     </row>
     <row r="167" ht="15.75" customHeight="1">
       <c r="B167" s="2"/>
@@ -10996,6 +11175,7 @@
       <c r="AC167" s="2"/>
       <c r="AD167" s="2"/>
       <c r="AE167" s="2"/>
+      <c r="AF167" s="2"/>
     </row>
     <row r="168" ht="15.75" customHeight="1">
       <c r="B168" s="2"/>
@@ -11028,6 +11208,7 @@
       <c r="AC168" s="2"/>
       <c r="AD168" s="2"/>
       <c r="AE168" s="2"/>
+      <c r="AF168" s="2"/>
     </row>
     <row r="169" ht="15.75" customHeight="1">
       <c r="B169" s="2"/>
@@ -11060,6 +11241,7 @@
       <c r="AC169" s="2"/>
       <c r="AD169" s="2"/>
       <c r="AE169" s="2"/>
+      <c r="AF169" s="2"/>
     </row>
     <row r="170" ht="15.75" customHeight="1">
       <c r="B170" s="2"/>
@@ -11092,6 +11274,7 @@
       <c r="AC170" s="2"/>
       <c r="AD170" s="2"/>
       <c r="AE170" s="2"/>
+      <c r="AF170" s="2"/>
     </row>
     <row r="171" ht="15.75" customHeight="1">
       <c r="B171" s="2"/>
@@ -11124,6 +11307,7 @@
       <c r="AC171" s="2"/>
       <c r="AD171" s="2"/>
       <c r="AE171" s="2"/>
+      <c r="AF171" s="2"/>
     </row>
     <row r="172" ht="15.75" customHeight="1">
       <c r="B172" s="2"/>
@@ -11156,6 +11340,7 @@
       <c r="AC172" s="2"/>
       <c r="AD172" s="2"/>
       <c r="AE172" s="2"/>
+      <c r="AF172" s="2"/>
     </row>
     <row r="173" ht="15.75" customHeight="1">
       <c r="B173" s="2"/>
@@ -11188,6 +11373,7 @@
       <c r="AC173" s="2"/>
       <c r="AD173" s="2"/>
       <c r="AE173" s="2"/>
+      <c r="AF173" s="2"/>
     </row>
     <row r="174" ht="15.75" customHeight="1">
       <c r="B174" s="2"/>
@@ -11220,6 +11406,7 @@
       <c r="AC174" s="2"/>
       <c r="AD174" s="2"/>
       <c r="AE174" s="2"/>
+      <c r="AF174" s="2"/>
     </row>
     <row r="175" ht="15.75" customHeight="1">
       <c r="B175" s="2"/>
@@ -11252,6 +11439,7 @@
       <c r="AC175" s="2"/>
       <c r="AD175" s="2"/>
       <c r="AE175" s="2"/>
+      <c r="AF175" s="2"/>
     </row>
     <row r="176" ht="15.75" customHeight="1">
       <c r="B176" s="2"/>
@@ -11284,6 +11472,7 @@
       <c r="AC176" s="2"/>
       <c r="AD176" s="2"/>
       <c r="AE176" s="2"/>
+      <c r="AF176" s="2"/>
     </row>
     <row r="177" ht="15.75" customHeight="1">
       <c r="B177" s="2"/>
@@ -11316,6 +11505,7 @@
       <c r="AC177" s="2"/>
       <c r="AD177" s="2"/>
       <c r="AE177" s="2"/>
+      <c r="AF177" s="2"/>
     </row>
     <row r="178" ht="15.75" customHeight="1">
       <c r="B178" s="2"/>
@@ -11348,6 +11538,7 @@
       <c r="AC178" s="2"/>
       <c r="AD178" s="2"/>
       <c r="AE178" s="2"/>
+      <c r="AF178" s="2"/>
     </row>
     <row r="179" ht="15.75" customHeight="1">
       <c r="B179" s="2"/>
@@ -11380,6 +11571,7 @@
       <c r="AC179" s="2"/>
       <c r="AD179" s="2"/>
       <c r="AE179" s="2"/>
+      <c r="AF179" s="2"/>
     </row>
     <row r="180" ht="15.75" customHeight="1">
       <c r="B180" s="2"/>
@@ -11412,6 +11604,7 @@
       <c r="AC180" s="2"/>
       <c r="AD180" s="2"/>
       <c r="AE180" s="2"/>
+      <c r="AF180" s="2"/>
     </row>
     <row r="181" ht="15.75" customHeight="1">
       <c r="B181" s="2"/>
@@ -11444,6 +11637,7 @@
       <c r="AC181" s="2"/>
       <c r="AD181" s="2"/>
       <c r="AE181" s="2"/>
+      <c r="AF181" s="2"/>
     </row>
     <row r="182" ht="15.75" customHeight="1">
       <c r="B182" s="2"/>
@@ -11476,6 +11670,7 @@
       <c r="AC182" s="2"/>
       <c r="AD182" s="2"/>
       <c r="AE182" s="2"/>
+      <c r="AF182" s="2"/>
     </row>
     <row r="183" ht="15.75" customHeight="1">
       <c r="B183" s="2"/>
@@ -11508,6 +11703,7 @@
       <c r="AC183" s="2"/>
       <c r="AD183" s="2"/>
       <c r="AE183" s="2"/>
+      <c r="AF183" s="2"/>
     </row>
     <row r="184" ht="15.75" customHeight="1">
       <c r="B184" s="2"/>
@@ -11540,6 +11736,7 @@
       <c r="AC184" s="2"/>
       <c r="AD184" s="2"/>
       <c r="AE184" s="2"/>
+      <c r="AF184" s="2"/>
     </row>
     <row r="185" ht="15.75" customHeight="1">
       <c r="B185" s="2"/>
@@ -11572,6 +11769,7 @@
       <c r="AC185" s="2"/>
       <c r="AD185" s="2"/>
       <c r="AE185" s="2"/>
+      <c r="AF185" s="2"/>
     </row>
     <row r="186" ht="15.75" customHeight="1">
       <c r="B186" s="2"/>
@@ -11604,6 +11802,7 @@
       <c r="AC186" s="2"/>
       <c r="AD186" s="2"/>
       <c r="AE186" s="2"/>
+      <c r="AF186" s="2"/>
     </row>
     <row r="187" ht="15.75" customHeight="1">
       <c r="B187" s="2"/>
@@ -11636,6 +11835,7 @@
       <c r="AC187" s="2"/>
       <c r="AD187" s="2"/>
       <c r="AE187" s="2"/>
+      <c r="AF187" s="2"/>
     </row>
     <row r="188" ht="15.75" customHeight="1">
       <c r="B188" s="2"/>
@@ -11668,6 +11868,7 @@
       <c r="AC188" s="2"/>
       <c r="AD188" s="2"/>
       <c r="AE188" s="2"/>
+      <c r="AF188" s="2"/>
     </row>
     <row r="189" ht="15.75" customHeight="1">
       <c r="B189" s="2"/>
@@ -11700,6 +11901,7 @@
       <c r="AC189" s="2"/>
       <c r="AD189" s="2"/>
       <c r="AE189" s="2"/>
+      <c r="AF189" s="2"/>
     </row>
     <row r="190" ht="15.75" customHeight="1">
       <c r="B190" s="2"/>
@@ -11732,6 +11934,7 @@
       <c r="AC190" s="2"/>
       <c r="AD190" s="2"/>
       <c r="AE190" s="2"/>
+      <c r="AF190" s="2"/>
     </row>
     <row r="191" ht="15.75" customHeight="1">
       <c r="B191" s="2"/>
@@ -11764,6 +11967,7 @@
       <c r="AC191" s="2"/>
       <c r="AD191" s="2"/>
       <c r="AE191" s="2"/>
+      <c r="AF191" s="2"/>
     </row>
     <row r="192" ht="15.75" customHeight="1">
       <c r="B192" s="2"/>
@@ -11796,6 +12000,7 @@
       <c r="AC192" s="2"/>
       <c r="AD192" s="2"/>
       <c r="AE192" s="2"/>
+      <c r="AF192" s="2"/>
     </row>
     <row r="193" ht="15.75" customHeight="1">
       <c r="B193" s="2"/>
@@ -11828,6 +12033,7 @@
       <c r="AC193" s="2"/>
       <c r="AD193" s="2"/>
       <c r="AE193" s="2"/>
+      <c r="AF193" s="2"/>
     </row>
     <row r="194" ht="15.75" customHeight="1">
       <c r="B194" s="2"/>
@@ -11860,6 +12066,7 @@
       <c r="AC194" s="2"/>
       <c r="AD194" s="2"/>
       <c r="AE194" s="2"/>
+      <c r="AF194" s="2"/>
     </row>
     <row r="195" ht="15.75" customHeight="1">
       <c r="B195" s="2"/>
@@ -11892,6 +12099,7 @@
       <c r="AC195" s="2"/>
       <c r="AD195" s="2"/>
       <c r="AE195" s="2"/>
+      <c r="AF195" s="2"/>
     </row>
     <row r="196" ht="15.75" customHeight="1">
       <c r="B196" s="2"/>
@@ -11924,6 +12132,7 @@
       <c r="AC196" s="2"/>
       <c r="AD196" s="2"/>
       <c r="AE196" s="2"/>
+      <c r="AF196" s="2"/>
     </row>
     <row r="197" ht="15.75" customHeight="1">
       <c r="B197" s="2"/>
@@ -11956,6 +12165,7 @@
       <c r="AC197" s="2"/>
       <c r="AD197" s="2"/>
       <c r="AE197" s="2"/>
+      <c r="AF197" s="2"/>
     </row>
     <row r="198" ht="15.75" customHeight="1">
       <c r="B198" s="2"/>
@@ -11988,6 +12198,7 @@
       <c r="AC198" s="2"/>
       <c r="AD198" s="2"/>
       <c r="AE198" s="2"/>
+      <c r="AF198" s="2"/>
     </row>
     <row r="199" ht="15.75" customHeight="1">
       <c r="B199" s="2"/>
@@ -12020,6 +12231,7 @@
       <c r="AC199" s="2"/>
       <c r="AD199" s="2"/>
       <c r="AE199" s="2"/>
+      <c r="AF199" s="2"/>
     </row>
     <row r="200" ht="15.75" customHeight="1">
       <c r="B200" s="2"/>
@@ -12052,6 +12264,7 @@
       <c r="AC200" s="2"/>
       <c r="AD200" s="2"/>
       <c r="AE200" s="2"/>
+      <c r="AF200" s="2"/>
     </row>
     <row r="201" ht="15.75" customHeight="1">
       <c r="B201" s="2"/>
@@ -12084,6 +12297,7 @@
       <c r="AC201" s="2"/>
       <c r="AD201" s="2"/>
       <c r="AE201" s="2"/>
+      <c r="AF201" s="2"/>
     </row>
     <row r="202" ht="15.75" customHeight="1">
       <c r="B202" s="2"/>
@@ -12116,6 +12330,7 @@
       <c r="AC202" s="2"/>
       <c r="AD202" s="2"/>
       <c r="AE202" s="2"/>
+      <c r="AF202" s="2"/>
     </row>
     <row r="203" ht="15.75" customHeight="1">
       <c r="B203" s="2"/>
@@ -12148,6 +12363,7 @@
       <c r="AC203" s="2"/>
       <c r="AD203" s="2"/>
       <c r="AE203" s="2"/>
+      <c r="AF203" s="2"/>
     </row>
     <row r="204" ht="15.75" customHeight="1">
       <c r="B204" s="2"/>
@@ -12180,6 +12396,7 @@
       <c r="AC204" s="2"/>
       <c r="AD204" s="2"/>
       <c r="AE204" s="2"/>
+      <c r="AF204" s="2"/>
     </row>
     <row r="205" ht="15.75" customHeight="1">
       <c r="B205" s="2"/>
@@ -12212,6 +12429,7 @@
       <c r="AC205" s="2"/>
       <c r="AD205" s="2"/>
       <c r="AE205" s="2"/>
+      <c r="AF205" s="2"/>
     </row>
     <row r="206" ht="15.75" customHeight="1">
       <c r="B206" s="2"/>
@@ -12244,6 +12462,7 @@
       <c r="AC206" s="2"/>
       <c r="AD206" s="2"/>
       <c r="AE206" s="2"/>
+      <c r="AF206" s="2"/>
     </row>
     <row r="207" ht="15.75" customHeight="1">
       <c r="B207" s="2"/>
@@ -12276,6 +12495,7 @@
       <c r="AC207" s="2"/>
       <c r="AD207" s="2"/>
       <c r="AE207" s="2"/>
+      <c r="AF207" s="2"/>
     </row>
     <row r="208" ht="15.75" customHeight="1">
       <c r="B208" s="2"/>
@@ -12308,6 +12528,7 @@
       <c r="AC208" s="2"/>
       <c r="AD208" s="2"/>
       <c r="AE208" s="2"/>
+      <c r="AF208" s="2"/>
     </row>
     <row r="209" ht="15.75" customHeight="1">
       <c r="B209" s="2"/>
@@ -12340,6 +12561,7 @@
       <c r="AC209" s="2"/>
       <c r="AD209" s="2"/>
       <c r="AE209" s="2"/>
+      <c r="AF209" s="2"/>
     </row>
     <row r="210" ht="15.75" customHeight="1">
       <c r="B210" s="2"/>
@@ -12372,6 +12594,7 @@
       <c r="AC210" s="2"/>
       <c r="AD210" s="2"/>
       <c r="AE210" s="2"/>
+      <c r="AF210" s="2"/>
     </row>
     <row r="211" ht="15.75" customHeight="1">
       <c r="B211" s="2"/>
@@ -12404,6 +12627,7 @@
       <c r="AC211" s="2"/>
       <c r="AD211" s="2"/>
       <c r="AE211" s="2"/>
+      <c r="AF211" s="2"/>
     </row>
     <row r="212" ht="15.75" customHeight="1">
       <c r="B212" s="2"/>
@@ -12436,6 +12660,7 @@
       <c r="AC212" s="2"/>
       <c r="AD212" s="2"/>
       <c r="AE212" s="2"/>
+      <c r="AF212" s="2"/>
     </row>
     <row r="213" ht="15.75" customHeight="1">
       <c r="B213" s="2"/>
@@ -12468,6 +12693,7 @@
       <c r="AC213" s="2"/>
       <c r="AD213" s="2"/>
       <c r="AE213" s="2"/>
+      <c r="AF213" s="2"/>
     </row>
     <row r="214" ht="15.75" customHeight="1">
       <c r="B214" s="2"/>
@@ -12500,6 +12726,7 @@
       <c r="AC214" s="2"/>
       <c r="AD214" s="2"/>
       <c r="AE214" s="2"/>
+      <c r="AF214" s="2"/>
     </row>
     <row r="215" ht="15.75" customHeight="1">
       <c r="B215" s="2"/>
@@ -12532,6 +12759,7 @@
       <c r="AC215" s="2"/>
       <c r="AD215" s="2"/>
       <c r="AE215" s="2"/>
+      <c r="AF215" s="2"/>
     </row>
     <row r="216" ht="15.75" customHeight="1">
       <c r="B216" s="2"/>
@@ -12564,6 +12792,7 @@
       <c r="AC216" s="2"/>
       <c r="AD216" s="2"/>
       <c r="AE216" s="2"/>
+      <c r="AF216" s="2"/>
     </row>
     <row r="217" ht="15.75" customHeight="1">
       <c r="B217" s="2"/>
@@ -12596,6 +12825,7 @@
       <c r="AC217" s="2"/>
       <c r="AD217" s="2"/>
       <c r="AE217" s="2"/>
+      <c r="AF217" s="2"/>
     </row>
     <row r="218" ht="15.75" customHeight="1">
       <c r="B218" s="2"/>
@@ -12628,6 +12858,7 @@
       <c r="AC218" s="2"/>
       <c r="AD218" s="2"/>
       <c r="AE218" s="2"/>
+      <c r="AF218" s="2"/>
     </row>
     <row r="219" ht="15.75" customHeight="1">
       <c r="B219" s="2"/>
@@ -12660,6 +12891,7 @@
       <c r="AC219" s="2"/>
       <c r="AD219" s="2"/>
       <c r="AE219" s="2"/>
+      <c r="AF219" s="2"/>
     </row>
     <row r="220" ht="15.75" customHeight="1">
       <c r="B220" s="2"/>
@@ -12692,6 +12924,7 @@
       <c r="AC220" s="2"/>
       <c r="AD220" s="2"/>
       <c r="AE220" s="2"/>
+      <c r="AF220" s="2"/>
     </row>
     <row r="221" ht="15.75" customHeight="1"/>
     <row r="222" ht="15.75" customHeight="1"/>
@@ -13474,7 +13707,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <mergeCells count="23">
+  <mergeCells count="24">
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B8:B9"/>
     <mergeCell ref="C8:C9"/>
@@ -13490,6 +13723,7 @@
     <mergeCell ref="M8:M9"/>
     <mergeCell ref="N8:N9"/>
     <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="AF8:AF9"/>
     <mergeCell ref="AE8:AE9"/>
     <mergeCell ref="O8:O9"/>
     <mergeCell ref="P8:P9"/>
@@ -13504,9 +13738,9 @@
       <formula>LEN(TRIM(H10))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AE10">
+  <conditionalFormatting sqref="AF10">
     <cfRule type="notContainsBlanks" dxfId="0" priority="2">
-      <formula>LEN(TRIM(AE10))&gt;0</formula>
+      <formula>LEN(TRIM(AF10))&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions/>
@@ -13532,7 +13766,7 @@
   <sheetData>
     <row r="1" ht="23.25" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -13659,11 +13893,11 @@
       <c r="H8" s="27"/>
       <c r="I8" s="27"/>
       <c r="J8" s="28"/>
-      <c r="K8" s="29" t="s">
-        <v>112</v>
-      </c>
-      <c r="L8" s="29" t="s">
-        <v>88</v>
+      <c r="K8" s="35" t="s">
+        <v>114</v>
+      </c>
+      <c r="L8" s="35" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1">
@@ -13693,44 +13927,44 @@
         <v>2022.0</v>
       </c>
       <c r="J9" s="31" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="K9" s="30"/>
       <c r="L9" s="30"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="22" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="F10" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="L10" s="2" t="str">
         <f>B10+C10+D10+E10+F10+G10+H10+I10+J10+K10</f>
@@ -17281,299 +17515,299 @@
   <sheetData>
     <row r="1" ht="21.75" customHeight="1">
       <c r="A1" s="20" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B1" s="20" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C1" s="20" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" ht="21.75" customHeight="1">
-      <c r="A2" s="35">
+      <c r="A2" s="36">
         <v>1001.0</v>
       </c>
-      <c r="B2" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C2" s="35" t="s">
-        <v>117</v>
+      <c r="B2" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C2" s="36" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="A3" s="35">
+      <c r="A3" s="36">
         <v>1002.0</v>
       </c>
-      <c r="B3" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C3" s="35" t="s">
+      <c r="B3" s="36" t="s">
         <v>118</v>
       </c>
+      <c r="C3" s="36" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="35">
+      <c r="A4" s="36">
         <v>1004.0</v>
       </c>
-      <c r="B4" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C4" s="35" t="s">
-        <v>119</v>
+      <c r="B4" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C4" s="36" t="s">
+        <v>121</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="35">
+      <c r="A5" s="36">
         <v>1005.0</v>
       </c>
-      <c r="B5" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C5" s="35" t="s">
-        <v>120</v>
+      <c r="B5" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C5" s="36" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="35">
+      <c r="A6" s="36">
         <v>1006.0</v>
       </c>
-      <c r="B6" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6" s="35" t="s">
-        <v>121</v>
+      <c r="B6" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C6" s="36" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="35">
+      <c r="A7" s="36">
         <v>1007.0</v>
       </c>
-      <c r="B7" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C7" s="35" t="s">
-        <v>122</v>
+      <c r="B7" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C7" s="36" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="35">
+      <c r="A8" s="36">
         <v>1017.0</v>
       </c>
-      <c r="B8" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C8" s="35" t="s">
-        <v>123</v>
+      <c r="B8" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="36" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="35">
+      <c r="A9" s="36">
         <v>1018.0</v>
       </c>
-      <c r="B9" s="35" t="s">
-        <v>116</v>
-      </c>
-      <c r="C9" s="35" t="s">
-        <v>124</v>
+      <c r="B9" s="36" t="s">
+        <v>118</v>
+      </c>
+      <c r="C9" s="36" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="35">
+      <c r="A10" s="36">
         <v>2003.0</v>
       </c>
-      <c r="B10" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C10" s="35" t="s">
-        <v>126</v>
+      <c r="B10" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="36" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="35">
+      <c r="A11" s="36">
         <v>2005.0</v>
       </c>
-      <c r="B11" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C11" s="35" t="s">
+      <c r="B11" s="36" t="s">
         <v>127</v>
       </c>
+      <c r="C11" s="36" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="35">
+      <c r="A12" s="36">
         <v>2008.0</v>
       </c>
-      <c r="B12" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C12" s="35" t="s">
-        <v>128</v>
+      <c r="B12" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C12" s="36" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="35">
+      <c r="A13" s="36">
         <v>2009.0</v>
       </c>
-      <c r="B13" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C13" s="35" t="s">
-        <v>129</v>
+      <c r="B13" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C13" s="36" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="35">
+      <c r="A14" s="36">
         <v>2011.0</v>
       </c>
-      <c r="B14" s="35" t="s">
-        <v>130</v>
-      </c>
-      <c r="C14" s="35" t="s">
-        <v>131</v>
+      <c r="B14" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="C14" s="36" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="35">
+      <c r="A15" s="36">
         <v>2014.0</v>
       </c>
-      <c r="B15" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C15" s="35" t="s">
+      <c r="B15" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C15" s="36" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="16" ht="21.75" customHeight="1">
+      <c r="A16" s="36">
+        <v>2016.0</v>
+      </c>
+      <c r="B16" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C16" s="36" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="17" ht="21.75" customHeight="1">
+      <c r="A17" s="36">
+        <v>2018.0</v>
+      </c>
+      <c r="B17" s="36" t="s">
         <v>132</v>
       </c>
-    </row>
-    <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="35">
-        <v>2016.0</v>
-      </c>
-      <c r="B16" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C16" s="35" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="35">
-        <v>2018.0</v>
-      </c>
-      <c r="B17" s="35" t="s">
-        <v>130</v>
-      </c>
-      <c r="C17" s="35" t="s">
+      <c r="C17" s="36" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="18" ht="21.75" customHeight="1">
+      <c r="A18" s="36">
+        <v>2022.0</v>
+      </c>
+      <c r="B18" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C18" s="36" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="19" ht="21.75" customHeight="1">
+      <c r="A19" s="36">
+        <v>2025.0</v>
+      </c>
+      <c r="B19" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="C19" s="36" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="20" ht="21.75" customHeight="1">
+      <c r="A20" s="36">
+        <v>2032.0</v>
+      </c>
+      <c r="B20" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C20" s="36" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="21" ht="21.75" customHeight="1">
+      <c r="A21" s="36">
+        <v>2034.0</v>
+      </c>
+      <c r="B21" s="36" t="s">
+        <v>127</v>
+      </c>
+      <c r="C21" s="36" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="22" ht="21.75" customHeight="1">
+      <c r="A22" s="36">
+        <v>2037.0</v>
+      </c>
+      <c r="B22" s="36" t="s">
+        <v>132</v>
+      </c>
+      <c r="C22" s="36" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="23" ht="21.75" customHeight="1">
+      <c r="A23" s="36">
+        <v>4010.0</v>
+      </c>
+      <c r="B23" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="C23" s="36" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="24" ht="21.75" customHeight="1">
+      <c r="A24" s="36">
+        <v>4017.0</v>
+      </c>
+      <c r="B24" s="36" t="s">
+        <v>142</v>
+      </c>
+      <c r="C24" s="36" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="35">
-        <v>2022.0</v>
-      </c>
-      <c r="B18" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C18" s="35" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="35">
-        <v>2025.0</v>
-      </c>
-      <c r="B19" s="35" t="s">
-        <v>130</v>
-      </c>
-      <c r="C19" s="35" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="35">
-        <v>2032.0</v>
-      </c>
-      <c r="B20" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C20" s="35" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="35">
-        <v>2034.0</v>
-      </c>
-      <c r="B21" s="35" t="s">
-        <v>125</v>
-      </c>
-      <c r="C21" s="35" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="35">
-        <v>2037.0</v>
-      </c>
-      <c r="B22" s="35" t="s">
-        <v>130</v>
-      </c>
-      <c r="C22" s="35" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="35">
-        <v>4010.0</v>
-      </c>
-      <c r="B23" s="35" t="s">
-        <v>140</v>
-      </c>
-      <c r="C23" s="35" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="35">
-        <v>4017.0</v>
-      </c>
-      <c r="B24" s="35" t="s">
-        <v>140</v>
-      </c>
-      <c r="C24" s="35" t="s">
-        <v>132</v>
-      </c>
-    </row>
     <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="35">
+      <c r="A25" s="36">
         <v>5006.0</v>
       </c>
-      <c r="B25" s="35" t="s">
-        <v>142</v>
-      </c>
-      <c r="C25" s="35" t="s">
-        <v>143</v>
+      <c r="B25" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="C25" s="36" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="35">
+      <c r="A26" s="36">
         <v>5007.0</v>
       </c>
-      <c r="B26" s="35" t="s">
-        <v>142</v>
-      </c>
-      <c r="C26" s="35" t="s">
+      <c r="B26" s="36" t="s">
         <v>144</v>
       </c>
+      <c r="C26" s="36" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="35">
+      <c r="A27" s="36">
         <v>5011.0</v>
       </c>
-      <c r="B27" s="35" t="s">
-        <v>142</v>
-      </c>
-      <c r="C27" s="35" t="s">
-        <v>145</v>
+      <c r="B27" s="36" t="s">
+        <v>144</v>
+      </c>
+      <c r="C27" s="36" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1"/>

</xml_diff>

<commit_message>
[feat/ASP-6682-Device-and-Site-Summary-Report-Request-for-an-additional-sheet] fix: excluded no result from the formula of xpert error/invalid
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -649,7 +649,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="35">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -719,18 +719,12 @@
     </xf>
     <xf borderId="6" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="7" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="4" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="8" fillId="0" fontId="7" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="2" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
     </xf>
     <xf borderId="4" fillId="2" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="center" wrapText="1"/>
@@ -5827,10 +5821,10 @@
       <c r="AA8" s="27"/>
       <c r="AB8" s="27"/>
       <c r="AC8" s="28"/>
-      <c r="AD8" s="29" t="s">
+      <c r="AD8" s="24" t="s">
         <v>87</v>
       </c>
-      <c r="AE8" s="29" t="s">
+      <c r="AE8" s="24" t="s">
         <v>88</v>
       </c>
       <c r="AF8" s="24" t="s">
@@ -5838,56 +5832,56 @@
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1">
-      <c r="A9" s="30"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
-      <c r="P9" s="30"/>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
-      <c r="S9" s="30"/>
-      <c r="T9" s="30"/>
-      <c r="U9" s="31">
+      <c r="A9" s="29"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="29"/>
+      <c r="D9" s="29"/>
+      <c r="E9" s="29"/>
+      <c r="F9" s="29"/>
+      <c r="G9" s="29"/>
+      <c r="H9" s="29"/>
+      <c r="I9" s="29"/>
+      <c r="J9" s="29"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="29"/>
+      <c r="M9" s="29"/>
+      <c r="N9" s="29"/>
+      <c r="O9" s="29"/>
+      <c r="P9" s="29"/>
+      <c r="Q9" s="29"/>
+      <c r="R9" s="29"/>
+      <c r="S9" s="29"/>
+      <c r="T9" s="29"/>
+      <c r="U9" s="30">
         <v>5011.0</v>
       </c>
-      <c r="V9" s="31">
+      <c r="V9" s="30">
         <v>5007.0</v>
       </c>
-      <c r="W9" s="31">
+      <c r="W9" s="30">
         <v>5006.0</v>
       </c>
-      <c r="X9" s="31">
+      <c r="X9" s="30">
         <v>2008.0</v>
       </c>
-      <c r="Y9" s="31">
+      <c r="Y9" s="30">
         <v>2005.0</v>
       </c>
-      <c r="Z9" s="31">
+      <c r="Z9" s="30">
         <v>2037.0</v>
       </c>
-      <c r="AA9" s="31">
+      <c r="AA9" s="30">
         <v>2025.0</v>
       </c>
-      <c r="AB9" s="31">
+      <c r="AB9" s="30">
         <v>2022.0</v>
       </c>
-      <c r="AC9" s="31" t="s">
+      <c r="AC9" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="AD9" s="30"/>
-      <c r="AE9" s="30"/>
-      <c r="AF9" s="30"/>
+      <c r="AD9" s="29"/>
+      <c r="AE9" s="29"/>
+      <c r="AF9" s="29"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="22" t="s">
@@ -5912,7 +5906,7 @@
       <c r="G10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="32">
+      <c r="H10" s="31">
         <f> IFERROR(IF(A10="No data","",IF(B10&lt;&gt;0, G10/B10, 0)),0)</f>
         <v>0</v>
       </c>
@@ -5923,7 +5917,7 @@
         <v>97</v>
       </c>
       <c r="K10" s="2">
-        <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10+AE10),0)</f>
+        <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
         <v>0</v>
       </c>
       <c r="L10" s="2">
@@ -5988,7 +5982,7 @@
       <c r="AD10" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="AE10" s="33" t="s">
+      <c r="AE10" s="2" t="s">
         <v>112</v>
       </c>
       <c r="AF10" s="2">
@@ -13723,8 +13717,8 @@
     <mergeCell ref="M8:M9"/>
     <mergeCell ref="N8:N9"/>
     <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="AE8:AE9"/>
     <mergeCell ref="AF8:AF9"/>
-    <mergeCell ref="AE8:AE9"/>
     <mergeCell ref="O8:O9"/>
     <mergeCell ref="P8:P9"/>
     <mergeCell ref="Q8:Q9"/>
@@ -13879,7 +13873,7 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8" ht="15.0" customHeight="1">
-      <c r="A8" s="34" t="s">
+      <c r="A8" s="32" t="s">
         <v>8</v>
       </c>
       <c r="B8" s="26" t="s">
@@ -13893,44 +13887,44 @@
       <c r="H8" s="27"/>
       <c r="I8" s="27"/>
       <c r="J8" s="28"/>
-      <c r="K8" s="35" t="s">
+      <c r="K8" s="33" t="s">
         <v>114</v>
       </c>
-      <c r="L8" s="35" t="s">
+      <c r="L8" s="33" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" ht="31.5" customHeight="1">
-      <c r="A9" s="30"/>
-      <c r="B9" s="31">
+      <c r="A9" s="29"/>
+      <c r="B9" s="30">
         <v>5011.0</v>
       </c>
-      <c r="C9" s="31">
+      <c r="C9" s="30">
         <v>5007.0</v>
       </c>
-      <c r="D9" s="31">
+      <c r="D9" s="30">
         <v>5006.0</v>
       </c>
-      <c r="E9" s="31">
+      <c r="E9" s="30">
         <v>2008.0</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="30">
         <v>2005.0</v>
       </c>
-      <c r="G9" s="31">
+      <c r="G9" s="30">
         <v>2037.0</v>
       </c>
-      <c r="H9" s="31">
+      <c r="H9" s="30">
         <v>2025.0</v>
       </c>
-      <c r="I9" s="31">
+      <c r="I9" s="30">
         <v>2022.0</v>
       </c>
-      <c r="J9" s="31" t="s">
+      <c r="J9" s="30" t="s">
         <v>90</v>
       </c>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30"/>
+      <c r="K9" s="29"/>
+      <c r="L9" s="29"/>
     </row>
     <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="22" t="s">
@@ -17525,288 +17519,288 @@
       </c>
     </row>
     <row r="2" ht="21.75" customHeight="1">
-      <c r="A2" s="36">
+      <c r="A2" s="34">
         <v>1001.0</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C2" s="36" t="s">
+      <c r="C2" s="34" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="3" ht="21.75" customHeight="1">
-      <c r="A3" s="36">
+      <c r="A3" s="34">
         <v>1002.0</v>
       </c>
-      <c r="B3" s="36" t="s">
+      <c r="B3" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="36" t="s">
+      <c r="C3" s="34" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="4" ht="21.75" customHeight="1">
-      <c r="A4" s="36">
+      <c r="A4" s="34">
         <v>1004.0</v>
       </c>
-      <c r="B4" s="36" t="s">
+      <c r="B4" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="36" t="s">
+      <c r="C4" s="34" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="5" ht="21.75" customHeight="1">
-      <c r="A5" s="36">
+      <c r="A5" s="34">
         <v>1005.0</v>
       </c>
-      <c r="B5" s="36" t="s">
+      <c r="B5" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C5" s="36" t="s">
+      <c r="C5" s="34" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="6" ht="21.75" customHeight="1">
-      <c r="A6" s="36">
+      <c r="A6" s="34">
         <v>1006.0</v>
       </c>
-      <c r="B6" s="36" t="s">
+      <c r="B6" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="36" t="s">
+      <c r="C6" s="34" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="7" ht="21.75" customHeight="1">
-      <c r="A7" s="36">
+      <c r="A7" s="34">
         <v>1007.0</v>
       </c>
-      <c r="B7" s="36" t="s">
+      <c r="B7" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C7" s="36" t="s">
+      <c r="C7" s="34" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="8" ht="21.75" customHeight="1">
-      <c r="A8" s="36">
+      <c r="A8" s="34">
         <v>1017.0</v>
       </c>
-      <c r="B8" s="36" t="s">
+      <c r="B8" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="36" t="s">
+      <c r="C8" s="34" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="9" ht="21.75" customHeight="1">
-      <c r="A9" s="36">
+      <c r="A9" s="34">
         <v>1018.0</v>
       </c>
-      <c r="B9" s="36" t="s">
+      <c r="B9" s="34" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="36" t="s">
+      <c r="C9" s="34" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="10" ht="21.75" customHeight="1">
-      <c r="A10" s="36">
+      <c r="A10" s="34">
         <v>2003.0</v>
       </c>
-      <c r="B10" s="36" t="s">
+      <c r="B10" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="34" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="11" ht="21.75" customHeight="1">
-      <c r="A11" s="36">
+      <c r="A11" s="34">
         <v>2005.0</v>
       </c>
-      <c r="B11" s="36" t="s">
+      <c r="B11" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C11" s="34" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="12" ht="21.75" customHeight="1">
-      <c r="A12" s="36">
+      <c r="A12" s="34">
         <v>2008.0</v>
       </c>
-      <c r="B12" s="36" t="s">
+      <c r="B12" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C12" s="36" t="s">
+      <c r="C12" s="34" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="13" ht="21.75" customHeight="1">
-      <c r="A13" s="36">
+      <c r="A13" s="34">
         <v>2009.0</v>
       </c>
-      <c r="B13" s="36" t="s">
+      <c r="B13" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C13" s="36" t="s">
+      <c r="C13" s="34" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="14" ht="21.75" customHeight="1">
-      <c r="A14" s="36">
+      <c r="A14" s="34">
         <v>2011.0</v>
       </c>
-      <c r="B14" s="36" t="s">
+      <c r="B14" s="34" t="s">
         <v>132</v>
       </c>
-      <c r="C14" s="36" t="s">
+      <c r="C14" s="34" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="15" ht="21.75" customHeight="1">
-      <c r="A15" s="36">
+      <c r="A15" s="34">
         <v>2014.0</v>
       </c>
-      <c r="B15" s="36" t="s">
+      <c r="B15" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C15" s="36" t="s">
+      <c r="C15" s="34" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="16" ht="21.75" customHeight="1">
-      <c r="A16" s="36">
+      <c r="A16" s="34">
         <v>2016.0</v>
       </c>
-      <c r="B16" s="36" t="s">
+      <c r="B16" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C16" s="36" t="s">
+      <c r="C16" s="34" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="17" ht="21.75" customHeight="1">
-      <c r="A17" s="36">
+      <c r="A17" s="34">
         <v>2018.0</v>
       </c>
-      <c r="B17" s="36" t="s">
+      <c r="B17" s="34" t="s">
         <v>132</v>
       </c>
-      <c r="C17" s="36" t="s">
+      <c r="C17" s="34" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="18" ht="21.75" customHeight="1">
-      <c r="A18" s="36">
+      <c r="A18" s="34">
         <v>2022.0</v>
       </c>
-      <c r="B18" s="36" t="s">
+      <c r="B18" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C18" s="36" t="s">
+      <c r="C18" s="34" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="19" ht="21.75" customHeight="1">
-      <c r="A19" s="36">
+      <c r="A19" s="34">
         <v>2025.0</v>
       </c>
-      <c r="B19" s="36" t="s">
+      <c r="B19" s="34" t="s">
         <v>132</v>
       </c>
-      <c r="C19" s="36" t="s">
+      <c r="C19" s="34" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="20" ht="21.75" customHeight="1">
-      <c r="A20" s="36">
+      <c r="A20" s="34">
         <v>2032.0</v>
       </c>
-      <c r="B20" s="36" t="s">
+      <c r="B20" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C20" s="36" t="s">
+      <c r="C20" s="34" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="21" ht="21.75" customHeight="1">
-      <c r="A21" s="36">
+      <c r="A21" s="34">
         <v>2034.0</v>
       </c>
-      <c r="B21" s="36" t="s">
+      <c r="B21" s="34" t="s">
         <v>127</v>
       </c>
-      <c r="C21" s="36" t="s">
+      <c r="C21" s="34" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="22" ht="21.75" customHeight="1">
-      <c r="A22" s="36">
+      <c r="A22" s="34">
         <v>2037.0</v>
       </c>
-      <c r="B22" s="36" t="s">
+      <c r="B22" s="34" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="36" t="s">
+      <c r="C22" s="34" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="23" ht="21.75" customHeight="1">
-      <c r="A23" s="36">
+      <c r="A23" s="34">
         <v>4010.0</v>
       </c>
-      <c r="B23" s="36" t="s">
+      <c r="B23" s="34" t="s">
         <v>142</v>
       </c>
-      <c r="C23" s="36" t="s">
+      <c r="C23" s="34" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="24" ht="21.75" customHeight="1">
-      <c r="A24" s="36">
+      <c r="A24" s="34">
         <v>4017.0</v>
       </c>
-      <c r="B24" s="36" t="s">
+      <c r="B24" s="34" t="s">
         <v>142</v>
       </c>
-      <c r="C24" s="36" t="s">
+      <c r="C24" s="34" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="25" ht="21.75" customHeight="1">
-      <c r="A25" s="36">
+      <c r="A25" s="34">
         <v>5006.0</v>
       </c>
-      <c r="B25" s="36" t="s">
+      <c r="B25" s="34" t="s">
         <v>144</v>
       </c>
-      <c r="C25" s="36" t="s">
+      <c r="C25" s="34" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="26" ht="21.75" customHeight="1">
-      <c r="A26" s="36">
+      <c r="A26" s="34">
         <v>5007.0</v>
       </c>
-      <c r="B26" s="36" t="s">
+      <c r="B26" s="34" t="s">
         <v>144</v>
       </c>
-      <c r="C26" s="36" t="s">
+      <c r="C26" s="34" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="27" ht="21.75" customHeight="1">
-      <c r="A27" s="36">
+      <c r="A27" s="34">
         <v>5011.0</v>
       </c>
-      <c r="B27" s="36" t="s">
+      <c r="B27" s="34" t="s">
         <v>144</v>
       </c>
-      <c r="C27" s="36" t="s">
+      <c r="C27" s="34" t="s">
         <v>147</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[feat/ASP-7746-Device-and-Sites-Summary-Report-include-Total-line] Fixed formats while streaming report
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_and_site_summary_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10D57388-7204-2E47-82F4-34A5A699F8CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B16E878-D488-A249-B3B0-BBFE867B3109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -781,6 +781,15 @@
     </xf>
     <xf numFmtId="165" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -808,15 +817,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1097,11 +1097,11 @@
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
       <c r="H2" s="5"/>
       <c r="J2" s="2"/>
       <c r="K2" s="3"/>
@@ -1117,11 +1117,11 @@
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="27"/>
-      <c r="D3" s="26"/>
-      <c r="E3" s="26"/>
-      <c r="F3" s="26"/>
-      <c r="G3" s="26"/>
+      <c r="C3" s="30"/>
+      <c r="D3" s="29"/>
+      <c r="E3" s="29"/>
+      <c r="F3" s="29"/>
+      <c r="G3" s="29"/>
       <c r="H3" s="5"/>
       <c r="J3" s="2"/>
       <c r="K3" s="3"/>
@@ -1137,9 +1137,9 @@
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="26"/>
-      <c r="F4" s="26"/>
-      <c r="G4" s="26"/>
+      <c r="E4" s="29"/>
+      <c r="F4" s="29"/>
+      <c r="G4" s="29"/>
       <c r="H4" s="5"/>
       <c r="J4" s="2"/>
       <c r="K4" s="3"/>
@@ -1155,9 +1155,9 @@
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="26"/>
-      <c r="F5" s="26"/>
-      <c r="G5" s="26"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
+      <c r="G5" s="29"/>
       <c r="H5" s="5"/>
       <c r="J5" s="2"/>
       <c r="K5" s="3"/>
@@ -1173,9 +1173,9 @@
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="26"/>
-      <c r="F6" s="26"/>
-      <c r="G6" s="26"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="29"/>
+      <c r="G6" s="29"/>
       <c r="J6" s="2"/>
       <c r="K6" s="3"/>
       <c r="L6" s="2"/>
@@ -4474,13 +4474,13 @@
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="28" t="s">
+      <c r="C2" s="31" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="26"/>
-      <c r="E2" s="26"/>
-      <c r="F2" s="26"/>
-      <c r="G2" s="26"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
@@ -5848,108 +5848,108 @@
       <c r="AF7" s="2"/>
     </row>
     <row r="8" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="29" t="s">
+      <c r="A8" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="31" t="s">
+      <c r="B8" s="34" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="31" t="s">
+      <c r="C8" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="31" t="s">
+      <c r="D8" s="34" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="31" t="s">
+      <c r="E8" s="34" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="31" t="s">
+      <c r="F8" s="34" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="31" t="s">
+      <c r="G8" s="34" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="31" t="s">
+      <c r="H8" s="34" t="s">
         <v>73</v>
       </c>
-      <c r="I8" s="31" t="s">
+      <c r="I8" s="34" t="s">
         <v>74</v>
       </c>
-      <c r="J8" s="31" t="s">
+      <c r="J8" s="34" t="s">
         <v>75</v>
       </c>
-      <c r="K8" s="31" t="s">
+      <c r="K8" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="L8" s="31" t="s">
+      <c r="L8" s="34" t="s">
         <v>77</v>
       </c>
-      <c r="M8" s="31" t="s">
+      <c r="M8" s="34" t="s">
         <v>78</v>
       </c>
-      <c r="N8" s="31" t="s">
+      <c r="N8" s="34" t="s">
         <v>79</v>
       </c>
-      <c r="O8" s="31" t="s">
+      <c r="O8" s="34" t="s">
         <v>80</v>
       </c>
-      <c r="P8" s="31" t="s">
+      <c r="P8" s="34" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="31" t="s">
+      <c r="Q8" s="34" t="s">
         <v>82</v>
       </c>
-      <c r="R8" s="31" t="s">
+      <c r="R8" s="34" t="s">
         <v>83</v>
       </c>
-      <c r="S8" s="31" t="s">
+      <c r="S8" s="34" t="s">
         <v>84</v>
       </c>
-      <c r="T8" s="31" t="s">
+      <c r="T8" s="34" t="s">
         <v>85</v>
       </c>
-      <c r="U8" s="32" t="s">
+      <c r="U8" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="V8" s="33"/>
-      <c r="W8" s="33"/>
-      <c r="X8" s="33"/>
-      <c r="Y8" s="33"/>
-      <c r="Z8" s="33"/>
-      <c r="AA8" s="33"/>
-      <c r="AB8" s="33"/>
-      <c r="AC8" s="34"/>
-      <c r="AD8" s="29" t="s">
+      <c r="V8" s="36"/>
+      <c r="W8" s="36"/>
+      <c r="X8" s="36"/>
+      <c r="Y8" s="36"/>
+      <c r="Z8" s="36"/>
+      <c r="AA8" s="36"/>
+      <c r="AB8" s="36"/>
+      <c r="AC8" s="37"/>
+      <c r="AD8" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="AE8" s="29" t="s">
+      <c r="AE8" s="32" t="s">
         <v>88</v>
       </c>
-      <c r="AF8" s="29" t="s">
+      <c r="AF8" s="32" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="30"/>
-      <c r="B9" s="30"/>
-      <c r="C9" s="30"/>
-      <c r="D9" s="30"/>
-      <c r="E9" s="30"/>
-      <c r="F9" s="30"/>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-      <c r="I9" s="30"/>
-      <c r="J9" s="30"/>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30"/>
-      <c r="M9" s="30"/>
-      <c r="N9" s="30"/>
-      <c r="O9" s="30"/>
-      <c r="P9" s="30"/>
-      <c r="Q9" s="30"/>
-      <c r="R9" s="30"/>
-      <c r="S9" s="30"/>
-      <c r="T9" s="30"/>
+      <c r="A9" s="33"/>
+      <c r="B9" s="33"/>
+      <c r="C9" s="33"/>
+      <c r="D9" s="33"/>
+      <c r="E9" s="33"/>
+      <c r="F9" s="33"/>
+      <c r="G9" s="33"/>
+      <c r="H9" s="33"/>
+      <c r="I9" s="33"/>
+      <c r="J9" s="33"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="33"/>
+      <c r="M9" s="33"/>
+      <c r="N9" s="33"/>
+      <c r="O9" s="33"/>
+      <c r="P9" s="33"/>
+      <c r="Q9" s="33"/>
+      <c r="R9" s="33"/>
+      <c r="S9" s="33"/>
+      <c r="T9" s="33"/>
       <c r="U9" s="21">
         <v>5011</v>
       </c>
@@ -5977,12 +5977,12 @@
       <c r="AC9" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="AD9" s="30"/>
-      <c r="AE9" s="30"/>
-      <c r="AF9" s="30"/>
+      <c r="AD9" s="33"/>
+      <c r="AE9" s="33"/>
+      <c r="AF9" s="33"/>
     </row>
     <row r="10" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="37" t="s">
+      <c r="A10" s="25" t="s">
         <v>91</v>
       </c>
       <c r="B10" s="16" t="s">
@@ -5997,14 +5997,14 @@
       <c r="E10" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="38">
+      <c r="F10" s="26">
         <f>IFERROR(IF(A10="No data","",IF(C10=0,0,D10/C10)),0)</f>
         <v>0</v>
       </c>
       <c r="G10" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="39">
+      <c r="H10" s="27">
         <f>IFERROR(IF(A10="No data","",IF(B10&lt;&gt;0, G10/B10, 0)),0)</f>
         <v>0</v>
       </c>
@@ -6018,19 +6018,19 @@
         <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="38">
+      <c r="L10" s="26">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,I10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="38">
+      <c r="M10" s="26">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,J10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="N10" s="38">
+      <c r="N10" s="26">
         <f>IFERROR(IF(A10="No data","",IF(D10=0,0,I10/D10)),0)</f>
         <v>0</v>
       </c>
-      <c r="O10" s="38">
+      <c r="O10" s="26">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,K10/G10)),0)</f>
         <v>0</v>
       </c>
@@ -6043,7 +6043,7 @@
       <c r="R10" s="16" t="s">
         <v>100</v>
       </c>
-      <c r="S10" s="38">
+      <c r="S10" s="26">
         <f>IFERROR(IF(A10="No data","",IF(I10=0,0,R10/I10)),0)</f>
         <v>0</v>
       </c>
@@ -13800,6 +13800,21 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="AD8:AD9"/>
     <mergeCell ref="AE8:AE9"/>
     <mergeCell ref="AF8:AF9"/>
     <mergeCell ref="O8:O9"/>
@@ -13809,21 +13824,6 @@
     <mergeCell ref="S8:S9"/>
     <mergeCell ref="T8:T9"/>
     <mergeCell ref="U8:AC8"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
   </mergeCells>
   <conditionalFormatting sqref="H10">
     <cfRule type="notContainsBlanks" dxfId="2" priority="1">
@@ -13967,29 +13967,29 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="35" t="s">
+      <c r="A8" s="38" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="35" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="33"/>
-      <c r="D8" s="33"/>
-      <c r="E8" s="33"/>
-      <c r="F8" s="33"/>
-      <c r="G8" s="33"/>
-      <c r="H8" s="33"/>
-      <c r="I8" s="33"/>
-      <c r="J8" s="34"/>
-      <c r="K8" s="36" t="s">
+      <c r="C8" s="36"/>
+      <c r="D8" s="36"/>
+      <c r="E8" s="36"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="36"/>
+      <c r="H8" s="36"/>
+      <c r="I8" s="36"/>
+      <c r="J8" s="37"/>
+      <c r="K8" s="39" t="s">
         <v>114</v>
       </c>
-      <c r="L8" s="36" t="s">
+      <c r="L8" s="39" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="30"/>
+      <c r="A9" s="33"/>
       <c r="B9" s="21">
         <v>5011</v>
       </c>
@@ -14017,8 +14017,8 @@
       <c r="J9" s="21" t="s">
         <v>90</v>
       </c>
-      <c r="K9" s="30"/>
-      <c r="L9" s="30"/>
+      <c r="K9" s="33"/>
+      <c r="L9" s="33"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="19" t="s">

</xml_diff>

<commit_message>
[feat/ASP-7746-Device-and-Sites-Summary-Report-include-Total-line] Fixed format and sum totals in dynamic columns
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_and_site_summary_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B16E878-D488-A249-B3B0-BBFE867B3109}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACB0970F-FE9C-8E4E-AC4A-E1D297E03903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="205" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="151">
   <si>
     <t>Device and Site Summary Report</t>
   </si>
@@ -514,16 +514,19 @@
   <si>
     <t>&lt;unreconciledResults&gt;</t>
   </si>
+  <si>
+    <t>#SUM_DYNAMIC</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -588,8 +591,15 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -608,8 +618,14 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFABEBEF"/>
+        <bgColor theme="4" tint="0.79995117038483843"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="9">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -721,11 +737,108 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -752,18 +865,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -776,9 +880,6 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -790,6 +891,65 @@
     <xf numFmtId="10" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -822,7 +982,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -847,8 +1007,24 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <fgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="1" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16">
+    <tableStyle name="Table Style 1" pivot="0" count="1" xr9:uid="{19082F53-8A79-6F4D-9D2A-0030ECE45304}">
+      <tableStyleElement type="wholeTable" dxfId="3"/>
+    </tableStyle>
+  </tableStyles>
+  <colors>
+    <mruColors>
+      <color rgb="FFABEBEF"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1058,7 +1234,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:T1000"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="3" width="27" customWidth="1"/>
@@ -1066,7 +1242,9 @@
     <col min="5" max="5" width="31.1640625" customWidth="1"/>
     <col min="6" max="9" width="19" customWidth="1"/>
     <col min="10" max="10" width="14.6640625" customWidth="1"/>
-    <col min="11" max="14" width="14.33203125" customWidth="1"/>
+    <col min="11" max="12" width="14.33203125" customWidth="1"/>
+    <col min="13" max="13" width="22.33203125" customWidth="1"/>
+    <col min="14" max="14" width="14.33203125" customWidth="1"/>
     <col min="15" max="15" width="13.1640625" customWidth="1"/>
     <col min="16" max="16" width="10.5" customWidth="1"/>
     <col min="17" max="17" width="18.1640625" customWidth="1"/>
@@ -1075,7 +1253,7 @@
     <col min="20" max="20" width="11.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1093,15 +1271,15 @@
       <c r="Q1" s="2"/>
       <c r="R1" s="3"/>
     </row>
-    <row r="2" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="28" t="s">
+      <c r="E2" s="45" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
       <c r="H2" s="5"/>
       <c r="J2" s="2"/>
       <c r="K2" s="3"/>
@@ -1113,15 +1291,15 @@
       <c r="Q2" s="2"/>
       <c r="R2" s="3"/>
     </row>
-    <row r="3" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
-      <c r="F3" s="29"/>
-      <c r="G3" s="29"/>
+      <c r="C3" s="47"/>
+      <c r="D3" s="46"/>
+      <c r="E3" s="46"/>
+      <c r="F3" s="46"/>
+      <c r="G3" s="46"/>
       <c r="H3" s="5"/>
       <c r="J3" s="2"/>
       <c r="K3" s="3"/>
@@ -1133,13 +1311,13 @@
       <c r="Q3" s="2"/>
       <c r="R3" s="3"/>
     </row>
-    <row r="4" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="29"/>
-      <c r="F4" s="29"/>
-      <c r="G4" s="29"/>
+      <c r="E4" s="46"/>
+      <c r="F4" s="46"/>
+      <c r="G4" s="46"/>
       <c r="H4" s="5"/>
       <c r="J4" s="2"/>
       <c r="K4" s="3"/>
@@ -1151,13 +1329,13 @@
       <c r="Q4" s="2"/>
       <c r="R4" s="3"/>
     </row>
-    <row r="5" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="29"/>
-      <c r="F5" s="29"/>
-      <c r="G5" s="29"/>
+      <c r="E5" s="46"/>
+      <c r="F5" s="46"/>
+      <c r="G5" s="46"/>
       <c r="H5" s="5"/>
       <c r="J5" s="2"/>
       <c r="K5" s="3"/>
@@ -1169,13 +1347,13 @@
       <c r="Q5" s="2"/>
       <c r="R5" s="3"/>
     </row>
-    <row r="6" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:21" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="29"/>
-      <c r="F6" s="29"/>
-      <c r="G6" s="29"/>
+      <c r="E6" s="46"/>
+      <c r="F6" s="46"/>
+      <c r="G6" s="46"/>
       <c r="J6" s="2"/>
       <c r="K6" s="3"/>
       <c r="L6" s="2"/>
@@ -1186,7 +1364,7 @@
       <c r="Q6" s="2"/>
       <c r="R6" s="3"/>
     </row>
-    <row r="7" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:21" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>7</v>
       </c>
@@ -1202,7 +1380,7 @@
       <c r="Q7" s="2"/>
       <c r="R7" s="3"/>
     </row>
-    <row r="8" spans="1:20" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:21" ht="67.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
         <v>8</v>
       </c>
@@ -1264,3174 +1442,99 @@
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:21" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="41" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="41" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="41" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="41" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="41" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="12" t="s">
+      <c r="F9" s="40" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="13" t="s">
+      <c r="G9" s="41" t="s">
         <v>34</v>
       </c>
-      <c r="H9" s="13" t="s">
+      <c r="H9" s="41" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="12" t="s">
+      <c r="I9" s="40" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="14" t="s">
+      <c r="J9" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="15" t="s">
+      <c r="K9" s="42" t="s">
         <v>38</v>
       </c>
-      <c r="L9" s="16" t="s">
+      <c r="L9" s="43" t="s">
         <v>39</v>
       </c>
-      <c r="M9" s="16" t="s">
+      <c r="M9" s="43" t="s">
         <v>40</v>
       </c>
-      <c r="N9" s="16" t="s">
+      <c r="N9" s="43" t="s">
         <v>41</v>
       </c>
-      <c r="O9" s="16" t="s">
+      <c r="O9" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="P9" s="16" t="s">
+      <c r="P9" s="43" t="s">
         <v>43</v>
       </c>
-      <c r="Q9" s="16" t="s">
+      <c r="Q9" s="43" t="s">
         <v>44</v>
       </c>
-      <c r="R9" s="15" t="s">
+      <c r="R9" s="42" t="s">
         <v>45</v>
       </c>
-      <c r="S9" s="10" t="s">
+      <c r="S9" s="39" t="s">
         <v>46</v>
       </c>
-      <c r="T9" s="10" t="s">
+      <c r="T9" s="39" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J10" s="2"/>
-      <c r="K10" s="3"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
-      <c r="N10" s="2"/>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="3"/>
-    </row>
-    <row r="11" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="17"/>
-      <c r="B11" s="17"/>
-      <c r="C11" s="17"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="3"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="3"/>
-    </row>
-    <row r="12" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J12" s="2"/>
-      <c r="K12" s="3"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2"/>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="3"/>
-    </row>
-    <row r="13" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J13" s="2"/>
-      <c r="K13" s="3"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
-      <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2"/>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="3"/>
-    </row>
-    <row r="14" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J14" s="2"/>
-      <c r="K14" s="3"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="3"/>
-    </row>
-    <row r="15" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J15" s="2"/>
-      <c r="K15" s="3"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
-      <c r="N15" s="2"/>
-      <c r="O15" s="2"/>
-      <c r="P15" s="2"/>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="3"/>
-    </row>
-    <row r="16" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J16" s="2"/>
-      <c r="K16" s="3"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
-      <c r="N16" s="2"/>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2"/>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="3"/>
-    </row>
-    <row r="17" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J17" s="2"/>
-      <c r="K17" s="3"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
-      <c r="N17" s="2"/>
-      <c r="O17" s="2"/>
-      <c r="P17" s="2"/>
-      <c r="Q17" s="2"/>
-      <c r="R17" s="3"/>
-    </row>
-    <row r="18" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J18" s="2"/>
-      <c r="K18" s="3"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
-      <c r="N18" s="2"/>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
-      <c r="Q18" s="2"/>
-      <c r="R18" s="3"/>
-    </row>
-    <row r="19" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J19" s="2"/>
-      <c r="K19" s="3"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
-      <c r="N19" s="2"/>
-      <c r="O19" s="2"/>
-      <c r="P19" s="2"/>
-      <c r="Q19" s="2"/>
-      <c r="R19" s="3"/>
-    </row>
-    <row r="20" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J20" s="2"/>
-      <c r="K20" s="3"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-      <c r="N20" s="2"/>
-      <c r="O20" s="2"/>
-      <c r="P20" s="2"/>
-      <c r="Q20" s="2"/>
-      <c r="R20" s="3"/>
-    </row>
-    <row r="21" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J21" s="2"/>
-      <c r="K21" s="3"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
-      <c r="N21" s="2"/>
-      <c r="O21" s="2"/>
-      <c r="P21" s="2"/>
-      <c r="Q21" s="2"/>
-      <c r="R21" s="3"/>
-    </row>
-    <row r="22" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J22" s="2"/>
-      <c r="K22" s="3"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-      <c r="N22" s="2"/>
-      <c r="O22" s="2"/>
-      <c r="P22" s="2"/>
-      <c r="Q22" s="2"/>
-      <c r="R22" s="3"/>
-    </row>
-    <row r="23" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J23" s="2"/>
-      <c r="K23" s="3"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="2"/>
-      <c r="N23" s="2"/>
-      <c r="O23" s="2"/>
-      <c r="P23" s="2"/>
-      <c r="Q23" s="2"/>
-      <c r="R23" s="3"/>
-    </row>
-    <row r="24" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J24" s="2"/>
-      <c r="K24" s="3"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="3"/>
-    </row>
-    <row r="25" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J25" s="2"/>
-      <c r="K25" s="3"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-      <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
-      <c r="P25" s="2"/>
-      <c r="Q25" s="2"/>
-      <c r="R25" s="3"/>
-    </row>
-    <row r="26" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J26" s="2"/>
-      <c r="K26" s="3"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-      <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
-      <c r="P26" s="2"/>
-      <c r="Q26" s="2"/>
-      <c r="R26" s="3"/>
-    </row>
-    <row r="27" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J27" s="2"/>
-      <c r="K27" s="3"/>
-      <c r="L27" s="2"/>
-      <c r="M27" s="2"/>
-      <c r="N27" s="2"/>
-      <c r="O27" s="2"/>
-      <c r="P27" s="2"/>
-      <c r="Q27" s="2"/>
-      <c r="R27" s="3"/>
-    </row>
-    <row r="28" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J28" s="2"/>
-      <c r="K28" s="3"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-      <c r="N28" s="2"/>
-      <c r="O28" s="2"/>
-      <c r="P28" s="2"/>
-      <c r="Q28" s="2"/>
-      <c r="R28" s="3"/>
-    </row>
-    <row r="29" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J29" s="2"/>
-      <c r="K29" s="3"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-      <c r="N29" s="2"/>
-      <c r="O29" s="2"/>
-      <c r="P29" s="2"/>
-      <c r="Q29" s="2"/>
-      <c r="R29" s="3"/>
-    </row>
-    <row r="30" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J30" s="2"/>
-      <c r="K30" s="3"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-      <c r="N30" s="2"/>
-      <c r="O30" s="2"/>
-      <c r="P30" s="2"/>
-      <c r="Q30" s="2"/>
-      <c r="R30" s="3"/>
-    </row>
-    <row r="31" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J31" s="2"/>
-      <c r="K31" s="3"/>
-      <c r="L31" s="2"/>
-      <c r="M31" s="2"/>
-      <c r="N31" s="2"/>
-      <c r="O31" s="2"/>
-      <c r="P31" s="2"/>
-      <c r="Q31" s="2"/>
-      <c r="R31" s="3"/>
-    </row>
-    <row r="32" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J32" s="2"/>
-      <c r="K32" s="3"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-      <c r="N32" s="2"/>
-      <c r="O32" s="2"/>
-      <c r="P32" s="2"/>
-      <c r="Q32" s="2"/>
-      <c r="R32" s="3"/>
-    </row>
-    <row r="33" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J33" s="2"/>
-      <c r="K33" s="3"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
-      <c r="O33" s="2"/>
-      <c r="P33" s="2"/>
-      <c r="Q33" s="2"/>
-      <c r="R33" s="3"/>
-    </row>
-    <row r="34" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J34" s="2"/>
-      <c r="K34" s="3"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
-      <c r="N34" s="2"/>
-      <c r="O34" s="2"/>
-      <c r="P34" s="2"/>
-      <c r="Q34" s="2"/>
-      <c r="R34" s="3"/>
-    </row>
-    <row r="35" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J35" s="2"/>
-      <c r="K35" s="3"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
-      <c r="N35" s="2"/>
-      <c r="O35" s="2"/>
-      <c r="P35" s="2"/>
-      <c r="Q35" s="2"/>
-      <c r="R35" s="3"/>
-    </row>
-    <row r="36" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J36" s="2"/>
-      <c r="K36" s="3"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-      <c r="N36" s="2"/>
-      <c r="O36" s="2"/>
-      <c r="P36" s="2"/>
-      <c r="Q36" s="2"/>
-      <c r="R36" s="3"/>
-    </row>
-    <row r="37" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J37" s="2"/>
-      <c r="K37" s="3"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="2"/>
-      <c r="O37" s="2"/>
-      <c r="P37" s="2"/>
-      <c r="Q37" s="2"/>
-      <c r="R37" s="3"/>
-    </row>
-    <row r="38" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J38" s="2"/>
-      <c r="K38" s="3"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-      <c r="N38" s="2"/>
-      <c r="O38" s="2"/>
-      <c r="P38" s="2"/>
-      <c r="Q38" s="2"/>
-      <c r="R38" s="3"/>
-    </row>
-    <row r="39" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J39" s="2"/>
-      <c r="K39" s="3"/>
-      <c r="L39" s="2"/>
-      <c r="M39" s="2"/>
-      <c r="N39" s="2"/>
-      <c r="O39" s="2"/>
-      <c r="P39" s="2"/>
-      <c r="Q39" s="2"/>
-      <c r="R39" s="3"/>
-    </row>
-    <row r="40" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J40" s="2"/>
-      <c r="K40" s="3"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-      <c r="N40" s="2"/>
-      <c r="O40" s="2"/>
-      <c r="P40" s="2"/>
-      <c r="Q40" s="2"/>
-      <c r="R40" s="3"/>
-    </row>
-    <row r="41" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J41" s="2"/>
-      <c r="K41" s="3"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2"/>
-      <c r="P41" s="2"/>
-      <c r="Q41" s="2"/>
-      <c r="R41" s="3"/>
-    </row>
-    <row r="42" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J42" s="2"/>
-      <c r="K42" s="3"/>
-      <c r="L42" s="2"/>
-      <c r="M42" s="2"/>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2"/>
-      <c r="P42" s="2"/>
-      <c r="Q42" s="2"/>
-      <c r="R42" s="3"/>
-    </row>
-    <row r="43" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J43" s="2"/>
-      <c r="K43" s="3"/>
-      <c r="L43" s="2"/>
-      <c r="M43" s="2"/>
-      <c r="N43" s="2"/>
-      <c r="O43" s="2"/>
-      <c r="P43" s="2"/>
-      <c r="Q43" s="2"/>
-      <c r="R43" s="3"/>
-    </row>
-    <row r="44" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J44" s="2"/>
-      <c r="K44" s="3"/>
-      <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
-      <c r="N44" s="2"/>
-      <c r="O44" s="2"/>
-      <c r="P44" s="2"/>
-      <c r="Q44" s="2"/>
-      <c r="R44" s="3"/>
-    </row>
-    <row r="45" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J45" s="2"/>
-      <c r="K45" s="3"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
-      <c r="P45" s="2"/>
-      <c r="Q45" s="2"/>
-      <c r="R45" s="3"/>
-    </row>
-    <row r="46" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J46" s="2"/>
-      <c r="K46" s="3"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
-      <c r="N46" s="2"/>
-      <c r="O46" s="2"/>
-      <c r="P46" s="2"/>
-      <c r="Q46" s="2"/>
-      <c r="R46" s="3"/>
-    </row>
-    <row r="47" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J47" s="2"/>
-      <c r="K47" s="3"/>
-      <c r="L47" s="2"/>
-      <c r="M47" s="2"/>
-      <c r="N47" s="2"/>
-      <c r="O47" s="2"/>
-      <c r="P47" s="2"/>
-      <c r="Q47" s="2"/>
-      <c r="R47" s="3"/>
-    </row>
-    <row r="48" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J48" s="2"/>
-      <c r="K48" s="3"/>
-      <c r="L48" s="2"/>
-      <c r="M48" s="2"/>
-      <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
-      <c r="P48" s="2"/>
-      <c r="Q48" s="2"/>
-      <c r="R48" s="3"/>
-    </row>
-    <row r="49" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J49" s="2"/>
-      <c r="K49" s="3"/>
-      <c r="L49" s="2"/>
-      <c r="M49" s="2"/>
-      <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
-      <c r="P49" s="2"/>
-      <c r="Q49" s="2"/>
-      <c r="R49" s="3"/>
-    </row>
-    <row r="50" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J50" s="2"/>
-      <c r="K50" s="3"/>
-      <c r="L50" s="2"/>
-      <c r="M50" s="2"/>
-      <c r="N50" s="2"/>
-      <c r="O50" s="2"/>
-      <c r="P50" s="2"/>
-      <c r="Q50" s="2"/>
-      <c r="R50" s="3"/>
-    </row>
-    <row r="51" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J51" s="2"/>
-      <c r="K51" s="3"/>
-      <c r="L51" s="2"/>
-      <c r="M51" s="2"/>
-      <c r="N51" s="2"/>
-      <c r="O51" s="2"/>
-      <c r="P51" s="2"/>
-      <c r="Q51" s="2"/>
-      <c r="R51" s="3"/>
-    </row>
-    <row r="52" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J52" s="2"/>
-      <c r="K52" s="3"/>
-      <c r="L52" s="2"/>
-      <c r="M52" s="2"/>
-      <c r="N52" s="2"/>
-      <c r="O52" s="2"/>
-      <c r="P52" s="2"/>
-      <c r="Q52" s="2"/>
-      <c r="R52" s="3"/>
-    </row>
-    <row r="53" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J53" s="2"/>
-      <c r="K53" s="3"/>
-      <c r="L53" s="2"/>
-      <c r="M53" s="2"/>
-      <c r="N53" s="2"/>
-      <c r="O53" s="2"/>
-      <c r="P53" s="2"/>
-      <c r="Q53" s="2"/>
-      <c r="R53" s="3"/>
-    </row>
-    <row r="54" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J54" s="2"/>
-      <c r="K54" s="3"/>
-      <c r="L54" s="2"/>
-      <c r="M54" s="2"/>
-      <c r="N54" s="2"/>
-      <c r="O54" s="2"/>
-      <c r="P54" s="2"/>
-      <c r="Q54" s="2"/>
-      <c r="R54" s="3"/>
-    </row>
-    <row r="55" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J55" s="2"/>
-      <c r="K55" s="3"/>
-      <c r="L55" s="2"/>
-      <c r="M55" s="2"/>
-      <c r="N55" s="2"/>
-      <c r="O55" s="2"/>
-      <c r="P55" s="2"/>
-      <c r="Q55" s="2"/>
-      <c r="R55" s="3"/>
-    </row>
-    <row r="56" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J56" s="2"/>
-      <c r="K56" s="3"/>
-      <c r="L56" s="2"/>
-      <c r="M56" s="2"/>
-      <c r="N56" s="2"/>
-      <c r="O56" s="2"/>
-      <c r="P56" s="2"/>
-      <c r="Q56" s="2"/>
-      <c r="R56" s="3"/>
-    </row>
-    <row r="57" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J57" s="2"/>
-      <c r="K57" s="3"/>
-      <c r="L57" s="2"/>
-      <c r="M57" s="2"/>
-      <c r="N57" s="2"/>
-      <c r="O57" s="2"/>
-      <c r="P57" s="2"/>
-      <c r="Q57" s="2"/>
-      <c r="R57" s="3"/>
-    </row>
-    <row r="58" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J58" s="2"/>
-      <c r="K58" s="3"/>
-      <c r="L58" s="2"/>
-      <c r="M58" s="2"/>
-      <c r="N58" s="2"/>
-      <c r="O58" s="2"/>
-      <c r="P58" s="2"/>
-      <c r="Q58" s="2"/>
-      <c r="R58" s="3"/>
-    </row>
-    <row r="59" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J59" s="2"/>
-      <c r="K59" s="3"/>
-      <c r="L59" s="2"/>
-      <c r="M59" s="2"/>
-      <c r="N59" s="2"/>
-      <c r="O59" s="2"/>
-      <c r="P59" s="2"/>
-      <c r="Q59" s="2"/>
-      <c r="R59" s="3"/>
-    </row>
-    <row r="60" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J60" s="2"/>
-      <c r="K60" s="3"/>
-      <c r="L60" s="2"/>
-      <c r="M60" s="2"/>
-      <c r="N60" s="2"/>
-      <c r="O60" s="2"/>
-      <c r="P60" s="2"/>
-      <c r="Q60" s="2"/>
-      <c r="R60" s="3"/>
-    </row>
-    <row r="61" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J61" s="2"/>
-      <c r="K61" s="3"/>
-      <c r="L61" s="2"/>
-      <c r="M61" s="2"/>
-      <c r="N61" s="2"/>
-      <c r="O61" s="2"/>
-      <c r="P61" s="2"/>
-      <c r="Q61" s="2"/>
-      <c r="R61" s="3"/>
-    </row>
-    <row r="62" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J62" s="2"/>
-      <c r="K62" s="3"/>
-      <c r="L62" s="2"/>
-      <c r="M62" s="2"/>
-      <c r="N62" s="2"/>
-      <c r="O62" s="2"/>
-      <c r="P62" s="2"/>
-      <c r="Q62" s="2"/>
-      <c r="R62" s="3"/>
-    </row>
-    <row r="63" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J63" s="2"/>
-      <c r="K63" s="3"/>
-      <c r="L63" s="2"/>
-      <c r="M63" s="2"/>
-      <c r="N63" s="2"/>
-      <c r="O63" s="2"/>
-      <c r="P63" s="2"/>
-      <c r="Q63" s="2"/>
-      <c r="R63" s="3"/>
-    </row>
-    <row r="64" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J64" s="2"/>
-      <c r="K64" s="3"/>
-      <c r="L64" s="2"/>
-      <c r="M64" s="2"/>
-      <c r="N64" s="2"/>
-      <c r="O64" s="2"/>
-      <c r="P64" s="2"/>
-      <c r="Q64" s="2"/>
-      <c r="R64" s="3"/>
-    </row>
-    <row r="65" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J65" s="2"/>
-      <c r="K65" s="3"/>
-      <c r="L65" s="2"/>
-      <c r="M65" s="2"/>
-      <c r="N65" s="2"/>
-      <c r="O65" s="2"/>
-      <c r="P65" s="2"/>
-      <c r="Q65" s="2"/>
-      <c r="R65" s="3"/>
-    </row>
-    <row r="66" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J66" s="2"/>
-      <c r="K66" s="3"/>
-      <c r="L66" s="2"/>
-      <c r="M66" s="2"/>
-      <c r="N66" s="2"/>
-      <c r="O66" s="2"/>
-      <c r="P66" s="2"/>
-      <c r="Q66" s="2"/>
-      <c r="R66" s="3"/>
-    </row>
-    <row r="67" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J67" s="2"/>
-      <c r="K67" s="3"/>
-      <c r="L67" s="2"/>
-      <c r="M67" s="2"/>
-      <c r="N67" s="2"/>
-      <c r="O67" s="2"/>
-      <c r="P67" s="2"/>
-      <c r="Q67" s="2"/>
-      <c r="R67" s="3"/>
-    </row>
-    <row r="68" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J68" s="2"/>
-      <c r="K68" s="3"/>
-      <c r="L68" s="2"/>
-      <c r="M68" s="2"/>
-      <c r="N68" s="2"/>
-      <c r="O68" s="2"/>
-      <c r="P68" s="2"/>
-      <c r="Q68" s="2"/>
-      <c r="R68" s="3"/>
-    </row>
-    <row r="69" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J69" s="2"/>
-      <c r="K69" s="3"/>
-      <c r="L69" s="2"/>
-      <c r="M69" s="2"/>
-      <c r="N69" s="2"/>
-      <c r="O69" s="2"/>
-      <c r="P69" s="2"/>
-      <c r="Q69" s="2"/>
-      <c r="R69" s="3"/>
-    </row>
-    <row r="70" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J70" s="2"/>
-      <c r="K70" s="3"/>
-      <c r="L70" s="2"/>
-      <c r="M70" s="2"/>
-      <c r="N70" s="2"/>
-      <c r="O70" s="2"/>
-      <c r="P70" s="2"/>
-      <c r="Q70" s="2"/>
-      <c r="R70" s="3"/>
-    </row>
-    <row r="71" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J71" s="2"/>
-      <c r="K71" s="3"/>
-      <c r="L71" s="2"/>
-      <c r="M71" s="2"/>
-      <c r="N71" s="2"/>
-      <c r="O71" s="2"/>
-      <c r="P71" s="2"/>
-      <c r="Q71" s="2"/>
-      <c r="R71" s="3"/>
-    </row>
-    <row r="72" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J72" s="2"/>
-      <c r="K72" s="3"/>
-      <c r="L72" s="2"/>
-      <c r="M72" s="2"/>
-      <c r="N72" s="2"/>
-      <c r="O72" s="2"/>
-      <c r="P72" s="2"/>
-      <c r="Q72" s="2"/>
-      <c r="R72" s="3"/>
-    </row>
-    <row r="73" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J73" s="2"/>
-      <c r="K73" s="3"/>
-      <c r="L73" s="2"/>
-      <c r="M73" s="2"/>
-      <c r="N73" s="2"/>
-      <c r="O73" s="2"/>
-      <c r="P73" s="2"/>
-      <c r="Q73" s="2"/>
-      <c r="R73" s="3"/>
-    </row>
-    <row r="74" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J74" s="2"/>
-      <c r="K74" s="3"/>
-      <c r="L74" s="2"/>
-      <c r="M74" s="2"/>
-      <c r="N74" s="2"/>
-      <c r="O74" s="2"/>
-      <c r="P74" s="2"/>
-      <c r="Q74" s="2"/>
-      <c r="R74" s="3"/>
-    </row>
-    <row r="75" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J75" s="2"/>
-      <c r="K75" s="3"/>
-      <c r="L75" s="2"/>
-      <c r="M75" s="2"/>
-      <c r="N75" s="2"/>
-      <c r="O75" s="2"/>
-      <c r="P75" s="2"/>
-      <c r="Q75" s="2"/>
-      <c r="R75" s="3"/>
-    </row>
-    <row r="76" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J76" s="2"/>
-      <c r="K76" s="3"/>
-      <c r="L76" s="2"/>
-      <c r="M76" s="2"/>
-      <c r="N76" s="2"/>
-      <c r="O76" s="2"/>
-      <c r="P76" s="2"/>
-      <c r="Q76" s="2"/>
-      <c r="R76" s="3"/>
-    </row>
-    <row r="77" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J77" s="2"/>
-      <c r="K77" s="3"/>
-      <c r="L77" s="2"/>
-      <c r="M77" s="2"/>
-      <c r="N77" s="2"/>
-      <c r="O77" s="2"/>
-      <c r="P77" s="2"/>
-      <c r="Q77" s="2"/>
-      <c r="R77" s="3"/>
-    </row>
-    <row r="78" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J78" s="2"/>
-      <c r="K78" s="3"/>
-      <c r="L78" s="2"/>
-      <c r="M78" s="2"/>
-      <c r="N78" s="2"/>
-      <c r="O78" s="2"/>
-      <c r="P78" s="2"/>
-      <c r="Q78" s="2"/>
-      <c r="R78" s="3"/>
-    </row>
-    <row r="79" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J79" s="2"/>
-      <c r="K79" s="3"/>
-      <c r="L79" s="2"/>
-      <c r="M79" s="2"/>
-      <c r="N79" s="2"/>
-      <c r="O79" s="2"/>
-      <c r="P79" s="2"/>
-      <c r="Q79" s="2"/>
-      <c r="R79" s="3"/>
-    </row>
-    <row r="80" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J80" s="2"/>
-      <c r="K80" s="3"/>
-      <c r="L80" s="2"/>
-      <c r="M80" s="2"/>
-      <c r="N80" s="2"/>
-      <c r="O80" s="2"/>
-      <c r="P80" s="2"/>
-      <c r="Q80" s="2"/>
-      <c r="R80" s="3"/>
-    </row>
-    <row r="81" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J81" s="2"/>
-      <c r="K81" s="3"/>
-      <c r="L81" s="2"/>
-      <c r="M81" s="2"/>
-      <c r="N81" s="2"/>
-      <c r="O81" s="2"/>
-      <c r="P81" s="2"/>
-      <c r="Q81" s="2"/>
-      <c r="R81" s="3"/>
-    </row>
-    <row r="82" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J82" s="2"/>
-      <c r="K82" s="3"/>
-      <c r="L82" s="2"/>
-      <c r="M82" s="2"/>
-      <c r="N82" s="2"/>
-      <c r="O82" s="2"/>
-      <c r="P82" s="2"/>
-      <c r="Q82" s="2"/>
-      <c r="R82" s="3"/>
-    </row>
-    <row r="83" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J83" s="2"/>
-      <c r="K83" s="3"/>
-      <c r="L83" s="2"/>
-      <c r="M83" s="2"/>
-      <c r="N83" s="2"/>
-      <c r="O83" s="2"/>
-      <c r="P83" s="2"/>
-      <c r="Q83" s="2"/>
-      <c r="R83" s="3"/>
-    </row>
-    <row r="84" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J84" s="2"/>
-      <c r="K84" s="3"/>
-      <c r="L84" s="2"/>
-      <c r="M84" s="2"/>
-      <c r="N84" s="2"/>
-      <c r="O84" s="2"/>
-      <c r="P84" s="2"/>
-      <c r="Q84" s="2"/>
-      <c r="R84" s="3"/>
-    </row>
-    <row r="85" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J85" s="2"/>
-      <c r="K85" s="3"/>
-      <c r="L85" s="2"/>
-      <c r="M85" s="2"/>
-      <c r="N85" s="2"/>
-      <c r="O85" s="2"/>
-      <c r="P85" s="2"/>
-      <c r="Q85" s="2"/>
-      <c r="R85" s="3"/>
-    </row>
-    <row r="86" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J86" s="2"/>
-      <c r="K86" s="3"/>
-      <c r="L86" s="2"/>
-      <c r="M86" s="2"/>
-      <c r="N86" s="2"/>
-      <c r="O86" s="2"/>
-      <c r="P86" s="2"/>
-      <c r="Q86" s="2"/>
-      <c r="R86" s="3"/>
-    </row>
-    <row r="87" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J87" s="2"/>
-      <c r="K87" s="3"/>
-      <c r="L87" s="2"/>
-      <c r="M87" s="2"/>
-      <c r="N87" s="2"/>
-      <c r="O87" s="2"/>
-      <c r="P87" s="2"/>
-      <c r="Q87" s="2"/>
-      <c r="R87" s="3"/>
-    </row>
-    <row r="88" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J88" s="2"/>
-      <c r="K88" s="3"/>
-      <c r="L88" s="2"/>
-      <c r="M88" s="2"/>
-      <c r="N88" s="2"/>
-      <c r="O88" s="2"/>
-      <c r="P88" s="2"/>
-      <c r="Q88" s="2"/>
-      <c r="R88" s="3"/>
-    </row>
-    <row r="89" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J89" s="2"/>
-      <c r="K89" s="3"/>
-      <c r="L89" s="2"/>
-      <c r="M89" s="2"/>
-      <c r="N89" s="2"/>
-      <c r="O89" s="2"/>
-      <c r="P89" s="2"/>
-      <c r="Q89" s="2"/>
-      <c r="R89" s="3"/>
-    </row>
-    <row r="90" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J90" s="2"/>
-      <c r="K90" s="3"/>
-      <c r="L90" s="2"/>
-      <c r="M90" s="2"/>
-      <c r="N90" s="2"/>
-      <c r="O90" s="2"/>
-      <c r="P90" s="2"/>
-      <c r="Q90" s="2"/>
-      <c r="R90" s="3"/>
-    </row>
-    <row r="91" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J91" s="2"/>
-      <c r="K91" s="3"/>
-      <c r="L91" s="2"/>
-      <c r="M91" s="2"/>
-      <c r="N91" s="2"/>
-      <c r="O91" s="2"/>
-      <c r="P91" s="2"/>
-      <c r="Q91" s="2"/>
-      <c r="R91" s="3"/>
-    </row>
-    <row r="92" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J92" s="2"/>
-      <c r="K92" s="3"/>
-      <c r="L92" s="2"/>
-      <c r="M92" s="2"/>
-      <c r="N92" s="2"/>
-      <c r="O92" s="2"/>
-      <c r="P92" s="2"/>
-      <c r="Q92" s="2"/>
-      <c r="R92" s="3"/>
-    </row>
-    <row r="93" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J93" s="2"/>
-      <c r="K93" s="3"/>
-      <c r="L93" s="2"/>
-      <c r="M93" s="2"/>
-      <c r="N93" s="2"/>
-      <c r="O93" s="2"/>
-      <c r="P93" s="2"/>
-      <c r="Q93" s="2"/>
-      <c r="R93" s="3"/>
-    </row>
-    <row r="94" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J94" s="2"/>
-      <c r="K94" s="3"/>
-      <c r="L94" s="2"/>
-      <c r="M94" s="2"/>
-      <c r="N94" s="2"/>
-      <c r="O94" s="2"/>
-      <c r="P94" s="2"/>
-      <c r="Q94" s="2"/>
-      <c r="R94" s="3"/>
-    </row>
-    <row r="95" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J95" s="2"/>
-      <c r="K95" s="3"/>
-      <c r="L95" s="2"/>
-      <c r="M95" s="2"/>
-      <c r="N95" s="2"/>
-      <c r="O95" s="2"/>
-      <c r="P95" s="2"/>
-      <c r="Q95" s="2"/>
-      <c r="R95" s="3"/>
-    </row>
-    <row r="96" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J96" s="2"/>
-      <c r="K96" s="3"/>
-      <c r="L96" s="2"/>
-      <c r="M96" s="2"/>
-      <c r="N96" s="2"/>
-      <c r="O96" s="2"/>
-      <c r="P96" s="2"/>
-      <c r="Q96" s="2"/>
-      <c r="R96" s="3"/>
-    </row>
-    <row r="97" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J97" s="2"/>
-      <c r="K97" s="3"/>
-      <c r="L97" s="2"/>
-      <c r="M97" s="2"/>
-      <c r="N97" s="2"/>
-      <c r="O97" s="2"/>
-      <c r="P97" s="2"/>
-      <c r="Q97" s="2"/>
-      <c r="R97" s="3"/>
-    </row>
-    <row r="98" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J98" s="2"/>
-      <c r="K98" s="3"/>
-      <c r="L98" s="2"/>
-      <c r="M98" s="2"/>
-      <c r="N98" s="2"/>
-      <c r="O98" s="2"/>
-      <c r="P98" s="2"/>
-      <c r="Q98" s="2"/>
-      <c r="R98" s="3"/>
-    </row>
-    <row r="99" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J99" s="2"/>
-      <c r="K99" s="3"/>
-      <c r="L99" s="2"/>
-      <c r="M99" s="2"/>
-      <c r="N99" s="2"/>
-      <c r="O99" s="2"/>
-      <c r="P99" s="2"/>
-      <c r="Q99" s="2"/>
-      <c r="R99" s="3"/>
-    </row>
-    <row r="100" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J100" s="2"/>
-      <c r="K100" s="3"/>
-      <c r="L100" s="2"/>
-      <c r="M100" s="2"/>
-      <c r="N100" s="2"/>
-      <c r="O100" s="2"/>
-      <c r="P100" s="2"/>
-      <c r="Q100" s="2"/>
-      <c r="R100" s="3"/>
-    </row>
-    <row r="101" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J101" s="2"/>
-      <c r="K101" s="3"/>
-      <c r="L101" s="2"/>
-      <c r="M101" s="2"/>
-      <c r="N101" s="2"/>
-      <c r="O101" s="2"/>
-      <c r="P101" s="2"/>
-      <c r="Q101" s="2"/>
-      <c r="R101" s="3"/>
-    </row>
-    <row r="102" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J102" s="2"/>
-      <c r="K102" s="3"/>
-      <c r="L102" s="2"/>
-      <c r="M102" s="2"/>
-      <c r="N102" s="2"/>
-      <c r="O102" s="2"/>
-      <c r="P102" s="2"/>
-      <c r="Q102" s="2"/>
-      <c r="R102" s="3"/>
-    </row>
-    <row r="103" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J103" s="2"/>
-      <c r="K103" s="3"/>
-      <c r="L103" s="2"/>
-      <c r="M103" s="2"/>
-      <c r="N103" s="2"/>
-      <c r="O103" s="2"/>
-      <c r="P103" s="2"/>
-      <c r="Q103" s="2"/>
-      <c r="R103" s="3"/>
-    </row>
-    <row r="104" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J104" s="2"/>
-      <c r="K104" s="3"/>
-      <c r="L104" s="2"/>
-      <c r="M104" s="2"/>
-      <c r="N104" s="2"/>
-      <c r="O104" s="2"/>
-      <c r="P104" s="2"/>
-      <c r="Q104" s="2"/>
-      <c r="R104" s="3"/>
-    </row>
-    <row r="105" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J105" s="2"/>
-      <c r="K105" s="3"/>
-      <c r="L105" s="2"/>
-      <c r="M105" s="2"/>
-      <c r="N105" s="2"/>
-      <c r="O105" s="2"/>
-      <c r="P105" s="2"/>
-      <c r="Q105" s="2"/>
-      <c r="R105" s="3"/>
-    </row>
-    <row r="106" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J106" s="2"/>
-      <c r="K106" s="3"/>
-      <c r="L106" s="2"/>
-      <c r="M106" s="2"/>
-      <c r="N106" s="2"/>
-      <c r="O106" s="2"/>
-      <c r="P106" s="2"/>
-      <c r="Q106" s="2"/>
-      <c r="R106" s="3"/>
-    </row>
-    <row r="107" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J107" s="2"/>
-      <c r="K107" s="3"/>
-      <c r="L107" s="2"/>
-      <c r="M107" s="2"/>
-      <c r="N107" s="2"/>
-      <c r="O107" s="2"/>
-      <c r="P107" s="2"/>
-      <c r="Q107" s="2"/>
-      <c r="R107" s="3"/>
-    </row>
-    <row r="108" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J108" s="2"/>
-      <c r="K108" s="3"/>
-      <c r="L108" s="2"/>
-      <c r="M108" s="2"/>
-      <c r="N108" s="2"/>
-      <c r="O108" s="2"/>
-      <c r="P108" s="2"/>
-      <c r="Q108" s="2"/>
-      <c r="R108" s="3"/>
-    </row>
-    <row r="109" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J109" s="2"/>
-      <c r="K109" s="3"/>
-      <c r="L109" s="2"/>
-      <c r="M109" s="2"/>
-      <c r="N109" s="2"/>
-      <c r="O109" s="2"/>
-      <c r="P109" s="2"/>
-      <c r="Q109" s="2"/>
-      <c r="R109" s="3"/>
-    </row>
-    <row r="110" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J110" s="2"/>
-      <c r="K110" s="3"/>
-      <c r="L110" s="2"/>
-      <c r="M110" s="2"/>
-      <c r="N110" s="2"/>
-      <c r="O110" s="2"/>
-      <c r="P110" s="2"/>
-      <c r="Q110" s="2"/>
-      <c r="R110" s="3"/>
-    </row>
-    <row r="111" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J111" s="2"/>
-      <c r="K111" s="3"/>
-      <c r="L111" s="2"/>
-      <c r="M111" s="2"/>
-      <c r="N111" s="2"/>
-      <c r="O111" s="2"/>
-      <c r="P111" s="2"/>
-      <c r="Q111" s="2"/>
-      <c r="R111" s="3"/>
-    </row>
-    <row r="112" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J112" s="2"/>
-      <c r="K112" s="3"/>
-      <c r="L112" s="2"/>
-      <c r="M112" s="2"/>
-      <c r="N112" s="2"/>
-      <c r="O112" s="2"/>
-      <c r="P112" s="2"/>
-      <c r="Q112" s="2"/>
-      <c r="R112" s="3"/>
-    </row>
-    <row r="113" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J113" s="2"/>
-      <c r="K113" s="3"/>
-      <c r="L113" s="2"/>
-      <c r="M113" s="2"/>
-      <c r="N113" s="2"/>
-      <c r="O113" s="2"/>
-      <c r="P113" s="2"/>
-      <c r="Q113" s="2"/>
-      <c r="R113" s="3"/>
-    </row>
-    <row r="114" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J114" s="2"/>
-      <c r="K114" s="3"/>
-      <c r="L114" s="2"/>
-      <c r="M114" s="2"/>
-      <c r="N114" s="2"/>
-      <c r="O114" s="2"/>
-      <c r="P114" s="2"/>
-      <c r="Q114" s="2"/>
-      <c r="R114" s="3"/>
-    </row>
-    <row r="115" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J115" s="2"/>
-      <c r="K115" s="3"/>
-      <c r="L115" s="2"/>
-      <c r="M115" s="2"/>
-      <c r="N115" s="2"/>
-      <c r="O115" s="2"/>
-      <c r="P115" s="2"/>
-      <c r="Q115" s="2"/>
-      <c r="R115" s="3"/>
-    </row>
-    <row r="116" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J116" s="2"/>
-      <c r="K116" s="3"/>
-      <c r="L116" s="2"/>
-      <c r="M116" s="2"/>
-      <c r="N116" s="2"/>
-      <c r="O116" s="2"/>
-      <c r="P116" s="2"/>
-      <c r="Q116" s="2"/>
-      <c r="R116" s="3"/>
-    </row>
-    <row r="117" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J117" s="2"/>
-      <c r="K117" s="3"/>
-      <c r="L117" s="2"/>
-      <c r="M117" s="2"/>
-      <c r="N117" s="2"/>
-      <c r="O117" s="2"/>
-      <c r="P117" s="2"/>
-      <c r="Q117" s="2"/>
-      <c r="R117" s="3"/>
-    </row>
-    <row r="118" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J118" s="2"/>
-      <c r="K118" s="3"/>
-      <c r="L118" s="2"/>
-      <c r="M118" s="2"/>
-      <c r="N118" s="2"/>
-      <c r="O118" s="2"/>
-      <c r="P118" s="2"/>
-      <c r="Q118" s="2"/>
-      <c r="R118" s="3"/>
-    </row>
-    <row r="119" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J119" s="2"/>
-      <c r="K119" s="3"/>
-      <c r="L119" s="2"/>
-      <c r="M119" s="2"/>
-      <c r="N119" s="2"/>
-      <c r="O119" s="2"/>
-      <c r="P119" s="2"/>
-      <c r="Q119" s="2"/>
-      <c r="R119" s="3"/>
-    </row>
-    <row r="120" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J120" s="2"/>
-      <c r="K120" s="3"/>
-      <c r="L120" s="2"/>
-      <c r="M120" s="2"/>
-      <c r="N120" s="2"/>
-      <c r="O120" s="2"/>
-      <c r="P120" s="2"/>
-      <c r="Q120" s="2"/>
-      <c r="R120" s="3"/>
-    </row>
-    <row r="121" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J121" s="2"/>
-      <c r="K121" s="3"/>
-      <c r="L121" s="2"/>
-      <c r="M121" s="2"/>
-      <c r="N121" s="2"/>
-      <c r="O121" s="2"/>
-      <c r="P121" s="2"/>
-      <c r="Q121" s="2"/>
-      <c r="R121" s="3"/>
-    </row>
-    <row r="122" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J122" s="2"/>
-      <c r="K122" s="3"/>
-      <c r="L122" s="2"/>
-      <c r="M122" s="2"/>
-      <c r="N122" s="2"/>
-      <c r="O122" s="2"/>
-      <c r="P122" s="2"/>
-      <c r="Q122" s="2"/>
-      <c r="R122" s="3"/>
-    </row>
-    <row r="123" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J123" s="2"/>
-      <c r="K123" s="3"/>
-      <c r="L123" s="2"/>
-      <c r="M123" s="2"/>
-      <c r="N123" s="2"/>
-      <c r="O123" s="2"/>
-      <c r="P123" s="2"/>
-      <c r="Q123" s="2"/>
-      <c r="R123" s="3"/>
-    </row>
-    <row r="124" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J124" s="2"/>
-      <c r="K124" s="3"/>
-      <c r="L124" s="2"/>
-      <c r="M124" s="2"/>
-      <c r="N124" s="2"/>
-      <c r="O124" s="2"/>
-      <c r="P124" s="2"/>
-      <c r="Q124" s="2"/>
-      <c r="R124" s="3"/>
-    </row>
-    <row r="125" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J125" s="2"/>
-      <c r="K125" s="3"/>
-      <c r="L125" s="2"/>
-      <c r="M125" s="2"/>
-      <c r="N125" s="2"/>
-      <c r="O125" s="2"/>
-      <c r="P125" s="2"/>
-      <c r="Q125" s="2"/>
-      <c r="R125" s="3"/>
-    </row>
-    <row r="126" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J126" s="2"/>
-      <c r="K126" s="3"/>
-      <c r="L126" s="2"/>
-      <c r="M126" s="2"/>
-      <c r="N126" s="2"/>
-      <c r="O126" s="2"/>
-      <c r="P126" s="2"/>
-      <c r="Q126" s="2"/>
-      <c r="R126" s="3"/>
-    </row>
-    <row r="127" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J127" s="2"/>
-      <c r="K127" s="3"/>
-      <c r="L127" s="2"/>
-      <c r="M127" s="2"/>
-      <c r="N127" s="2"/>
-      <c r="O127" s="2"/>
-      <c r="P127" s="2"/>
-      <c r="Q127" s="2"/>
-      <c r="R127" s="3"/>
-    </row>
-    <row r="128" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J128" s="2"/>
-      <c r="K128" s="3"/>
-      <c r="L128" s="2"/>
-      <c r="M128" s="2"/>
-      <c r="N128" s="2"/>
-      <c r="O128" s="2"/>
-      <c r="P128" s="2"/>
-      <c r="Q128" s="2"/>
-      <c r="R128" s="3"/>
-    </row>
-    <row r="129" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J129" s="2"/>
-      <c r="K129" s="3"/>
-      <c r="L129" s="2"/>
-      <c r="M129" s="2"/>
-      <c r="N129" s="2"/>
-      <c r="O129" s="2"/>
-      <c r="P129" s="2"/>
-      <c r="Q129" s="2"/>
-      <c r="R129" s="3"/>
-    </row>
-    <row r="130" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J130" s="2"/>
-      <c r="K130" s="3"/>
-      <c r="L130" s="2"/>
-      <c r="M130" s="2"/>
-      <c r="N130" s="2"/>
-      <c r="O130" s="2"/>
-      <c r="P130" s="2"/>
-      <c r="Q130" s="2"/>
-      <c r="R130" s="3"/>
-    </row>
-    <row r="131" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J131" s="2"/>
-      <c r="K131" s="3"/>
-      <c r="L131" s="2"/>
-      <c r="M131" s="2"/>
-      <c r="N131" s="2"/>
-      <c r="O131" s="2"/>
-      <c r="P131" s="2"/>
-      <c r="Q131" s="2"/>
-      <c r="R131" s="3"/>
-    </row>
-    <row r="132" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J132" s="2"/>
-      <c r="K132" s="3"/>
-      <c r="L132" s="2"/>
-      <c r="M132" s="2"/>
-      <c r="N132" s="2"/>
-      <c r="O132" s="2"/>
-      <c r="P132" s="2"/>
-      <c r="Q132" s="2"/>
-      <c r="R132" s="3"/>
-    </row>
-    <row r="133" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J133" s="2"/>
-      <c r="K133" s="3"/>
-      <c r="L133" s="2"/>
-      <c r="M133" s="2"/>
-      <c r="N133" s="2"/>
-      <c r="O133" s="2"/>
-      <c r="P133" s="2"/>
-      <c r="Q133" s="2"/>
-      <c r="R133" s="3"/>
-    </row>
-    <row r="134" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J134" s="2"/>
-      <c r="K134" s="3"/>
-      <c r="L134" s="2"/>
-      <c r="M134" s="2"/>
-      <c r="N134" s="2"/>
-      <c r="O134" s="2"/>
-      <c r="P134" s="2"/>
-      <c r="Q134" s="2"/>
-      <c r="R134" s="3"/>
-    </row>
-    <row r="135" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J135" s="2"/>
-      <c r="K135" s="3"/>
-      <c r="L135" s="2"/>
-      <c r="M135" s="2"/>
-      <c r="N135" s="2"/>
-      <c r="O135" s="2"/>
-      <c r="P135" s="2"/>
-      <c r="Q135" s="2"/>
-      <c r="R135" s="3"/>
-    </row>
-    <row r="136" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J136" s="2"/>
-      <c r="K136" s="3"/>
-      <c r="L136" s="2"/>
-      <c r="M136" s="2"/>
-      <c r="N136" s="2"/>
-      <c r="O136" s="2"/>
-      <c r="P136" s="2"/>
-      <c r="Q136" s="2"/>
-      <c r="R136" s="3"/>
-    </row>
-    <row r="137" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J137" s="2"/>
-      <c r="K137" s="3"/>
-      <c r="L137" s="2"/>
-      <c r="M137" s="2"/>
-      <c r="N137" s="2"/>
-      <c r="O137" s="2"/>
-      <c r="P137" s="2"/>
-      <c r="Q137" s="2"/>
-      <c r="R137" s="3"/>
-    </row>
-    <row r="138" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J138" s="2"/>
-      <c r="K138" s="3"/>
-      <c r="L138" s="2"/>
-      <c r="M138" s="2"/>
-      <c r="N138" s="2"/>
-      <c r="O138" s="2"/>
-      <c r="P138" s="2"/>
-      <c r="Q138" s="2"/>
-      <c r="R138" s="3"/>
-    </row>
-    <row r="139" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J139" s="2"/>
-      <c r="K139" s="3"/>
-      <c r="L139" s="2"/>
-      <c r="M139" s="2"/>
-      <c r="N139" s="2"/>
-      <c r="O139" s="2"/>
-      <c r="P139" s="2"/>
-      <c r="Q139" s="2"/>
-      <c r="R139" s="3"/>
-    </row>
-    <row r="140" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J140" s="2"/>
-      <c r="K140" s="3"/>
-      <c r="L140" s="2"/>
-      <c r="M140" s="2"/>
-      <c r="N140" s="2"/>
-      <c r="O140" s="2"/>
-      <c r="P140" s="2"/>
-      <c r="Q140" s="2"/>
-      <c r="R140" s="3"/>
-    </row>
-    <row r="141" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J141" s="2"/>
-      <c r="K141" s="3"/>
-      <c r="L141" s="2"/>
-      <c r="M141" s="2"/>
-      <c r="N141" s="2"/>
-      <c r="O141" s="2"/>
-      <c r="P141" s="2"/>
-      <c r="Q141" s="2"/>
-      <c r="R141" s="3"/>
-    </row>
-    <row r="142" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J142" s="2"/>
-      <c r="K142" s="3"/>
-      <c r="L142" s="2"/>
-      <c r="M142" s="2"/>
-      <c r="N142" s="2"/>
-      <c r="O142" s="2"/>
-      <c r="P142" s="2"/>
-      <c r="Q142" s="2"/>
-      <c r="R142" s="3"/>
-    </row>
-    <row r="143" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J143" s="2"/>
-      <c r="K143" s="3"/>
-      <c r="L143" s="2"/>
-      <c r="M143" s="2"/>
-      <c r="N143" s="2"/>
-      <c r="O143" s="2"/>
-      <c r="P143" s="2"/>
-      <c r="Q143" s="2"/>
-      <c r="R143" s="3"/>
-    </row>
-    <row r="144" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J144" s="2"/>
-      <c r="K144" s="3"/>
-      <c r="L144" s="2"/>
-      <c r="M144" s="2"/>
-      <c r="N144" s="2"/>
-      <c r="O144" s="2"/>
-      <c r="P144" s="2"/>
-      <c r="Q144" s="2"/>
-      <c r="R144" s="3"/>
-    </row>
-    <row r="145" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J145" s="2"/>
-      <c r="K145" s="3"/>
-      <c r="L145" s="2"/>
-      <c r="M145" s="2"/>
-      <c r="N145" s="2"/>
-      <c r="O145" s="2"/>
-      <c r="P145" s="2"/>
-      <c r="Q145" s="2"/>
-      <c r="R145" s="3"/>
-    </row>
-    <row r="146" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J146" s="2"/>
-      <c r="K146" s="3"/>
-      <c r="L146" s="2"/>
-      <c r="M146" s="2"/>
-      <c r="N146" s="2"/>
-      <c r="O146" s="2"/>
-      <c r="P146" s="2"/>
-      <c r="Q146" s="2"/>
-      <c r="R146" s="3"/>
-    </row>
-    <row r="147" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J147" s="2"/>
-      <c r="K147" s="3"/>
-      <c r="L147" s="2"/>
-      <c r="M147" s="2"/>
-      <c r="N147" s="2"/>
-      <c r="O147" s="2"/>
-      <c r="P147" s="2"/>
-      <c r="Q147" s="2"/>
-      <c r="R147" s="3"/>
-    </row>
-    <row r="148" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J148" s="2"/>
-      <c r="K148" s="3"/>
-      <c r="L148" s="2"/>
-      <c r="M148" s="2"/>
-      <c r="N148" s="2"/>
-      <c r="O148" s="2"/>
-      <c r="P148" s="2"/>
-      <c r="Q148" s="2"/>
-      <c r="R148" s="3"/>
-    </row>
-    <row r="149" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J149" s="2"/>
-      <c r="K149" s="3"/>
-      <c r="L149" s="2"/>
-      <c r="M149" s="2"/>
-      <c r="N149" s="2"/>
-      <c r="O149" s="2"/>
-      <c r="P149" s="2"/>
-      <c r="Q149" s="2"/>
-      <c r="R149" s="3"/>
-    </row>
-    <row r="150" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J150" s="2"/>
-      <c r="K150" s="3"/>
-      <c r="L150" s="2"/>
-      <c r="M150" s="2"/>
-      <c r="N150" s="2"/>
-      <c r="O150" s="2"/>
-      <c r="P150" s="2"/>
-      <c r="Q150" s="2"/>
-      <c r="R150" s="3"/>
-    </row>
-    <row r="151" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J151" s="2"/>
-      <c r="K151" s="3"/>
-      <c r="L151" s="2"/>
-      <c r="M151" s="2"/>
-      <c r="N151" s="2"/>
-      <c r="O151" s="2"/>
-      <c r="P151" s="2"/>
-      <c r="Q151" s="2"/>
-      <c r="R151" s="3"/>
-    </row>
-    <row r="152" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J152" s="2"/>
-      <c r="K152" s="3"/>
-      <c r="L152" s="2"/>
-      <c r="M152" s="2"/>
-      <c r="N152" s="2"/>
-      <c r="O152" s="2"/>
-      <c r="P152" s="2"/>
-      <c r="Q152" s="2"/>
-      <c r="R152" s="3"/>
-    </row>
-    <row r="153" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J153" s="2"/>
-      <c r="K153" s="3"/>
-      <c r="L153" s="2"/>
-      <c r="M153" s="2"/>
-      <c r="N153" s="2"/>
-      <c r="O153" s="2"/>
-      <c r="P153" s="2"/>
-      <c r="Q153" s="2"/>
-      <c r="R153" s="3"/>
-    </row>
-    <row r="154" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J154" s="2"/>
-      <c r="K154" s="3"/>
-      <c r="L154" s="2"/>
-      <c r="M154" s="2"/>
-      <c r="N154" s="2"/>
-      <c r="O154" s="2"/>
-      <c r="P154" s="2"/>
-      <c r="Q154" s="2"/>
-      <c r="R154" s="3"/>
-    </row>
-    <row r="155" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J155" s="2"/>
-      <c r="K155" s="3"/>
-      <c r="L155" s="2"/>
-      <c r="M155" s="2"/>
-      <c r="N155" s="2"/>
-      <c r="O155" s="2"/>
-      <c r="P155" s="2"/>
-      <c r="Q155" s="2"/>
-      <c r="R155" s="3"/>
-    </row>
-    <row r="156" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J156" s="2"/>
-      <c r="K156" s="3"/>
-      <c r="L156" s="2"/>
-      <c r="M156" s="2"/>
-      <c r="N156" s="2"/>
-      <c r="O156" s="2"/>
-      <c r="P156" s="2"/>
-      <c r="Q156" s="2"/>
-      <c r="R156" s="3"/>
-    </row>
-    <row r="157" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J157" s="2"/>
-      <c r="K157" s="3"/>
-      <c r="L157" s="2"/>
-      <c r="M157" s="2"/>
-      <c r="N157" s="2"/>
-      <c r="O157" s="2"/>
-      <c r="P157" s="2"/>
-      <c r="Q157" s="2"/>
-      <c r="R157" s="3"/>
-    </row>
-    <row r="158" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J158" s="2"/>
-      <c r="K158" s="3"/>
-      <c r="L158" s="2"/>
-      <c r="M158" s="2"/>
-      <c r="N158" s="2"/>
-      <c r="O158" s="2"/>
-      <c r="P158" s="2"/>
-      <c r="Q158" s="2"/>
-      <c r="R158" s="3"/>
-    </row>
-    <row r="159" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J159" s="2"/>
-      <c r="K159" s="3"/>
-      <c r="L159" s="2"/>
-      <c r="M159" s="2"/>
-      <c r="N159" s="2"/>
-      <c r="O159" s="2"/>
-      <c r="P159" s="2"/>
-      <c r="Q159" s="2"/>
-      <c r="R159" s="3"/>
-    </row>
-    <row r="160" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J160" s="2"/>
-      <c r="K160" s="3"/>
-      <c r="L160" s="2"/>
-      <c r="M160" s="2"/>
-      <c r="N160" s="2"/>
-      <c r="O160" s="2"/>
-      <c r="P160" s="2"/>
-      <c r="Q160" s="2"/>
-      <c r="R160" s="3"/>
-    </row>
-    <row r="161" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J161" s="2"/>
-      <c r="K161" s="3"/>
-      <c r="L161" s="2"/>
-      <c r="M161" s="2"/>
-      <c r="N161" s="2"/>
-      <c r="O161" s="2"/>
-      <c r="P161" s="2"/>
-      <c r="Q161" s="2"/>
-      <c r="R161" s="3"/>
-    </row>
-    <row r="162" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J162" s="2"/>
-      <c r="K162" s="3"/>
-      <c r="L162" s="2"/>
-      <c r="M162" s="2"/>
-      <c r="N162" s="2"/>
-      <c r="O162" s="2"/>
-      <c r="P162" s="2"/>
-      <c r="Q162" s="2"/>
-      <c r="R162" s="3"/>
-    </row>
-    <row r="163" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J163" s="2"/>
-      <c r="K163" s="3"/>
-      <c r="L163" s="2"/>
-      <c r="M163" s="2"/>
-      <c r="N163" s="2"/>
-      <c r="O163" s="2"/>
-      <c r="P163" s="2"/>
-      <c r="Q163" s="2"/>
-      <c r="R163" s="3"/>
-    </row>
-    <row r="164" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J164" s="2"/>
-      <c r="K164" s="3"/>
-      <c r="L164" s="2"/>
-      <c r="M164" s="2"/>
-      <c r="N164" s="2"/>
-      <c r="O164" s="2"/>
-      <c r="P164" s="2"/>
-      <c r="Q164" s="2"/>
-      <c r="R164" s="3"/>
-    </row>
-    <row r="165" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J165" s="2"/>
-      <c r="K165" s="3"/>
-      <c r="L165" s="2"/>
-      <c r="M165" s="2"/>
-      <c r="N165" s="2"/>
-      <c r="O165" s="2"/>
-      <c r="P165" s="2"/>
-      <c r="Q165" s="2"/>
-      <c r="R165" s="3"/>
-    </row>
-    <row r="166" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J166" s="2"/>
-      <c r="K166" s="3"/>
-      <c r="L166" s="2"/>
-      <c r="M166" s="2"/>
-      <c r="N166" s="2"/>
-      <c r="O166" s="2"/>
-      <c r="P166" s="2"/>
-      <c r="Q166" s="2"/>
-      <c r="R166" s="3"/>
-    </row>
-    <row r="167" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J167" s="2"/>
-      <c r="K167" s="3"/>
-      <c r="L167" s="2"/>
-      <c r="M167" s="2"/>
-      <c r="N167" s="2"/>
-      <c r="O167" s="2"/>
-      <c r="P167" s="2"/>
-      <c r="Q167" s="2"/>
-      <c r="R167" s="3"/>
-    </row>
-    <row r="168" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J168" s="2"/>
-      <c r="K168" s="3"/>
-      <c r="L168" s="2"/>
-      <c r="M168" s="2"/>
-      <c r="N168" s="2"/>
-      <c r="O168" s="2"/>
-      <c r="P168" s="2"/>
-      <c r="Q168" s="2"/>
-      <c r="R168" s="3"/>
-    </row>
-    <row r="169" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J169" s="2"/>
-      <c r="K169" s="3"/>
-      <c r="L169" s="2"/>
-      <c r="M169" s="2"/>
-      <c r="N169" s="2"/>
-      <c r="O169" s="2"/>
-      <c r="P169" s="2"/>
-      <c r="Q169" s="2"/>
-      <c r="R169" s="3"/>
-    </row>
-    <row r="170" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J170" s="2"/>
-      <c r="K170" s="3"/>
-      <c r="L170" s="2"/>
-      <c r="M170" s="2"/>
-      <c r="N170" s="2"/>
-      <c r="O170" s="2"/>
-      <c r="P170" s="2"/>
-      <c r="Q170" s="2"/>
-      <c r="R170" s="3"/>
-    </row>
-    <row r="171" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J171" s="2"/>
-      <c r="K171" s="3"/>
-      <c r="L171" s="2"/>
-      <c r="M171" s="2"/>
-      <c r="N171" s="2"/>
-      <c r="O171" s="2"/>
-      <c r="P171" s="2"/>
-      <c r="Q171" s="2"/>
-      <c r="R171" s="3"/>
-    </row>
-    <row r="172" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J172" s="2"/>
-      <c r="K172" s="3"/>
-      <c r="L172" s="2"/>
-      <c r="M172" s="2"/>
-      <c r="N172" s="2"/>
-      <c r="O172" s="2"/>
-      <c r="P172" s="2"/>
-      <c r="Q172" s="2"/>
-      <c r="R172" s="3"/>
-    </row>
-    <row r="173" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J173" s="2"/>
-      <c r="K173" s="3"/>
-      <c r="L173" s="2"/>
-      <c r="M173" s="2"/>
-      <c r="N173" s="2"/>
-      <c r="O173" s="2"/>
-      <c r="P173" s="2"/>
-      <c r="Q173" s="2"/>
-      <c r="R173" s="3"/>
-    </row>
-    <row r="174" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J174" s="2"/>
-      <c r="K174" s="3"/>
-      <c r="L174" s="2"/>
-      <c r="M174" s="2"/>
-      <c r="N174" s="2"/>
-      <c r="O174" s="2"/>
-      <c r="P174" s="2"/>
-      <c r="Q174" s="2"/>
-      <c r="R174" s="3"/>
-    </row>
-    <row r="175" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J175" s="2"/>
-      <c r="K175" s="3"/>
-      <c r="L175" s="2"/>
-      <c r="M175" s="2"/>
-      <c r="N175" s="2"/>
-      <c r="O175" s="2"/>
-      <c r="P175" s="2"/>
-      <c r="Q175" s="2"/>
-      <c r="R175" s="3"/>
-    </row>
-    <row r="176" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J176" s="2"/>
-      <c r="K176" s="3"/>
-      <c r="L176" s="2"/>
-      <c r="M176" s="2"/>
-      <c r="N176" s="2"/>
-      <c r="O176" s="2"/>
-      <c r="P176" s="2"/>
-      <c r="Q176" s="2"/>
-      <c r="R176" s="3"/>
-    </row>
-    <row r="177" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J177" s="2"/>
-      <c r="K177" s="3"/>
-      <c r="L177" s="2"/>
-      <c r="M177" s="2"/>
-      <c r="N177" s="2"/>
-      <c r="O177" s="2"/>
-      <c r="P177" s="2"/>
-      <c r="Q177" s="2"/>
-      <c r="R177" s="3"/>
-    </row>
-    <row r="178" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J178" s="2"/>
-      <c r="K178" s="3"/>
-      <c r="L178" s="2"/>
-      <c r="M178" s="2"/>
-      <c r="N178" s="2"/>
-      <c r="O178" s="2"/>
-      <c r="P178" s="2"/>
-      <c r="Q178" s="2"/>
-      <c r="R178" s="3"/>
-    </row>
-    <row r="179" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J179" s="2"/>
-      <c r="K179" s="3"/>
-      <c r="L179" s="2"/>
-      <c r="M179" s="2"/>
-      <c r="N179" s="2"/>
-      <c r="O179" s="2"/>
-      <c r="P179" s="2"/>
-      <c r="Q179" s="2"/>
-      <c r="R179" s="3"/>
-    </row>
-    <row r="180" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J180" s="2"/>
-      <c r="K180" s="3"/>
-      <c r="L180" s="2"/>
-      <c r="M180" s="2"/>
-      <c r="N180" s="2"/>
-      <c r="O180" s="2"/>
-      <c r="P180" s="2"/>
-      <c r="Q180" s="2"/>
-      <c r="R180" s="3"/>
-    </row>
-    <row r="181" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J181" s="2"/>
-      <c r="K181" s="3"/>
-      <c r="L181" s="2"/>
-      <c r="M181" s="2"/>
-      <c r="N181" s="2"/>
-      <c r="O181" s="2"/>
-      <c r="P181" s="2"/>
-      <c r="Q181" s="2"/>
-      <c r="R181" s="3"/>
-    </row>
-    <row r="182" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J182" s="2"/>
-      <c r="K182" s="3"/>
-      <c r="L182" s="2"/>
-      <c r="M182" s="2"/>
-      <c r="N182" s="2"/>
-      <c r="O182" s="2"/>
-      <c r="P182" s="2"/>
-      <c r="Q182" s="2"/>
-      <c r="R182" s="3"/>
-    </row>
-    <row r="183" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J183" s="2"/>
-      <c r="K183" s="3"/>
-      <c r="L183" s="2"/>
-      <c r="M183" s="2"/>
-      <c r="N183" s="2"/>
-      <c r="O183" s="2"/>
-      <c r="P183" s="2"/>
-      <c r="Q183" s="2"/>
-      <c r="R183" s="3"/>
-    </row>
-    <row r="184" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J184" s="2"/>
-      <c r="K184" s="3"/>
-      <c r="L184" s="2"/>
-      <c r="M184" s="2"/>
-      <c r="N184" s="2"/>
-      <c r="O184" s="2"/>
-      <c r="P184" s="2"/>
-      <c r="Q184" s="2"/>
-      <c r="R184" s="3"/>
-    </row>
-    <row r="185" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J185" s="2"/>
-      <c r="K185" s="3"/>
-      <c r="L185" s="2"/>
-      <c r="M185" s="2"/>
-      <c r="N185" s="2"/>
-      <c r="O185" s="2"/>
-      <c r="P185" s="2"/>
-      <c r="Q185" s="2"/>
-      <c r="R185" s="3"/>
-    </row>
-    <row r="186" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J186" s="2"/>
-      <c r="K186" s="3"/>
-      <c r="L186" s="2"/>
-      <c r="M186" s="2"/>
-      <c r="N186" s="2"/>
-      <c r="O186" s="2"/>
-      <c r="P186" s="2"/>
-      <c r="Q186" s="2"/>
-      <c r="R186" s="3"/>
-    </row>
-    <row r="187" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J187" s="2"/>
-      <c r="K187" s="3"/>
-      <c r="L187" s="2"/>
-      <c r="M187" s="2"/>
-      <c r="N187" s="2"/>
-      <c r="O187" s="2"/>
-      <c r="P187" s="2"/>
-      <c r="Q187" s="2"/>
-      <c r="R187" s="3"/>
-    </row>
-    <row r="188" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J188" s="2"/>
-      <c r="K188" s="3"/>
-      <c r="L188" s="2"/>
-      <c r="M188" s="2"/>
-      <c r="N188" s="2"/>
-      <c r="O188" s="2"/>
-      <c r="P188" s="2"/>
-      <c r="Q188" s="2"/>
-      <c r="R188" s="3"/>
-    </row>
-    <row r="189" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J189" s="2"/>
-      <c r="K189" s="3"/>
-      <c r="L189" s="2"/>
-      <c r="M189" s="2"/>
-      <c r="N189" s="2"/>
-      <c r="O189" s="2"/>
-      <c r="P189" s="2"/>
-      <c r="Q189" s="2"/>
-      <c r="R189" s="3"/>
-    </row>
-    <row r="190" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J190" s="2"/>
-      <c r="K190" s="3"/>
-      <c r="L190" s="2"/>
-      <c r="M190" s="2"/>
-      <c r="N190" s="2"/>
-      <c r="O190" s="2"/>
-      <c r="P190" s="2"/>
-      <c r="Q190" s="2"/>
-      <c r="R190" s="3"/>
-    </row>
-    <row r="191" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J191" s="2"/>
-      <c r="K191" s="3"/>
-      <c r="L191" s="2"/>
-      <c r="M191" s="2"/>
-      <c r="N191" s="2"/>
-      <c r="O191" s="2"/>
-      <c r="P191" s="2"/>
-      <c r="Q191" s="2"/>
-      <c r="R191" s="3"/>
-    </row>
-    <row r="192" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J192" s="2"/>
-      <c r="K192" s="3"/>
-      <c r="L192" s="2"/>
-      <c r="M192" s="2"/>
-      <c r="N192" s="2"/>
-      <c r="O192" s="2"/>
-      <c r="P192" s="2"/>
-      <c r="Q192" s="2"/>
-      <c r="R192" s="3"/>
-    </row>
-    <row r="193" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J193" s="2"/>
-      <c r="K193" s="3"/>
-      <c r="L193" s="2"/>
-      <c r="M193" s="2"/>
-      <c r="N193" s="2"/>
-      <c r="O193" s="2"/>
-      <c r="P193" s="2"/>
-      <c r="Q193" s="2"/>
-      <c r="R193" s="3"/>
-    </row>
-    <row r="194" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J194" s="2"/>
-      <c r="K194" s="3"/>
-      <c r="L194" s="2"/>
-      <c r="M194" s="2"/>
-      <c r="N194" s="2"/>
-      <c r="O194" s="2"/>
-      <c r="P194" s="2"/>
-      <c r="Q194" s="2"/>
-      <c r="R194" s="3"/>
-    </row>
-    <row r="195" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J195" s="2"/>
-      <c r="K195" s="3"/>
-      <c r="L195" s="2"/>
-      <c r="M195" s="2"/>
-      <c r="N195" s="2"/>
-      <c r="O195" s="2"/>
-      <c r="P195" s="2"/>
-      <c r="Q195" s="2"/>
-      <c r="R195" s="3"/>
-    </row>
-    <row r="196" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J196" s="2"/>
-      <c r="K196" s="3"/>
-      <c r="L196" s="2"/>
-      <c r="M196" s="2"/>
-      <c r="N196" s="2"/>
-      <c r="O196" s="2"/>
-      <c r="P196" s="2"/>
-      <c r="Q196" s="2"/>
-      <c r="R196" s="3"/>
-    </row>
-    <row r="197" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J197" s="2"/>
-      <c r="K197" s="3"/>
-      <c r="L197" s="2"/>
-      <c r="M197" s="2"/>
-      <c r="N197" s="2"/>
-      <c r="O197" s="2"/>
-      <c r="P197" s="2"/>
-      <c r="Q197" s="2"/>
-      <c r="R197" s="3"/>
-    </row>
-    <row r="198" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J198" s="2"/>
-      <c r="K198" s="3"/>
-      <c r="L198" s="2"/>
-      <c r="M198" s="2"/>
-      <c r="N198" s="2"/>
-      <c r="O198" s="2"/>
-      <c r="P198" s="2"/>
-      <c r="Q198" s="2"/>
-      <c r="R198" s="3"/>
-    </row>
-    <row r="199" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J199" s="2"/>
-      <c r="K199" s="3"/>
-      <c r="L199" s="2"/>
-      <c r="M199" s="2"/>
-      <c r="N199" s="2"/>
-      <c r="O199" s="2"/>
-      <c r="P199" s="2"/>
-      <c r="Q199" s="2"/>
-      <c r="R199" s="3"/>
-    </row>
-    <row r="200" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J200" s="2"/>
-      <c r="K200" s="3"/>
-      <c r="L200" s="2"/>
-      <c r="M200" s="2"/>
-      <c r="N200" s="2"/>
-      <c r="O200" s="2"/>
-      <c r="P200" s="2"/>
-      <c r="Q200" s="2"/>
-      <c r="R200" s="3"/>
-    </row>
-    <row r="201" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J201" s="2"/>
-      <c r="K201" s="3"/>
-      <c r="L201" s="2"/>
-      <c r="M201" s="2"/>
-      <c r="N201" s="2"/>
-      <c r="O201" s="2"/>
-      <c r="P201" s="2"/>
-      <c r="Q201" s="2"/>
-      <c r="R201" s="3"/>
-    </row>
-    <row r="202" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J202" s="2"/>
-      <c r="K202" s="3"/>
-      <c r="L202" s="2"/>
-      <c r="M202" s="2"/>
-      <c r="N202" s="2"/>
-      <c r="O202" s="2"/>
-      <c r="P202" s="2"/>
-      <c r="Q202" s="2"/>
-      <c r="R202" s="3"/>
-    </row>
-    <row r="203" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J203" s="2"/>
-      <c r="K203" s="3"/>
-      <c r="L203" s="2"/>
-      <c r="M203" s="2"/>
-      <c r="N203" s="2"/>
-      <c r="O203" s="2"/>
-      <c r="P203" s="2"/>
-      <c r="Q203" s="2"/>
-      <c r="R203" s="3"/>
-    </row>
-    <row r="204" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J204" s="2"/>
-      <c r="K204" s="3"/>
-      <c r="L204" s="2"/>
-      <c r="M204" s="2"/>
-      <c r="N204" s="2"/>
-      <c r="O204" s="2"/>
-      <c r="P204" s="2"/>
-      <c r="Q204" s="2"/>
-      <c r="R204" s="3"/>
-    </row>
-    <row r="205" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J205" s="2"/>
-      <c r="K205" s="3"/>
-      <c r="L205" s="2"/>
-      <c r="M205" s="2"/>
-      <c r="N205" s="2"/>
-      <c r="O205" s="2"/>
-      <c r="P205" s="2"/>
-      <c r="Q205" s="2"/>
-      <c r="R205" s="3"/>
-    </row>
-    <row r="206" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J206" s="2"/>
-      <c r="K206" s="3"/>
-      <c r="L206" s="2"/>
-      <c r="M206" s="2"/>
-      <c r="N206" s="2"/>
-      <c r="O206" s="2"/>
-      <c r="P206" s="2"/>
-      <c r="Q206" s="2"/>
-      <c r="R206" s="3"/>
-    </row>
-    <row r="207" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J207" s="2"/>
-      <c r="K207" s="3"/>
-      <c r="L207" s="2"/>
-      <c r="M207" s="2"/>
-      <c r="N207" s="2"/>
-      <c r="O207" s="2"/>
-      <c r="P207" s="2"/>
-      <c r="Q207" s="2"/>
-      <c r="R207" s="3"/>
-    </row>
-    <row r="208" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J208" s="2"/>
-      <c r="K208" s="3"/>
-      <c r="L208" s="2"/>
-      <c r="M208" s="2"/>
-      <c r="N208" s="2"/>
-      <c r="O208" s="2"/>
-      <c r="P208" s="2"/>
-      <c r="Q208" s="2"/>
-      <c r="R208" s="3"/>
-    </row>
-    <row r="209" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J209" s="2"/>
-      <c r="K209" s="3"/>
-      <c r="L209" s="2"/>
-      <c r="M209" s="2"/>
-      <c r="N209" s="2"/>
-      <c r="O209" s="2"/>
-      <c r="P209" s="2"/>
-      <c r="Q209" s="2"/>
-      <c r="R209" s="3"/>
-    </row>
-    <row r="210" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J210" s="2"/>
-      <c r="K210" s="3"/>
-      <c r="L210" s="2"/>
-      <c r="M210" s="2"/>
-      <c r="N210" s="2"/>
-      <c r="O210" s="2"/>
-      <c r="P210" s="2"/>
-      <c r="Q210" s="2"/>
-      <c r="R210" s="3"/>
-    </row>
-    <row r="211" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J211" s="2"/>
-      <c r="K211" s="3"/>
-      <c r="L211" s="2"/>
-      <c r="M211" s="2"/>
-      <c r="N211" s="2"/>
-      <c r="O211" s="2"/>
-      <c r="P211" s="2"/>
-      <c r="Q211" s="2"/>
-      <c r="R211" s="3"/>
-    </row>
-    <row r="212" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J212" s="2"/>
-      <c r="K212" s="3"/>
-      <c r="L212" s="2"/>
-      <c r="M212" s="2"/>
-      <c r="N212" s="2"/>
-      <c r="O212" s="2"/>
-      <c r="P212" s="2"/>
-      <c r="Q212" s="2"/>
-      <c r="R212" s="3"/>
-    </row>
-    <row r="213" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J213" s="2"/>
-      <c r="K213" s="3"/>
-      <c r="L213" s="2"/>
-      <c r="M213" s="2"/>
-      <c r="N213" s="2"/>
-      <c r="O213" s="2"/>
-      <c r="P213" s="2"/>
-      <c r="Q213" s="2"/>
-      <c r="R213" s="3"/>
-    </row>
-    <row r="214" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J214" s="2"/>
-      <c r="K214" s="3"/>
-      <c r="L214" s="2"/>
-      <c r="M214" s="2"/>
-      <c r="N214" s="2"/>
-      <c r="O214" s="2"/>
-      <c r="P214" s="2"/>
-      <c r="Q214" s="2"/>
-      <c r="R214" s="3"/>
-    </row>
-    <row r="215" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J215" s="2"/>
-      <c r="K215" s="3"/>
-      <c r="L215" s="2"/>
-      <c r="M215" s="2"/>
-      <c r="N215" s="2"/>
-      <c r="O215" s="2"/>
-      <c r="P215" s="2"/>
-      <c r="Q215" s="2"/>
-      <c r="R215" s="3"/>
-    </row>
-    <row r="216" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J216" s="2"/>
-      <c r="K216" s="3"/>
-      <c r="L216" s="2"/>
-      <c r="M216" s="2"/>
-      <c r="N216" s="2"/>
-      <c r="O216" s="2"/>
-      <c r="P216" s="2"/>
-      <c r="Q216" s="2"/>
-      <c r="R216" s="3"/>
-    </row>
-    <row r="217" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J217" s="2"/>
-      <c r="K217" s="3"/>
-      <c r="L217" s="2"/>
-      <c r="M217" s="2"/>
-      <c r="N217" s="2"/>
-      <c r="O217" s="2"/>
-      <c r="P217" s="2"/>
-      <c r="Q217" s="2"/>
-      <c r="R217" s="3"/>
-    </row>
-    <row r="218" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J218" s="2"/>
-      <c r="K218" s="3"/>
-      <c r="L218" s="2"/>
-      <c r="M218" s="2"/>
-      <c r="N218" s="2"/>
-      <c r="O218" s="2"/>
-      <c r="P218" s="2"/>
-      <c r="Q218" s="2"/>
-      <c r="R218" s="3"/>
-    </row>
-    <row r="219" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J219" s="2"/>
-      <c r="K219" s="3"/>
-      <c r="L219" s="2"/>
-      <c r="M219" s="2"/>
-      <c r="N219" s="2"/>
-      <c r="O219" s="2"/>
-      <c r="P219" s="2"/>
-      <c r="Q219" s="2"/>
-      <c r="R219" s="3"/>
-    </row>
-    <row r="220" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="J220" s="2"/>
-      <c r="K220" s="3"/>
-      <c r="L220" s="2"/>
-      <c r="M220" s="2"/>
-      <c r="N220" s="2"/>
-      <c r="O220" s="2"/>
-      <c r="P220" s="2"/>
-      <c r="Q220" s="2"/>
-      <c r="R220" s="3"/>
-    </row>
-    <row r="221" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="222" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="223" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="224" spans="10:18" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="225" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="226" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="227" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="228" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="229" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="230" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="231" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="232" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="233" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="234" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="235" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="236" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="237" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="238" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="239" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="240" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="241" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="242" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="243" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="244" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="245" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="246" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="247" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="248" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="249" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="250" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="251" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="252" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="253" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="254" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="255" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="256" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="257" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="258" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="259" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="260" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="261" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="262" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="263" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="264" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="265" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="266" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="267" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="268" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="269" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="270" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="271" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="272" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="273" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="274" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="275" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="276" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="277" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="278" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="279" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="280" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="281" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="282" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="283" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="284" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="285" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="286" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="287" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="288" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="289" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="290" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="291" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="292" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="293" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="294" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="295" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="296" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="297" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="298" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="299" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="300" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="301" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="302" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="303" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="304" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="305" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="306" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="307" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="308" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="309" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="310" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="311" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="312" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="313" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="314" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="315" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="316" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="317" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="318" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="319" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="320" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="321" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="322" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="323" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="324" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="325" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="326" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="327" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="328" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="329" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="330" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="331" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="332" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="333" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="334" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="335" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="336" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="337" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="338" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="339" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="340" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="341" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="342" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="343" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="344" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="345" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="346" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="347" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="348" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="349" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="350" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="351" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="352" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="353" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="354" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="355" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="356" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="357" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="358" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="359" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="360" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="361" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="362" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="363" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="364" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="365" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="366" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="367" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="368" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="369" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="370" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="371" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="372" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="373" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="374" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="375" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="376" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="377" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="378" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="379" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="380" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="381" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="382" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="383" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="384" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="385" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="386" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="387" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="388" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="389" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="390" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="391" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="392" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="393" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="394" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="395" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="396" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="397" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="398" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="399" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="400" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="401" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="402" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="403" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="404" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="405" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="406" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="407" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="408" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="409" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="410" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="411" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="412" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="413" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="414" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="415" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="416" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="417" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="418" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="419" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="420" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="421" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="422" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="423" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="424" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="425" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="426" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="427" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="428" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="429" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="430" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="431" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="432" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="433" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="434" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="435" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="436" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="437" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="438" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="439" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="440" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="441" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="442" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="443" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="444" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="445" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="446" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="447" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="448" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="449" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="450" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="451" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="452" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="453" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="454" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="455" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="456" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="457" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="458" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="459" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="460" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="461" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="462" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="463" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="464" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="465" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="466" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="467" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="468" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="469" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="470" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="471" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="472" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="473" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="474" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="475" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="476" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="477" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="478" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="479" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="480" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="481" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="482" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="483" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="484" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="485" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="486" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="487" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="488" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="489" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="490" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="491" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="492" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="493" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="494" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="495" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="496" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="497" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="498" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="499" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="500" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="501" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="502" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="503" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="504" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="505" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="506" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="507" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="508" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="509" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="510" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="511" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="512" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="513" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="514" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="515" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="516" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="517" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="518" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="519" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="520" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="521" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="522" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="523" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="524" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="525" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="526" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="527" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="528" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="529" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="530" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="531" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="532" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="533" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="534" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="535" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="536" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="537" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="538" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="539" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="540" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="541" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="542" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="543" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="544" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="545" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="546" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="547" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="548" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="549" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="550" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="551" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="552" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="553" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="554" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="555" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="556" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="557" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="558" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="559" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="560" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="561" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="562" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="563" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="564" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="565" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="566" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="567" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="568" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="569" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="570" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="571" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="572" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="573" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="574" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="575" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="576" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="577" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="578" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="579" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="580" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="581" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="582" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="583" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="584" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="585" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="586" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="587" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="588" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="589" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="590" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="591" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="592" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="593" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="594" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="595" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="596" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="597" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="598" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="599" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="600" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="601" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="602" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="603" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="604" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="605" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="606" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="607" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="608" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="609" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="610" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="611" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="612" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="613" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="614" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="615" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="616" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="617" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="618" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="619" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="620" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="621" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="622" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="623" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="624" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="625" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="626" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="627" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="628" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="629" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="630" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="631" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="632" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="633" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="634" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="635" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="636" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="637" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="638" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="639" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="640" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="641" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="642" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="643" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="644" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="645" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="646" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="647" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="648" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="649" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="650" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="651" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="652" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="653" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="654" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="655" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="656" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="657" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="658" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="659" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="660" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="661" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="662" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="663" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="664" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="665" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="666" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="667" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="668" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="669" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="670" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="671" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="672" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="673" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="674" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="675" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="676" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="677" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="678" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="679" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="680" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="681" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="682" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="683" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="684" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="685" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="686" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="687" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="688" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="689" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="690" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="691" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="692" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="693" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="694" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="695" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="696" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="697" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="698" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="699" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="700" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="701" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="702" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="703" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="704" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="705" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="706" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="707" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="708" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="709" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="710" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="711" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="712" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="713" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="714" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="715" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="716" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="717" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="718" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="719" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="720" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="721" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="722" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="723" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="724" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="725" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="726" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="727" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="728" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="729" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="730" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="731" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="732" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="733" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="734" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="735" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="736" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="737" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="738" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="739" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="740" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="741" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="742" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="743" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="744" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="745" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="746" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="747" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="748" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="749" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="750" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="751" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="752" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="753" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="754" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="755" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="756" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="757" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="758" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="759" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="760" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="761" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="762" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="763" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="764" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="765" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="766" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="767" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="768" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="769" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="770" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="771" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="772" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="773" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="774" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="775" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="776" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="777" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="778" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="779" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="780" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="781" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="782" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="783" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="784" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="785" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="786" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="787" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="788" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="789" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="790" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="791" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="792" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="793" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="794" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="795" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="796" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="797" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="798" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="799" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="800" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="801" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="802" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="803" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="804" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="805" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="806" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="807" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="808" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="809" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="810" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="811" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="812" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="813" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="814" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="815" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="816" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="817" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="818" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="819" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="820" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="821" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="822" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="823" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="824" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="825" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="826" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="827" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="828" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="829" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="830" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="831" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="832" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="833" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="834" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="835" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="836" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="837" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="838" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="839" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="840" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="841" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="842" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="843" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="844" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="845" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="846" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="847" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="848" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="849" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="850" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="851" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="852" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="853" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="854" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="855" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="856" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="857" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="858" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="859" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="860" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="861" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="862" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="863" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="864" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="865" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="866" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="867" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="868" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="869" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="870" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="871" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="872" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="873" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="874" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="875" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="876" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="877" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="878" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="879" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="880" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="881" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="882" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="883" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="884" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="885" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="886" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="887" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="888" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="889" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="890" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="891" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="892" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="927" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="928" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="929" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="930" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="931" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="932" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="933" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="934" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="935" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="936" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="937" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="938" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="939" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="940" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="941" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="942" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="943" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="944" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="945" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="946" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="947" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="948" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="949" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="950" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="951" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="952" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="953" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="954" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="955" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="956" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="957" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="958" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="959" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="960" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="961" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="962" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="963" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="964" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="965" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="966" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="967" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="968" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="969" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="970" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="971" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="972" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="973" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="974" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="975" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="976" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="977" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="978" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="979" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="980" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="981" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="982" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="983" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="984" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="985" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="986" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="987" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="988" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="989" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="990" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="991" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="992" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="993" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="994" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="10" spans="1:21" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="44"/>
+      <c r="B10" s="44"/>
+      <c r="C10" s="44"/>
+      <c r="D10" s="44"/>
+      <c r="E10" s="44"/>
+      <c r="F10" s="44"/>
+      <c r="G10" s="44"/>
+      <c r="H10" s="44"/>
+      <c r="I10" s="44"/>
+      <c r="J10" s="44"/>
+      <c r="K10" s="44"/>
+      <c r="L10" s="44"/>
+      <c r="M10" s="44"/>
+      <c r="N10" s="44"/>
+      <c r="O10" s="44"/>
+      <c r="P10" s="44"/>
+      <c r="Q10" s="44"/>
+      <c r="R10" s="44"/>
+      <c r="S10" s="44">
+        <f>SUM(S$9:S9)</f>
+        <v>0</v>
+      </c>
+      <c r="T10" s="44">
+        <f>SUM(T$9:T9)</f>
+        <v>0</v>
+      </c>
+      <c r="U10" s="22" t="s">
+        <v>150</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="E2:G6"/>
@@ -4463,7 +1566,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="13" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="1"/>
@@ -4474,13 +1577,13 @@
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="31" t="s">
+      <c r="C2" s="48" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="29"/>
-      <c r="E2" s="29"/>
-      <c r="F2" s="29"/>
-      <c r="G2" s="29"/>
+      <c r="D2" s="46"/>
+      <c r="E2" s="46"/>
+      <c r="F2" s="46"/>
+      <c r="G2" s="46"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
@@ -4488,12 +1591,12 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="14" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="14" t="s">
         <v>5</v>
       </c>
     </row>
@@ -4536,7 +1639,7 @@
       <c r="H8" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="23" t="s">
+      <c r="I8" s="17" t="s">
         <v>148</v>
       </c>
     </row>
@@ -4565,7 +1668,7 @@
       <c r="H9" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="I9" s="24" t="s">
+      <c r="I9" s="18" t="s">
         <v>149</v>
       </c>
     </row>
@@ -5706,7 +2809,7 @@
       <c r="AF3" s="2"/>
     </row>
     <row r="4" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="14" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="2"/>
@@ -5742,7 +2845,7 @@
       <c r="AF4" s="2"/>
     </row>
     <row r="5" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="19"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -5810,7 +2913,7 @@
       <c r="AF6" s="2"/>
     </row>
     <row r="7" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="15" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2">
@@ -5848,242 +2951,242 @@
       <c r="AF7" s="2"/>
     </row>
     <row r="8" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="32" t="s">
+      <c r="A8" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="34" t="s">
+      <c r="B8" s="51" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="34" t="s">
+      <c r="C8" s="51" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="34" t="s">
+      <c r="D8" s="51" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="34" t="s">
+      <c r="E8" s="51" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="34" t="s">
+      <c r="F8" s="51" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="34" t="s">
+      <c r="G8" s="51" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="34" t="s">
+      <c r="H8" s="51" t="s">
         <v>73</v>
       </c>
-      <c r="I8" s="34" t="s">
+      <c r="I8" s="51" t="s">
         <v>74</v>
       </c>
-      <c r="J8" s="34" t="s">
+      <c r="J8" s="51" t="s">
         <v>75</v>
       </c>
-      <c r="K8" s="34" t="s">
+      <c r="K8" s="51" t="s">
         <v>76</v>
       </c>
-      <c r="L8" s="34" t="s">
+      <c r="L8" s="51" t="s">
         <v>77</v>
       </c>
-      <c r="M8" s="34" t="s">
+      <c r="M8" s="51" t="s">
         <v>78</v>
       </c>
-      <c r="N8" s="34" t="s">
+      <c r="N8" s="51" t="s">
         <v>79</v>
       </c>
-      <c r="O8" s="34" t="s">
+      <c r="O8" s="51" t="s">
         <v>80</v>
       </c>
-      <c r="P8" s="34" t="s">
+      <c r="P8" s="51" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="34" t="s">
+      <c r="Q8" s="51" t="s">
         <v>82</v>
       </c>
-      <c r="R8" s="34" t="s">
+      <c r="R8" s="51" t="s">
         <v>83</v>
       </c>
-      <c r="S8" s="34" t="s">
+      <c r="S8" s="51" t="s">
         <v>84</v>
       </c>
-      <c r="T8" s="34" t="s">
+      <c r="T8" s="51" t="s">
         <v>85</v>
       </c>
-      <c r="U8" s="35" t="s">
+      <c r="U8" s="52" t="s">
         <v>86</v>
       </c>
-      <c r="V8" s="36"/>
-      <c r="W8" s="36"/>
-      <c r="X8" s="36"/>
-      <c r="Y8" s="36"/>
-      <c r="Z8" s="36"/>
-      <c r="AA8" s="36"/>
-      <c r="AB8" s="36"/>
-      <c r="AC8" s="37"/>
-      <c r="AD8" s="32" t="s">
+      <c r="V8" s="53"/>
+      <c r="W8" s="53"/>
+      <c r="X8" s="53"/>
+      <c r="Y8" s="53"/>
+      <c r="Z8" s="53"/>
+      <c r="AA8" s="53"/>
+      <c r="AB8" s="53"/>
+      <c r="AC8" s="54"/>
+      <c r="AD8" s="49" t="s">
         <v>87</v>
       </c>
-      <c r="AE8" s="32" t="s">
+      <c r="AE8" s="49" t="s">
         <v>88</v>
       </c>
-      <c r="AF8" s="32" t="s">
+      <c r="AF8" s="49" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="33"/>
-      <c r="B9" s="33"/>
-      <c r="C9" s="33"/>
-      <c r="D9" s="33"/>
-      <c r="E9" s="33"/>
-      <c r="F9" s="33"/>
-      <c r="G9" s="33"/>
-      <c r="H9" s="33"/>
-      <c r="I9" s="33"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="33"/>
-      <c r="L9" s="33"/>
-      <c r="M9" s="33"/>
-      <c r="N9" s="33"/>
-      <c r="O9" s="33"/>
-      <c r="P9" s="33"/>
-      <c r="Q9" s="33"/>
-      <c r="R9" s="33"/>
-      <c r="S9" s="33"/>
-      <c r="T9" s="33"/>
-      <c r="U9" s="21">
+      <c r="A9" s="50"/>
+      <c r="B9" s="50"/>
+      <c r="C9" s="50"/>
+      <c r="D9" s="50"/>
+      <c r="E9" s="50"/>
+      <c r="F9" s="50"/>
+      <c r="G9" s="50"/>
+      <c r="H9" s="50"/>
+      <c r="I9" s="50"/>
+      <c r="J9" s="50"/>
+      <c r="K9" s="50"/>
+      <c r="L9" s="50"/>
+      <c r="M9" s="50"/>
+      <c r="N9" s="50"/>
+      <c r="O9" s="50"/>
+      <c r="P9" s="50"/>
+      <c r="Q9" s="50"/>
+      <c r="R9" s="50"/>
+      <c r="S9" s="50"/>
+      <c r="T9" s="50"/>
+      <c r="U9" s="16">
         <v>5011</v>
       </c>
-      <c r="V9" s="21">
+      <c r="V9" s="16">
         <v>5007</v>
       </c>
-      <c r="W9" s="21">
+      <c r="W9" s="16">
         <v>5006</v>
       </c>
-      <c r="X9" s="21">
+      <c r="X9" s="16">
         <v>2008</v>
       </c>
-      <c r="Y9" s="21">
+      <c r="Y9" s="16">
         <v>2005</v>
       </c>
-      <c r="Z9" s="21">
+      <c r="Z9" s="16">
         <v>2037</v>
       </c>
-      <c r="AA9" s="21">
+      <c r="AA9" s="16">
         <v>2025</v>
       </c>
-      <c r="AB9" s="21">
+      <c r="AB9" s="16">
         <v>2022</v>
       </c>
-      <c r="AC9" s="21" t="s">
+      <c r="AC9" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="AD9" s="33"/>
-      <c r="AE9" s="33"/>
-      <c r="AF9" s="33"/>
+      <c r="AD9" s="50"/>
+      <c r="AE9" s="50"/>
+      <c r="AF9" s="50"/>
     </row>
     <row r="10" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="12" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="26">
+      <c r="F10" s="20">
         <f>IFERROR(IF(A10="No data","",IF(C10=0,0,D10/C10)),0)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="16" t="s">
+      <c r="G10" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="27">
+      <c r="H10" s="21">
         <f>IFERROR(IF(A10="No data","",IF(B10&lt;&gt;0, G10/B10, 0)),0)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="16" t="s">
+      <c r="I10" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="J10" s="16" t="s">
+      <c r="J10" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="K10" s="16">
+      <c r="K10" s="12">
         <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="26">
+      <c r="L10" s="20">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,I10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="26">
+      <c r="M10" s="20">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,J10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="N10" s="26">
+      <c r="N10" s="20">
         <f>IFERROR(IF(A10="No data","",IF(D10=0,0,I10/D10)),0)</f>
         <v>0</v>
       </c>
-      <c r="O10" s="26">
+      <c r="O10" s="20">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,K10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="P10" s="16" t="s">
+      <c r="P10" s="12" t="s">
         <v>98</v>
       </c>
-      <c r="Q10" s="16" t="s">
+      <c r="Q10" s="12" t="s">
         <v>99</v>
       </c>
-      <c r="R10" s="16" t="s">
+      <c r="R10" s="12" t="s">
         <v>100</v>
       </c>
-      <c r="S10" s="26">
+      <c r="S10" s="20">
         <f>IFERROR(IF(A10="No data","",IF(I10=0,0,R10/I10)),0)</f>
         <v>0</v>
       </c>
-      <c r="T10" s="16" t="s">
+      <c r="T10" s="12" t="s">
         <v>101</v>
       </c>
-      <c r="U10" s="16" t="s">
+      <c r="U10" s="12" t="s">
         <v>102</v>
       </c>
-      <c r="V10" s="16" t="s">
+      <c r="V10" s="12" t="s">
         <v>103</v>
       </c>
-      <c r="W10" s="16" t="s">
+      <c r="W10" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="X10" s="16" t="s">
+      <c r="X10" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="Y10" s="16" t="s">
+      <c r="Y10" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="Z10" s="16" t="s">
+      <c r="Z10" s="12" t="s">
         <v>107</v>
       </c>
-      <c r="AA10" s="16" t="s">
+      <c r="AA10" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="AB10" s="16" t="s">
+      <c r="AB10" s="12" t="s">
         <v>109</v>
       </c>
-      <c r="AC10" s="16" t="s">
+      <c r="AC10" s="12" t="s">
         <v>110</v>
       </c>
-      <c r="AD10" s="16" t="s">
+      <c r="AD10" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="AE10" s="16" t="s">
+      <c r="AE10" s="12" t="s">
         <v>112</v>
       </c>
-      <c r="AF10" s="16">
+      <c r="AF10" s="12">
         <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10+AE10),0)</f>
         <v>0</v>
       </c>
@@ -13901,7 +11004,7 @@
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="19" t="s">
+      <c r="A4" s="14" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="2"/>
@@ -13917,7 +11020,7 @@
       <c r="L4" s="2"/>
     </row>
     <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="14" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="2"/>
@@ -13949,7 +11052,7 @@
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="20" t="s">
+      <c r="A7" s="15" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2">
@@ -13967,94 +11070,94 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="38" t="s">
+      <c r="A8" s="55" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="35" t="s">
+      <c r="B8" s="52" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="36"/>
-      <c r="D8" s="36"/>
-      <c r="E8" s="36"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="36"/>
-      <c r="H8" s="36"/>
-      <c r="I8" s="36"/>
-      <c r="J8" s="37"/>
-      <c r="K8" s="39" t="s">
+      <c r="C8" s="53"/>
+      <c r="D8" s="53"/>
+      <c r="E8" s="53"/>
+      <c r="F8" s="53"/>
+      <c r="G8" s="53"/>
+      <c r="H8" s="53"/>
+      <c r="I8" s="53"/>
+      <c r="J8" s="54"/>
+      <c r="K8" s="56" t="s">
         <v>114</v>
       </c>
-      <c r="L8" s="39" t="s">
+      <c r="L8" s="56" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="33"/>
-      <c r="B9" s="21">
+      <c r="A9" s="50"/>
+      <c r="B9" s="16">
         <v>5011</v>
       </c>
-      <c r="C9" s="21">
+      <c r="C9" s="16">
         <v>5007</v>
       </c>
-      <c r="D9" s="21">
+      <c r="D9" s="16">
         <v>5006</v>
       </c>
-      <c r="E9" s="21">
+      <c r="E9" s="16">
         <v>2008</v>
       </c>
-      <c r="F9" s="21">
+      <c r="F9" s="16">
         <v>2005</v>
       </c>
-      <c r="G9" s="21">
+      <c r="G9" s="16">
         <v>2037</v>
       </c>
-      <c r="H9" s="21">
+      <c r="H9" s="16">
         <v>2025</v>
       </c>
-      <c r="I9" s="21">
+      <c r="I9" s="16">
         <v>2022</v>
       </c>
-      <c r="J9" s="21" t="s">
+      <c r="J9" s="16" t="s">
         <v>90</v>
       </c>
-      <c r="K9" s="33"/>
-      <c r="L9" s="33"/>
+      <c r="K9" s="50"/>
+      <c r="L9" s="50"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="19" t="s">
+      <c r="A10" s="23" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="24" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="24" t="s">
         <v>103</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="24" t="s">
         <v>104</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="24" t="s">
         <v>105</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="24" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="24" t="s">
         <v>108</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="J10" s="2" t="s">
+      <c r="J10" s="24" t="s">
         <v>110</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="24" t="s">
         <v>111</v>
       </c>
-      <c r="L10" s="2" t="e">
+      <c r="L10" s="25" t="e">
         <f>B10+C10+D10+E10+F10+G10+H10+I10+J10+K10</f>
         <v>#VALUE!</v>
       </c>
@@ -17588,317 +14691,317 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:C1000"/>
+  <dimension ref="B2:D1001"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.1640625" customWidth="1"/>
-    <col min="2" max="2" width="39.1640625" customWidth="1"/>
-    <col min="3" max="3" width="100.6640625" customWidth="1"/>
-    <col min="4" max="6" width="8.6640625" customWidth="1"/>
+    <col min="1" max="1" width="3.5" customWidth="1"/>
+    <col min="2" max="2" width="7.5" customWidth="1"/>
+    <col min="3" max="3" width="39.1640625" customWidth="1"/>
+    <col min="4" max="4" width="74.1640625" customWidth="1"/>
+    <col min="5" max="7" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="17" t="s">
+    <row r="2" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="38" t="s">
         <v>115</v>
       </c>
-      <c r="B1" s="17" t="s">
+      <c r="C2" s="38" t="s">
         <v>116</v>
       </c>
-      <c r="C1" s="17" t="s">
+      <c r="D2" s="38" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="22">
+    <row r="3" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B3" s="35">
         <v>1001</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="C3" s="36" t="s">
         <v>118</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="D3" s="37" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="22">
+    <row r="4" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B4" s="26">
         <v>1002</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="C4" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="D4" s="28" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="22">
+    <row r="5" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B5" s="32">
         <v>1004</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="C5" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="D5" s="34" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="22">
+    <row r="6" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="26">
         <v>1005</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="C6" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="C5" s="22" t="s">
+      <c r="D6" s="28" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="22">
+    <row r="7" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="32">
         <v>1006</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="C7" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="C6" s="22" t="s">
+      <c r="D7" s="34" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="22">
+    <row r="8" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="26">
         <v>1007</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="C8" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="C7" s="22" t="s">
+      <c r="D8" s="28" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="22">
+    <row r="9" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="32">
         <v>1017</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="C9" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="D9" s="34" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="22">
+    <row r="10" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="26">
         <v>1018</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="C10" s="27" t="s">
         <v>118</v>
       </c>
-      <c r="C9" s="22" t="s">
+      <c r="D10" s="28" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="22">
+    <row r="11" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="32">
         <v>2003</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="C11" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="C10" s="22" t="s">
+      <c r="D11" s="34" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="22">
+    <row r="12" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="26">
         <v>2005</v>
       </c>
-      <c r="B11" s="22" t="s">
+      <c r="C12" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="D12" s="28" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="22">
+    <row r="13" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="32">
         <v>2008</v>
       </c>
-      <c r="B12" s="22" t="s">
+      <c r="C13" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="C12" s="22" t="s">
+      <c r="D13" s="34" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="22">
+    <row r="14" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B14" s="26">
         <v>2009</v>
       </c>
-      <c r="B13" s="22" t="s">
+      <c r="C14" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="C13" s="22" t="s">
+      <c r="D14" s="28" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="22">
+    <row r="15" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="32">
         <v>2011</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="C15" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="D15" s="34" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="22">
+    <row r="16" spans="2:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B16" s="26">
         <v>2014</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="C16" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="D16" s="28" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="22">
+    <row r="17" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="32">
         <v>2016</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="C17" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="D17" s="34" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="22">
+    <row r="18" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B18" s="26">
         <v>2018</v>
       </c>
-      <c r="B17" s="22" t="s">
+      <c r="C18" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="C17" s="22" t="s">
+      <c r="D18" s="28" t="s">
         <v>136</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="22">
+    <row r="19" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="32">
         <v>2022</v>
       </c>
-      <c r="B18" s="22" t="s">
+      <c r="C19" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="C18" s="22" t="s">
+      <c r="D19" s="34" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="22">
+    <row r="20" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B20" s="26">
         <v>2025</v>
       </c>
-      <c r="B19" s="22" t="s">
+      <c r="C20" s="27" t="s">
         <v>132</v>
       </c>
-      <c r="C19" s="22" t="s">
+      <c r="D20" s="28" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="22">
+    <row r="21" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="32">
         <v>2032</v>
       </c>
-      <c r="B20" s="22" t="s">
+      <c r="C21" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="C20" s="22" t="s">
+      <c r="D21" s="34" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="22">
+    <row r="22" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B22" s="26">
         <v>2034</v>
       </c>
-      <c r="B21" s="22" t="s">
+      <c r="C22" s="27" t="s">
         <v>127</v>
       </c>
-      <c r="C21" s="22" t="s">
+      <c r="D22" s="28" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="22">
+    <row r="23" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B23" s="32">
         <v>2037</v>
       </c>
-      <c r="B22" s="22" t="s">
+      <c r="C23" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="C22" s="22" t="s">
+      <c r="D23" s="34" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="22">
+    <row r="24" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B24" s="26">
         <v>4010</v>
       </c>
-      <c r="B23" s="22" t="s">
+      <c r="C24" s="27" t="s">
         <v>142</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="D24" s="28" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="22">
+    <row r="25" spans="2:4" ht="34" x14ac:dyDescent="0.2">
+      <c r="B25" s="32">
         <v>4017</v>
       </c>
-      <c r="B24" s="22" t="s">
+      <c r="C25" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="C24" s="22" t="s">
+      <c r="D25" s="34" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="22">
+    <row r="26" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B26" s="26">
         <v>5006</v>
       </c>
-      <c r="B25" s="22" t="s">
+      <c r="C26" s="27" t="s">
         <v>144</v>
       </c>
-      <c r="C25" s="22" t="s">
+      <c r="D26" s="28" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="22">
+    <row r="27" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B27" s="32">
         <v>5007</v>
       </c>
-      <c r="B26" s="22" t="s">
+      <c r="C27" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="C26" s="22" t="s">
+      <c r="D27" s="34" t="s">
         <v>146</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="22">
+    <row r="28" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="29">
         <v>5011</v>
       </c>
-      <c r="B27" s="22" t="s">
+      <c r="C28" s="30" t="s">
         <v>144</v>
       </c>
-      <c r="C27" s="22" t="s">
+      <c r="D28" s="31" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="28" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="29" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="30" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="31" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="32" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="29" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="30" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="31" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="32" spans="2:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -18867,6 +15970,7 @@
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="1001" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="portrait"/>

</xml_diff>

<commit_message>
[feat/ASP-7746-Device-and-Sites-Summary-Report-include-Total-line] Added TB Reach to Uk template, normalized formats and formulas. Added totals to all sheets.
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10420"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10526"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_and_site_summary_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACB0970F-FE9C-8E4E-AC4A-E1D297E03903}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F0C0E2-5A41-F74E-BBE7-C332410CB92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="152">
   <si>
     <t>Device and Site Summary Report</t>
   </si>
@@ -517,6 +517,9 @@
   <si>
     <t>#SUM_DYNAMIC</t>
   </si>
+  <si>
+    <t>Totals</t>
+  </si>
 </sst>
 </file>
 
@@ -526,7 +529,7 @@
     <numFmt numFmtId="164" formatCode="[$-409]mmmm\ d&quot;, &quot;yyyy"/>
     <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color rgb="FF000000"/>
@@ -598,6 +601,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -625,7 +636,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -658,17 +669,6 @@
       <top style="thin">
         <color rgb="FF000000"/>
       </top>
-      <bottom style="thin">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
@@ -834,11 +834,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="57">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -861,13 +924,6 @@
     <xf numFmtId="165" fontId="5" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -881,25 +937,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="2" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -907,7 +947,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -916,7 +956,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -928,28 +968,66 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -960,22 +1038,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1275,11 +1353,11 @@
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="45" t="s">
+      <c r="E2" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
       <c r="H2" s="5"/>
       <c r="J2" s="2"/>
       <c r="K2" s="3"/>
@@ -1295,11 +1373,11 @@
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="47"/>
-      <c r="D3" s="46"/>
-      <c r="E3" s="46"/>
-      <c r="F3" s="46"/>
-      <c r="G3" s="46"/>
+      <c r="C3" s="56"/>
+      <c r="D3" s="55"/>
+      <c r="E3" s="55"/>
+      <c r="F3" s="55"/>
+      <c r="G3" s="55"/>
       <c r="H3" s="5"/>
       <c r="J3" s="2"/>
       <c r="K3" s="3"/>
@@ -1315,9 +1393,9 @@
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="46"/>
-      <c r="F4" s="46"/>
-      <c r="G4" s="46"/>
+      <c r="E4" s="55"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="55"/>
       <c r="H4" s="5"/>
       <c r="J4" s="2"/>
       <c r="K4" s="3"/>
@@ -1333,9 +1411,9 @@
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="46"/>
-      <c r="F5" s="46"/>
-      <c r="G5" s="46"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
       <c r="H5" s="5"/>
       <c r="J5" s="2"/>
       <c r="K5" s="3"/>
@@ -1351,9 +1429,9 @@
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="46"/>
-      <c r="F6" s="46"/>
-      <c r="G6" s="46"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
       <c r="J6" s="2"/>
       <c r="K6" s="3"/>
       <c r="L6" s="2"/>
@@ -1443,95 +1521,97 @@
       </c>
     </row>
     <row r="9" spans="1:21" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C9" s="41" t="s">
+      <c r="C9" s="31" t="s">
         <v>30</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="31" t="s">
         <v>31</v>
       </c>
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="F9" s="40" t="s">
+      <c r="F9" s="30" t="s">
         <v>33</v>
       </c>
-      <c r="G9" s="41" t="s">
+      <c r="G9" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="H9" s="41" t="s">
+      <c r="H9" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="40" t="s">
+      <c r="I9" s="30" t="s">
         <v>36</v>
       </c>
-      <c r="J9" s="42" t="s">
+      <c r="J9" s="32" t="s">
         <v>37</v>
       </c>
-      <c r="K9" s="42" t="s">
+      <c r="K9" s="32" t="s">
         <v>38</v>
       </c>
-      <c r="L9" s="43" t="s">
+      <c r="L9" s="33" t="s">
         <v>39</v>
       </c>
-      <c r="M9" s="43" t="s">
+      <c r="M9" s="33" t="s">
         <v>40</v>
       </c>
-      <c r="N9" s="43" t="s">
+      <c r="N9" s="33" t="s">
         <v>41</v>
       </c>
-      <c r="O9" s="43" t="s">
+      <c r="O9" s="33" t="s">
         <v>42</v>
       </c>
-      <c r="P9" s="43" t="s">
+      <c r="P9" s="33" t="s">
         <v>43</v>
       </c>
-      <c r="Q9" s="43" t="s">
+      <c r="Q9" s="33" t="s">
         <v>44</v>
       </c>
-      <c r="R9" s="42" t="s">
+      <c r="R9" s="32" t="s">
         <v>45</v>
       </c>
-      <c r="S9" s="39" t="s">
+      <c r="S9" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="T9" s="39" t="s">
+      <c r="T9" s="29" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:21" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="44"/>
-      <c r="B10" s="44"/>
-      <c r="C10" s="44"/>
-      <c r="D10" s="44"/>
-      <c r="E10" s="44"/>
-      <c r="F10" s="44"/>
-      <c r="G10" s="44"/>
-      <c r="H10" s="44"/>
-      <c r="I10" s="44"/>
-      <c r="J10" s="44"/>
-      <c r="K10" s="44"/>
-      <c r="L10" s="44"/>
-      <c r="M10" s="44"/>
-      <c r="N10" s="44"/>
-      <c r="O10" s="44"/>
-      <c r="P10" s="44"/>
-      <c r="Q10" s="44"/>
-      <c r="R10" s="44"/>
-      <c r="S10" s="44">
+      <c r="A10" s="35" t="s">
+        <v>151</v>
+      </c>
+      <c r="B10" s="34"/>
+      <c r="C10" s="34"/>
+      <c r="D10" s="34"/>
+      <c r="E10" s="34"/>
+      <c r="F10" s="34"/>
+      <c r="G10" s="34"/>
+      <c r="H10" s="34"/>
+      <c r="I10" s="34"/>
+      <c r="J10" s="34"/>
+      <c r="K10" s="34"/>
+      <c r="L10" s="34"/>
+      <c r="M10" s="34"/>
+      <c r="N10" s="34"/>
+      <c r="O10" s="34"/>
+      <c r="P10" s="34"/>
+      <c r="Q10" s="34"/>
+      <c r="R10" s="34"/>
+      <c r="S10" s="34">
         <f>SUM(S$9:S9)</f>
         <v>0</v>
       </c>
-      <c r="T10" s="44">
+      <c r="T10" s="34">
         <f>SUM(T$9:T9)</f>
         <v>0</v>
       </c>
-      <c r="U10" s="22" t="s">
+      <c r="U10" s="15" t="s">
         <v>150</v>
       </c>
     </row>
@@ -1566,7 +1646,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="10" t="s">
         <v>48</v>
       </c>
       <c r="B1" s="1"/>
@@ -1577,13 +1657,13 @@
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="57" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="46"/>
-      <c r="E2" s="46"/>
-      <c r="F2" s="46"/>
-      <c r="G2" s="46"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="55"/>
+      <c r="F2" s="55"/>
+      <c r="G2" s="55"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
@@ -1591,12 +1671,12 @@
       </c>
     </row>
     <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="11" t="s">
         <v>5</v>
       </c>
     </row>
@@ -1639,40 +1719,73 @@
       <c r="H8" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="I8" s="17" t="s">
+      <c r="I8" s="14" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="41" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="41" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="47" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="D9" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="41" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="10" t="s">
+      <c r="F9" s="41" t="s">
         <v>63</v>
       </c>
-      <c r="G9" s="10" t="s">
+      <c r="G9" s="41" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="10" t="s">
+      <c r="H9" s="41" t="s">
         <v>65</v>
       </c>
-      <c r="I9" s="18" t="s">
+      <c r="I9" s="42" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="43" t="s">
+        <v>151</v>
+      </c>
+      <c r="B10" s="44"/>
+      <c r="C10" s="46" t="e">
+        <f>AVERAGE(C$9:C9)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="D10" s="44">
+        <f>SUM(D$9:D9)</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="44">
+        <f>SUM(E$9:E9)</f>
+        <v>0</v>
+      </c>
+      <c r="F10" s="44">
+        <f>SUM(F$9:F9)</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="46" t="e">
+        <f>AVERAGE(G$9:G9)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="H10" s="44">
+        <f>SUM(H$9:H9)</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="45">
+        <f>SUM(I$9:I9)</f>
+        <v>0</v>
+      </c>
+    </row>
     <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="12" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="13" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -2809,7 +2922,7 @@
       <c r="AF3" s="2"/>
     </row>
     <row r="4" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="2"/>
@@ -2845,7 +2958,7 @@
       <c r="AF4" s="2"/>
     </row>
     <row r="5" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14"/>
+      <c r="A5" s="11"/>
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2913,7 +3026,7 @@
       <c r="AF6" s="2"/>
     </row>
     <row r="7" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2">
@@ -2951,278 +3064,362 @@
       <c r="AF7" s="2"/>
     </row>
     <row r="8" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="49" t="s">
+      <c r="A8" s="58" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="51" t="s">
+      <c r="B8" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="51" t="s">
+      <c r="C8" s="60" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="51" t="s">
+      <c r="D8" s="60" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="51" t="s">
+      <c r="E8" s="60" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="51" t="s">
+      <c r="F8" s="60" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="51" t="s">
+      <c r="G8" s="60" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="51" t="s">
+      <c r="H8" s="60" t="s">
         <v>73</v>
       </c>
-      <c r="I8" s="51" t="s">
+      <c r="I8" s="60" t="s">
         <v>74</v>
       </c>
-      <c r="J8" s="51" t="s">
+      <c r="J8" s="60" t="s">
         <v>75</v>
       </c>
-      <c r="K8" s="51" t="s">
+      <c r="K8" s="60" t="s">
         <v>76</v>
       </c>
-      <c r="L8" s="51" t="s">
+      <c r="L8" s="60" t="s">
         <v>77</v>
       </c>
-      <c r="M8" s="51" t="s">
+      <c r="M8" s="60" t="s">
         <v>78</v>
       </c>
-      <c r="N8" s="51" t="s">
+      <c r="N8" s="60" t="s">
         <v>79</v>
       </c>
-      <c r="O8" s="51" t="s">
+      <c r="O8" s="60" t="s">
         <v>80</v>
       </c>
-      <c r="P8" s="51" t="s">
+      <c r="P8" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="51" t="s">
+      <c r="Q8" s="60" t="s">
         <v>82</v>
       </c>
-      <c r="R8" s="51" t="s">
+      <c r="R8" s="60" t="s">
         <v>83</v>
       </c>
-      <c r="S8" s="51" t="s">
+      <c r="S8" s="60" t="s">
         <v>84</v>
       </c>
-      <c r="T8" s="51" t="s">
+      <c r="T8" s="60" t="s">
         <v>85</v>
       </c>
-      <c r="U8" s="52" t="s">
+      <c r="U8" s="61" t="s">
         <v>86</v>
       </c>
-      <c r="V8" s="53"/>
-      <c r="W8" s="53"/>
-      <c r="X8" s="53"/>
-      <c r="Y8" s="53"/>
-      <c r="Z8" s="53"/>
-      <c r="AA8" s="53"/>
-      <c r="AB8" s="53"/>
-      <c r="AC8" s="54"/>
-      <c r="AD8" s="49" t="s">
+      <c r="V8" s="62"/>
+      <c r="W8" s="62"/>
+      <c r="X8" s="62"/>
+      <c r="Y8" s="62"/>
+      <c r="Z8" s="62"/>
+      <c r="AA8" s="62"/>
+      <c r="AB8" s="62"/>
+      <c r="AC8" s="63"/>
+      <c r="AD8" s="58" t="s">
         <v>87</v>
       </c>
-      <c r="AE8" s="49" t="s">
+      <c r="AE8" s="58" t="s">
         <v>88</v>
       </c>
-      <c r="AF8" s="49" t="s">
+      <c r="AF8" s="58" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="50"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="50"/>
-      <c r="E9" s="50"/>
-      <c r="F9" s="50"/>
-      <c r="G9" s="50"/>
-      <c r="H9" s="50"/>
-      <c r="I9" s="50"/>
-      <c r="J9" s="50"/>
-      <c r="K9" s="50"/>
-      <c r="L9" s="50"/>
-      <c r="M9" s="50"/>
-      <c r="N9" s="50"/>
-      <c r="O9" s="50"/>
-      <c r="P9" s="50"/>
-      <c r="Q9" s="50"/>
-      <c r="R9" s="50"/>
-      <c r="S9" s="50"/>
-      <c r="T9" s="50"/>
-      <c r="U9" s="16">
+      <c r="A9" s="59"/>
+      <c r="B9" s="59"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="59"/>
+      <c r="E9" s="59"/>
+      <c r="F9" s="59"/>
+      <c r="G9" s="59"/>
+      <c r="H9" s="59"/>
+      <c r="I9" s="59"/>
+      <c r="J9" s="59"/>
+      <c r="K9" s="59"/>
+      <c r="L9" s="59"/>
+      <c r="M9" s="59"/>
+      <c r="N9" s="59"/>
+      <c r="O9" s="59"/>
+      <c r="P9" s="59"/>
+      <c r="Q9" s="59"/>
+      <c r="R9" s="59"/>
+      <c r="S9" s="59"/>
+      <c r="T9" s="59"/>
+      <c r="U9" s="13">
         <v>5011</v>
       </c>
-      <c r="V9" s="16">
+      <c r="V9" s="13">
         <v>5007</v>
       </c>
-      <c r="W9" s="16">
+      <c r="W9" s="13">
         <v>5006</v>
       </c>
-      <c r="X9" s="16">
+      <c r="X9" s="13">
         <v>2008</v>
       </c>
-      <c r="Y9" s="16">
+      <c r="Y9" s="13">
         <v>2005</v>
       </c>
-      <c r="Z9" s="16">
+      <c r="Z9" s="13">
         <v>2037</v>
       </c>
-      <c r="AA9" s="16">
+      <c r="AA9" s="13">
         <v>2025</v>
       </c>
-      <c r="AB9" s="16">
+      <c r="AB9" s="13">
         <v>2022</v>
       </c>
-      <c r="AC9" s="16" t="s">
+      <c r="AC9" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="AD9" s="50"/>
-      <c r="AE9" s="50"/>
-      <c r="AF9" s="50"/>
-    </row>
-    <row r="10" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="19" t="s">
+      <c r="AD9" s="59"/>
+      <c r="AE9" s="59"/>
+      <c r="AF9" s="59"/>
+    </row>
+    <row r="10" spans="1:32" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="36" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="37" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="37" t="s">
         <v>93</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="20">
+      <c r="F10" s="48">
         <f>IFERROR(IF(A10="No data","",IF(C10=0,0,D10/C10)),0)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="37" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="21">
+      <c r="H10" s="49">
         <f>IFERROR(IF(A10="No data","",IF(B10&lt;&gt;0, G10/B10, 0)),0)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="12" t="s">
+      <c r="I10" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="J10" s="12" t="s">
+      <c r="J10" s="37" t="s">
         <v>97</v>
       </c>
-      <c r="K10" s="12">
+      <c r="K10" s="37">
         <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="20">
+      <c r="L10" s="48">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,I10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="20">
+      <c r="M10" s="48">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,J10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="N10" s="20">
+      <c r="N10" s="48">
         <f>IFERROR(IF(A10="No data","",IF(D10=0,0,I10/D10)),0)</f>
         <v>0</v>
       </c>
-      <c r="O10" s="20">
+      <c r="O10" s="48">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,K10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="P10" s="12" t="s">
+      <c r="P10" s="37" t="s">
         <v>98</v>
       </c>
-      <c r="Q10" s="12" t="s">
+      <c r="Q10" s="37" t="s">
         <v>99</v>
       </c>
-      <c r="R10" s="12" t="s">
+      <c r="R10" s="37" t="s">
         <v>100</v>
       </c>
-      <c r="S10" s="20">
+      <c r="S10" s="48">
         <f>IFERROR(IF(A10="No data","",IF(I10=0,0,R10/I10)),0)</f>
         <v>0</v>
       </c>
-      <c r="T10" s="12" t="s">
+      <c r="T10" s="52" t="s">
         <v>101</v>
       </c>
-      <c r="U10" s="12" t="s">
+      <c r="U10" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="V10" s="12" t="s">
+      <c r="V10" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="W10" s="12" t="s">
+      <c r="W10" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="X10" s="12" t="s">
+      <c r="X10" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="Y10" s="12" t="s">
+      <c r="Y10" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="Z10" s="12" t="s">
+      <c r="Z10" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="AA10" s="12" t="s">
+      <c r="AA10" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="AB10" s="12" t="s">
+      <c r="AB10" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="AC10" s="12" t="s">
+      <c r="AC10" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="AD10" s="12" t="s">
+      <c r="AD10" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="AE10" s="12" t="s">
+      <c r="AE10" s="37" t="s">
         <v>112</v>
       </c>
-      <c r="AF10" s="12">
+      <c r="AF10" s="37">
         <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10+AE10),0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
-      <c r="N11" s="2"/>
-      <c r="O11" s="2"/>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="2"/>
-      <c r="U11" s="2"/>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
-      <c r="Y11" s="2"/>
-      <c r="Z11" s="2"/>
-      <c r="AA11" s="2"/>
-      <c r="AB11" s="2"/>
-      <c r="AC11" s="2"/>
-      <c r="AD11" s="2"/>
-      <c r="AE11" s="2"/>
-      <c r="AF11" s="2"/>
+    <row r="11" spans="1:32" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="40" t="s">
+        <v>151</v>
+      </c>
+      <c r="B11" s="38"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="50">
+        <f>AVERAGE(F$10:F10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="51">
+        <f>SUM(G$10:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="50">
+        <f>AVERAGE(H$10:H10)</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="51">
+        <f>SUM(I$10:I10)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="51">
+        <f>SUM(J$10:J10)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="51">
+        <f>SUM(K$10:K10)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="50">
+        <f>AVERAGE(L$10:L10)</f>
+        <v>0</v>
+      </c>
+      <c r="M11" s="50">
+        <f>AVERAGE(M$10:M10)</f>
+        <v>0</v>
+      </c>
+      <c r="N11" s="50">
+        <f>AVERAGE(N$10:N10)</f>
+        <v>0</v>
+      </c>
+      <c r="O11" s="50">
+        <f>AVERAGE(O$10:O10)</f>
+        <v>0</v>
+      </c>
+      <c r="P11" s="51">
+        <f>SUM(P$10:P10)</f>
+        <v>0</v>
+      </c>
+      <c r="Q11" s="51">
+        <f>SUM(Q$10:Q10)</f>
+        <v>0</v>
+      </c>
+      <c r="R11" s="51">
+        <f>SUM(R$10:R10)</f>
+        <v>0</v>
+      </c>
+      <c r="S11" s="50">
+        <f>AVERAGE(S$10:S10)</f>
+        <v>0</v>
+      </c>
+      <c r="T11" s="50" t="e">
+        <f>AVERAGE(T$10:T10)</f>
+        <v>#DIV/0!</v>
+      </c>
+      <c r="U11" s="51">
+        <f>SUM(U$10:U10)</f>
+        <v>0</v>
+      </c>
+      <c r="V11" s="51">
+        <f>SUM(V$10:V10)</f>
+        <v>0</v>
+      </c>
+      <c r="W11" s="51">
+        <f>SUM(W$10:W10)</f>
+        <v>0</v>
+      </c>
+      <c r="X11" s="51">
+        <f>SUM(X$10:X10)</f>
+        <v>0</v>
+      </c>
+      <c r="Y11" s="51">
+        <f>SUM(Y$10:Y10)</f>
+        <v>0</v>
+      </c>
+      <c r="Z11" s="51">
+        <f>SUM(Z$10:Z10)</f>
+        <v>0</v>
+      </c>
+      <c r="AA11" s="51">
+        <f>SUM(AA$10:AA10)</f>
+        <v>0</v>
+      </c>
+      <c r="AB11" s="51">
+        <f>SUM(AB$10:AB10)</f>
+        <v>0</v>
+      </c>
+      <c r="AC11" s="51">
+        <f>SUM(AC$10:AC10)</f>
+        <v>0</v>
+      </c>
+      <c r="AD11" s="51">
+        <f>SUM(AD$10:AD10)</f>
+        <v>0</v>
+      </c>
+      <c r="AE11" s="51">
+        <f>SUM(AE$10:AE10)</f>
+        <v>0</v>
+      </c>
+      <c r="AF11" s="53">
+        <f>SUM(AF$10:AF10)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" spans="1:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="2"/>
@@ -10903,21 +11100,6 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="24">
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="AD8:AD9"/>
     <mergeCell ref="AE8:AE9"/>
     <mergeCell ref="AF8:AF9"/>
     <mergeCell ref="O8:O9"/>
@@ -10927,6 +11109,21 @@
     <mergeCell ref="S8:S9"/>
     <mergeCell ref="T8:T9"/>
     <mergeCell ref="U8:AC8"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="AD8:AD9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
   </mergeCells>
   <conditionalFormatting sqref="H10">
     <cfRule type="notContainsBlanks" dxfId="2" priority="1">
@@ -11004,7 +11201,7 @@
       <c r="L3" s="2"/>
     </row>
     <row r="4" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="14" t="s">
+      <c r="A4" s="11" t="s">
         <v>4</v>
       </c>
       <c r="B4" s="2"/>
@@ -11020,7 +11217,7 @@
       <c r="L4" s="2"/>
     </row>
     <row r="5" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="14" t="s">
+      <c r="A5" s="11" t="s">
         <v>5</v>
       </c>
       <c r="B5" s="2"/>
@@ -11052,7 +11249,7 @@
       <c r="L6" s="2"/>
     </row>
     <row r="7" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="12" t="s">
         <v>7</v>
       </c>
       <c r="B7" s="2">
@@ -11070,110 +11267,146 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="55" t="s">
+      <c r="A8" s="64" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="52" t="s">
+      <c r="B8" s="61" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="53"/>
-      <c r="D8" s="53"/>
-      <c r="E8" s="53"/>
-      <c r="F8" s="53"/>
-      <c r="G8" s="53"/>
-      <c r="H8" s="53"/>
-      <c r="I8" s="53"/>
-      <c r="J8" s="54"/>
-      <c r="K8" s="56" t="s">
+      <c r="C8" s="62"/>
+      <c r="D8" s="62"/>
+      <c r="E8" s="62"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="62"/>
+      <c r="I8" s="62"/>
+      <c r="J8" s="63"/>
+      <c r="K8" s="65" t="s">
         <v>114</v>
       </c>
-      <c r="L8" s="56" t="s">
+      <c r="L8" s="65" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="50"/>
-      <c r="B9" s="16">
+      <c r="A9" s="59"/>
+      <c r="B9" s="13">
         <v>5011</v>
       </c>
-      <c r="C9" s="16">
+      <c r="C9" s="13">
         <v>5007</v>
       </c>
-      <c r="D9" s="16">
+      <c r="D9" s="13">
         <v>5006</v>
       </c>
-      <c r="E9" s="16">
+      <c r="E9" s="13">
         <v>2008</v>
       </c>
-      <c r="F9" s="16">
+      <c r="F9" s="13">
         <v>2005</v>
       </c>
-      <c r="G9" s="16">
+      <c r="G9" s="13">
         <v>2037</v>
       </c>
-      <c r="H9" s="16">
+      <c r="H9" s="13">
         <v>2025</v>
       </c>
-      <c r="I9" s="16">
+      <c r="I9" s="13">
         <v>2022</v>
       </c>
-      <c r="J9" s="16" t="s">
+      <c r="J9" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="K9" s="50"/>
-      <c r="L9" s="50"/>
-    </row>
-    <row r="10" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="23" t="s">
+      <c r="K9" s="59"/>
+      <c r="L9" s="59"/>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="36" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="24" t="s">
+      <c r="B10" s="37" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="37" t="s">
         <v>103</v>
       </c>
-      <c r="D10" s="24" t="s">
+      <c r="D10" s="37" t="s">
         <v>104</v>
       </c>
-      <c r="E10" s="24" t="s">
+      <c r="E10" s="37" t="s">
         <v>105</v>
       </c>
-      <c r="F10" s="24" t="s">
+      <c r="F10" s="37" t="s">
         <v>106</v>
       </c>
-      <c r="G10" s="24" t="s">
+      <c r="G10" s="37" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="24" t="s">
+      <c r="H10" s="37" t="s">
         <v>108</v>
       </c>
-      <c r="I10" s="24" t="s">
+      <c r="I10" s="37" t="s">
         <v>109</v>
       </c>
-      <c r="J10" s="24" t="s">
+      <c r="J10" s="37" t="s">
         <v>110</v>
       </c>
-      <c r="K10" s="24" t="s">
+      <c r="K10" s="37" t="s">
         <v>111</v>
       </c>
-      <c r="L10" s="25" t="e">
+      <c r="L10" s="37" t="e">
         <f>B10+C10+D10+E10+F10+G10+H10+I10+J10+K10</f>
         <v>#VALUE!</v>
       </c>
     </row>
-    <row r="11" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="2"/>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
+    <row r="11" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="40" t="s">
+        <v>151</v>
+      </c>
+      <c r="B11" s="38">
+        <f>SUM(B$10:B10)</f>
+        <v>0</v>
+      </c>
+      <c r="C11" s="38">
+        <f>SUM(C$10:C10)</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="38">
+        <f>SUM(D$10:D10)</f>
+        <v>0</v>
+      </c>
+      <c r="E11" s="38">
+        <f>SUM(E$10:E10)</f>
+        <v>0</v>
+      </c>
+      <c r="F11" s="38">
+        <f>SUM(F$10:F10)</f>
+        <v>0</v>
+      </c>
+      <c r="G11" s="38">
+        <f>SUM(G$10:G10)</f>
+        <v>0</v>
+      </c>
+      <c r="H11" s="38">
+        <f>SUM(H$10:H10)</f>
+        <v>0</v>
+      </c>
+      <c r="I11" s="38">
+        <f>SUM(I$10:I10)</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="38">
+        <f>SUM(J$10:J10)</f>
+        <v>0</v>
+      </c>
+      <c r="K11" s="38">
+        <f>SUM(K$10:K10)</f>
+        <v>0</v>
+      </c>
+      <c r="L11" s="39" t="e">
+        <f>SUM(L$10:L10)</f>
+        <v>#VALUE!</v>
+      </c>
     </row>
     <row r="12" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="2"/>
@@ -14702,299 +14935,299 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="38" t="s">
+      <c r="B2" s="28" t="s">
         <v>115</v>
       </c>
-      <c r="C2" s="38" t="s">
+      <c r="C2" s="28" t="s">
         <v>116</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="28" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="3" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="35">
+      <c r="B3" s="25">
         <v>1001</v>
       </c>
-      <c r="C3" s="36" t="s">
+      <c r="C3" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="D3" s="27" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="4" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B4" s="26">
+      <c r="B4" s="16">
         <v>1002</v>
       </c>
-      <c r="C4" s="27" t="s">
+      <c r="C4" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="18" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="5" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B5" s="32">
+      <c r="B5" s="22">
         <v>1004</v>
       </c>
-      <c r="C5" s="33" t="s">
+      <c r="C5" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="D5" s="34" t="s">
+      <c r="D5" s="24" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="6" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="26">
+      <c r="B6" s="16">
         <v>1005</v>
       </c>
-      <c r="C6" s="27" t="s">
+      <c r="C6" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="D6" s="28" t="s">
+      <c r="D6" s="18" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="7" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="32">
+      <c r="B7" s="22">
         <v>1006</v>
       </c>
-      <c r="C7" s="33" t="s">
+      <c r="C7" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="D7" s="34" t="s">
+      <c r="D7" s="24" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="8" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="26">
+      <c r="B8" s="16">
         <v>1007</v>
       </c>
-      <c r="C8" s="27" t="s">
+      <c r="C8" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="D8" s="28" t="s">
+      <c r="D8" s="18" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="9" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="32">
+      <c r="B9" s="22">
         <v>1017</v>
       </c>
-      <c r="C9" s="33" t="s">
+      <c r="C9" s="23" t="s">
         <v>118</v>
       </c>
-      <c r="D9" s="34" t="s">
+      <c r="D9" s="24" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="10" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="26">
+      <c r="B10" s="16">
         <v>1018</v>
       </c>
-      <c r="C10" s="27" t="s">
+      <c r="C10" s="17" t="s">
         <v>118</v>
       </c>
-      <c r="D10" s="28" t="s">
+      <c r="D10" s="18" t="s">
         <v>126</v>
       </c>
     </row>
     <row r="11" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="32">
+      <c r="B11" s="22">
         <v>2003</v>
       </c>
-      <c r="C11" s="33" t="s">
+      <c r="C11" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="D11" s="34" t="s">
+      <c r="D11" s="24" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="12" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="26">
+      <c r="B12" s="16">
         <v>2005</v>
       </c>
-      <c r="C12" s="27" t="s">
+      <c r="C12" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="D12" s="28" t="s">
+      <c r="D12" s="18" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="13" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="32">
+      <c r="B13" s="22">
         <v>2008</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="D13" s="34" t="s">
+      <c r="D13" s="24" t="s">
         <v>130</v>
       </c>
     </row>
     <row r="14" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="26">
+      <c r="B14" s="16">
         <v>2009</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="D14" s="28" t="s">
+      <c r="D14" s="18" t="s">
         <v>131</v>
       </c>
     </row>
     <row r="15" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="32">
+      <c r="B15" s="22">
         <v>2011</v>
       </c>
-      <c r="C15" s="33" t="s">
+      <c r="C15" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="D15" s="34" t="s">
+      <c r="D15" s="24" t="s">
         <v>133</v>
       </c>
     </row>
     <row r="16" spans="2:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="B16" s="26">
+      <c r="B16" s="16">
         <v>2014</v>
       </c>
-      <c r="C16" s="27" t="s">
+      <c r="C16" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="D16" s="28" t="s">
+      <c r="D16" s="18" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="17" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="32">
+      <c r="B17" s="22">
         <v>2016</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="C17" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="D17" s="34" t="s">
+      <c r="D17" s="24" t="s">
         <v>135</v>
       </c>
     </row>
     <row r="18" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="26">
+      <c r="B18" s="16">
         <v>2018</v>
       </c>
-      <c r="C18" s="27" t="s">
+      <c r="C18" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="D18" s="28" t="s">
+      <c r="D18" s="18" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="19" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B19" s="32">
+      <c r="B19" s="22">
         <v>2022</v>
       </c>
-      <c r="C19" s="33" t="s">
+      <c r="C19" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="D19" s="34" t="s">
+      <c r="D19" s="24" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="20" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B20" s="26">
+      <c r="B20" s="16">
         <v>2025</v>
       </c>
-      <c r="C20" s="27" t="s">
+      <c r="C20" s="17" t="s">
         <v>132</v>
       </c>
-      <c r="D20" s="28" t="s">
+      <c r="D20" s="18" t="s">
         <v>138</v>
       </c>
     </row>
     <row r="21" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="32">
+      <c r="B21" s="22">
         <v>2032</v>
       </c>
-      <c r="C21" s="33" t="s">
+      <c r="C21" s="23" t="s">
         <v>127</v>
       </c>
-      <c r="D21" s="34" t="s">
+      <c r="D21" s="24" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="22" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="26">
+      <c r="B22" s="16">
         <v>2034</v>
       </c>
-      <c r="C22" s="27" t="s">
+      <c r="C22" s="17" t="s">
         <v>127</v>
       </c>
-      <c r="D22" s="28" t="s">
+      <c r="D22" s="18" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="23" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="32">
+      <c r="B23" s="22">
         <v>2037</v>
       </c>
-      <c r="C23" s="33" t="s">
+      <c r="C23" s="23" t="s">
         <v>132</v>
       </c>
-      <c r="D23" s="34" t="s">
+      <c r="D23" s="24" t="s">
         <v>141</v>
       </c>
     </row>
     <row r="24" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="26">
+      <c r="B24" s="16">
         <v>4010</v>
       </c>
-      <c r="C24" s="27" t="s">
+      <c r="C24" s="17" t="s">
         <v>142</v>
       </c>
-      <c r="D24" s="28" t="s">
+      <c r="D24" s="18" t="s">
         <v>143</v>
       </c>
     </row>
     <row r="25" spans="2:4" ht="34" x14ac:dyDescent="0.2">
-      <c r="B25" s="32">
+      <c r="B25" s="22">
         <v>4017</v>
       </c>
-      <c r="C25" s="33" t="s">
+      <c r="C25" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="D25" s="34" t="s">
+      <c r="D25" s="24" t="s">
         <v>134</v>
       </c>
     </row>
     <row r="26" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="26">
+      <c r="B26" s="16">
         <v>5006</v>
       </c>
-      <c r="C26" s="27" t="s">
+      <c r="C26" s="17" t="s">
         <v>144</v>
       </c>
-      <c r="D26" s="28" t="s">
+      <c r="D26" s="18" t="s">
         <v>145</v>
       </c>
     </row>
     <row r="27" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B27" s="32">
+      <c r="B27" s="22">
         <v>5007</v>
       </c>
-      <c r="C27" s="33" t="s">
+      <c r="C27" s="23" t="s">
         <v>144</v>
       </c>
-      <c r="D27" s="34" t="s">
+      <c r="D27" s="24" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="28" spans="2:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B28" s="29">
+      <c r="B28" s="19">
         <v>5011</v>
       </c>
-      <c r="C28" s="30" t="s">
+      <c r="C28" s="20" t="s">
         <v>144</v>
       </c>
-      <c r="D28" s="31" t="s">
+      <c r="D28" s="21" t="s">
         <v>147</v>
       </c>
     </row>

</xml_diff>

<commit_message>
[feat/ASP-7746-Device-and-Sites-Summary-Report-include-Total-line] fixed totals row inner borders
</commit_message>
<xml_diff>
--- a/api/templates/device_and_site_summary_report/en.xlsx
+++ b/api/templates/device_and_site_summary_report/en.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10608"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ahernandez/repos/aspect/api/templates/device_and_site_summary_report/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F0C0E2-5A41-F74E-BBE7-C332410CB92E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24CE3355-3C43-C947-A9BA-88FB4F1EBF9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4340" yWindow="760" windowWidth="30220" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -636,7 +636,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -825,7 +825,9 @@
     </border>
     <border>
       <left/>
-      <right/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
       <top style="medium">
         <color rgb="FF000000"/>
       </top>
@@ -835,7 +837,22 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
         <color rgb="FF000000"/>
       </left>
       <right/>
@@ -848,7 +865,69 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
@@ -860,48 +939,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="67">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -986,27 +1028,14 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -1016,16 +1045,7 @@
     <xf numFmtId="10" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="10" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="2" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="2" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1055,6 +1075,29 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1353,11 +1396,11 @@
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="54" t="s">
+      <c r="E2" s="42" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
       <c r="H2" s="5"/>
       <c r="J2" s="2"/>
       <c r="K2" s="3"/>
@@ -1373,11 +1416,11 @@
       <c r="A3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="56"/>
-      <c r="D3" s="55"/>
-      <c r="E3" s="55"/>
-      <c r="F3" s="55"/>
-      <c r="G3" s="55"/>
+      <c r="C3" s="44"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
       <c r="H3" s="5"/>
       <c r="J3" s="2"/>
       <c r="K3" s="3"/>
@@ -1393,9 +1436,9 @@
       <c r="A4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="55"/>
-      <c r="F4" s="55"/>
-      <c r="G4" s="55"/>
+      <c r="E4" s="43"/>
+      <c r="F4" s="43"/>
+      <c r="G4" s="43"/>
       <c r="H4" s="5"/>
       <c r="J4" s="2"/>
       <c r="K4" s="3"/>
@@ -1411,9 +1454,9 @@
       <c r="A5" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="55"/>
-      <c r="F5" s="55"/>
-      <c r="G5" s="55"/>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="43"/>
       <c r="H5" s="5"/>
       <c r="J5" s="2"/>
       <c r="K5" s="3"/>
@@ -1429,9 +1472,9 @@
       <c r="A6" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="E6" s="55"/>
-      <c r="F6" s="55"/>
-      <c r="G6" s="55"/>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
       <c r="J6" s="2"/>
       <c r="K6" s="3"/>
       <c r="L6" s="2"/>
@@ -1583,31 +1626,31 @@
       </c>
     </row>
     <row r="10" spans="1:21" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="35" t="s">
+      <c r="A10" s="54" t="s">
         <v>151</v>
       </c>
-      <c r="B10" s="34"/>
-      <c r="C10" s="34"/>
-      <c r="D10" s="34"/>
-      <c r="E10" s="34"/>
-      <c r="F10" s="34"/>
-      <c r="G10" s="34"/>
-      <c r="H10" s="34"/>
-      <c r="I10" s="34"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="34"/>
-      <c r="L10" s="34"/>
-      <c r="M10" s="34"/>
-      <c r="N10" s="34"/>
-      <c r="O10" s="34"/>
-      <c r="P10" s="34"/>
-      <c r="Q10" s="34"/>
-      <c r="R10" s="34"/>
-      <c r="S10" s="34">
+      <c r="B10" s="55"/>
+      <c r="C10" s="55"/>
+      <c r="D10" s="55"/>
+      <c r="E10" s="55"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="55"/>
+      <c r="J10" s="55"/>
+      <c r="K10" s="55"/>
+      <c r="L10" s="55"/>
+      <c r="M10" s="55"/>
+      <c r="N10" s="55"/>
+      <c r="O10" s="55"/>
+      <c r="P10" s="55"/>
+      <c r="Q10" s="55"/>
+      <c r="R10" s="55"/>
+      <c r="S10" s="55">
         <f>SUM(S$9:S9)</f>
         <v>0</v>
       </c>
-      <c r="T10" s="34">
+      <c r="T10" s="56">
         <f>SUM(T$9:T9)</f>
         <v>0</v>
       </c>
@@ -1657,13 +1700,13 @@
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="57" t="s">
+      <c r="C2" s="45" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="55"/>
-      <c r="E2" s="55"/>
-      <c r="F2" s="55"/>
-      <c r="G2" s="55"/>
+      <c r="D2" s="43"/>
+      <c r="E2" s="43"/>
+      <c r="F2" s="43"/>
+      <c r="G2" s="43"/>
     </row>
     <row r="3" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4" t="s">
@@ -1724,64 +1767,64 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="41" t="s">
+      <c r="A9" s="36" t="s">
         <v>58</v>
       </c>
-      <c r="B9" s="41" t="s">
+      <c r="B9" s="36" t="s">
         <v>59</v>
       </c>
-      <c r="C9" s="47" t="s">
+      <c r="C9" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="D9" s="41" t="s">
+      <c r="D9" s="36" t="s">
         <v>61</v>
       </c>
-      <c r="E9" s="41" t="s">
+      <c r="E9" s="36" t="s">
         <v>62</v>
       </c>
-      <c r="F9" s="41" t="s">
+      <c r="F9" s="36" t="s">
         <v>63</v>
       </c>
-      <c r="G9" s="41" t="s">
+      <c r="G9" s="36" t="s">
         <v>64</v>
       </c>
-      <c r="H9" s="41" t="s">
+      <c r="H9" s="36" t="s">
         <v>65</v>
       </c>
-      <c r="I9" s="42" t="s">
+      <c r="I9" s="37" t="s">
         <v>149</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="43" t="s">
+      <c r="A10" s="57" t="s">
         <v>151</v>
       </c>
-      <c r="B10" s="44"/>
-      <c r="C10" s="46" t="e">
+      <c r="B10" s="58"/>
+      <c r="C10" s="59" t="e">
         <f>AVERAGE(C$9:C9)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="D10" s="44">
+      <c r="D10" s="58">
         <f>SUM(D$9:D9)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="44">
+      <c r="E10" s="58">
         <f>SUM(E$9:E9)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="44">
+      <c r="F10" s="58">
         <f>SUM(F$9:F9)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="46" t="e">
+      <c r="G10" s="59" t="e">
         <f>AVERAGE(G$9:G9)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="H10" s="44">
+      <c r="H10" s="58">
         <f>SUM(H$9:H9)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="45">
+      <c r="I10" s="60">
         <f>SUM(I$9:I9)</f>
         <v>0</v>
       </c>
@@ -3064,108 +3107,108 @@
       <c r="AF7" s="2"/>
     </row>
     <row r="8" spans="1:32" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="58" t="s">
+      <c r="A8" s="46" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="60" t="s">
+      <c r="B8" s="48" t="s">
         <v>67</v>
       </c>
-      <c r="C8" s="60" t="s">
+      <c r="C8" s="48" t="s">
         <v>68</v>
       </c>
-      <c r="D8" s="60" t="s">
+      <c r="D8" s="48" t="s">
         <v>69</v>
       </c>
-      <c r="E8" s="60" t="s">
+      <c r="E8" s="48" t="s">
         <v>70</v>
       </c>
-      <c r="F8" s="60" t="s">
+      <c r="F8" s="48" t="s">
         <v>71</v>
       </c>
-      <c r="G8" s="60" t="s">
+      <c r="G8" s="48" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="60" t="s">
+      <c r="H8" s="48" t="s">
         <v>73</v>
       </c>
-      <c r="I8" s="60" t="s">
+      <c r="I8" s="48" t="s">
         <v>74</v>
       </c>
-      <c r="J8" s="60" t="s">
+      <c r="J8" s="48" t="s">
         <v>75</v>
       </c>
-      <c r="K8" s="60" t="s">
+      <c r="K8" s="48" t="s">
         <v>76</v>
       </c>
-      <c r="L8" s="60" t="s">
+      <c r="L8" s="48" t="s">
         <v>77</v>
       </c>
-      <c r="M8" s="60" t="s">
+      <c r="M8" s="48" t="s">
         <v>78</v>
       </c>
-      <c r="N8" s="60" t="s">
+      <c r="N8" s="48" t="s">
         <v>79</v>
       </c>
-      <c r="O8" s="60" t="s">
+      <c r="O8" s="48" t="s">
         <v>80</v>
       </c>
-      <c r="P8" s="60" t="s">
+      <c r="P8" s="48" t="s">
         <v>81</v>
       </c>
-      <c r="Q8" s="60" t="s">
+      <c r="Q8" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="R8" s="60" t="s">
+      <c r="R8" s="48" t="s">
         <v>83</v>
       </c>
-      <c r="S8" s="60" t="s">
+      <c r="S8" s="48" t="s">
         <v>84</v>
       </c>
-      <c r="T8" s="60" t="s">
+      <c r="T8" s="48" t="s">
         <v>85</v>
       </c>
-      <c r="U8" s="61" t="s">
+      <c r="U8" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="V8" s="62"/>
-      <c r="W8" s="62"/>
-      <c r="X8" s="62"/>
-      <c r="Y8" s="62"/>
-      <c r="Z8" s="62"/>
-      <c r="AA8" s="62"/>
-      <c r="AB8" s="62"/>
-      <c r="AC8" s="63"/>
-      <c r="AD8" s="58" t="s">
+      <c r="V8" s="50"/>
+      <c r="W8" s="50"/>
+      <c r="X8" s="50"/>
+      <c r="Y8" s="50"/>
+      <c r="Z8" s="50"/>
+      <c r="AA8" s="50"/>
+      <c r="AB8" s="50"/>
+      <c r="AC8" s="51"/>
+      <c r="AD8" s="46" t="s">
         <v>87</v>
       </c>
-      <c r="AE8" s="58" t="s">
+      <c r="AE8" s="46" t="s">
         <v>88</v>
       </c>
-      <c r="AF8" s="58" t="s">
+      <c r="AF8" s="46" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:32" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="59"/>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
-      <c r="M9" s="59"/>
-      <c r="N9" s="59"/>
-      <c r="O9" s="59"/>
-      <c r="P9" s="59"/>
-      <c r="Q9" s="59"/>
-      <c r="R9" s="59"/>
-      <c r="S9" s="59"/>
-      <c r="T9" s="59"/>
+      <c r="A9" s="47"/>
+      <c r="B9" s="47"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="47"/>
+      <c r="E9" s="47"/>
+      <c r="F9" s="47"/>
+      <c r="G9" s="47"/>
+      <c r="H9" s="47"/>
+      <c r="I9" s="47"/>
+      <c r="J9" s="47"/>
+      <c r="K9" s="47"/>
+      <c r="L9" s="47"/>
+      <c r="M9" s="47"/>
+      <c r="N9" s="47"/>
+      <c r="O9" s="47"/>
+      <c r="P9" s="47"/>
+      <c r="Q9" s="47"/>
+      <c r="R9" s="47"/>
+      <c r="S9" s="47"/>
+      <c r="T9" s="47"/>
       <c r="U9" s="13">
         <v>5011</v>
       </c>
@@ -3193,230 +3236,230 @@
       <c r="AC9" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="AD9" s="59"/>
-      <c r="AE9" s="59"/>
-      <c r="AF9" s="59"/>
+      <c r="AD9" s="47"/>
+      <c r="AE9" s="47"/>
+      <c r="AF9" s="47"/>
     </row>
     <row r="10" spans="1:32" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="35" t="s">
         <v>92</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="35" t="s">
         <v>93</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="35" t="s">
         <v>94</v>
       </c>
-      <c r="E10" s="37" t="s">
+      <c r="E10" s="35" t="s">
         <v>95</v>
       </c>
-      <c r="F10" s="48">
+      <c r="F10" s="39">
         <f>IFERROR(IF(A10="No data","",IF(C10=0,0,D10/C10)),0)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="37" t="s">
+      <c r="G10" s="35" t="s">
         <v>46</v>
       </c>
-      <c r="H10" s="49">
+      <c r="H10" s="40">
         <f>IFERROR(IF(A10="No data","",IF(B10&lt;&gt;0, G10/B10, 0)),0)</f>
         <v>0</v>
       </c>
-      <c r="I10" s="37" t="s">
+      <c r="I10" s="35" t="s">
         <v>96</v>
       </c>
-      <c r="J10" s="37" t="s">
+      <c r="J10" s="35" t="s">
         <v>97</v>
       </c>
-      <c r="K10" s="37">
+      <c r="K10" s="35">
         <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10),0)</f>
         <v>0</v>
       </c>
-      <c r="L10" s="48">
+      <c r="L10" s="39">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,I10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="M10" s="48">
+      <c r="M10" s="39">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,J10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="N10" s="48">
+      <c r="N10" s="39">
         <f>IFERROR(IF(A10="No data","",IF(D10=0,0,I10/D10)),0)</f>
         <v>0</v>
       </c>
-      <c r="O10" s="48">
+      <c r="O10" s="39">
         <f>IFERROR(IF(A10="No data","",IF(G10=0,0,K10/G10)),0)</f>
         <v>0</v>
       </c>
-      <c r="P10" s="37" t="s">
+      <c r="P10" s="35" t="s">
         <v>98</v>
       </c>
-      <c r="Q10" s="37" t="s">
+      <c r="Q10" s="35" t="s">
         <v>99</v>
       </c>
-      <c r="R10" s="37" t="s">
+      <c r="R10" s="35" t="s">
         <v>100</v>
       </c>
-      <c r="S10" s="48">
+      <c r="S10" s="39">
         <f>IFERROR(IF(A10="No data","",IF(I10=0,0,R10/I10)),0)</f>
         <v>0</v>
       </c>
-      <c r="T10" s="52" t="s">
+      <c r="T10" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="U10" s="37" t="s">
+      <c r="U10" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="V10" s="37" t="s">
+      <c r="V10" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="W10" s="37" t="s">
+      <c r="W10" s="35" t="s">
         <v>104</v>
       </c>
-      <c r="X10" s="37" t="s">
+      <c r="X10" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="Y10" s="37" t="s">
+      <c r="Y10" s="35" t="s">
         <v>106</v>
       </c>
-      <c r="Z10" s="37" t="s">
+      <c r="Z10" s="35" t="s">
         <v>107</v>
       </c>
-      <c r="AA10" s="37" t="s">
+      <c r="AA10" s="35" t="s">
         <v>108</v>
       </c>
-      <c r="AB10" s="37" t="s">
+      <c r="AB10" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="AC10" s="37" t="s">
+      <c r="AC10" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="AD10" s="37" t="s">
+      <c r="AD10" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="AE10" s="37" t="s">
+      <c r="AE10" s="35" t="s">
         <v>112</v>
       </c>
-      <c r="AF10" s="37">
+      <c r="AF10" s="35">
         <f>IFERROR(IF(A10="No data","",U10+V10+W10+X10+Y10+Z10+AA10+AB10+AC10+AD10+AE10),0)</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:32" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="61" t="s">
         <v>151</v>
       </c>
-      <c r="B11" s="38"/>
-      <c r="C11" s="38"/>
-      <c r="D11" s="38"/>
-      <c r="E11" s="38"/>
-      <c r="F11" s="50">
+      <c r="B11" s="62"/>
+      <c r="C11" s="62"/>
+      <c r="D11" s="62"/>
+      <c r="E11" s="62"/>
+      <c r="F11" s="63">
         <f>AVERAGE(F$10:F10)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="51">
+      <c r="G11" s="64">
         <f>SUM(G$10:G10)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="50">
+      <c r="H11" s="63">
         <f>AVERAGE(H$10:H10)</f>
         <v>0</v>
       </c>
-      <c r="I11" s="51">
+      <c r="I11" s="64">
         <f>SUM(I$10:I10)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="51">
+      <c r="J11" s="64">
         <f>SUM(J$10:J10)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="51">
+      <c r="K11" s="64">
         <f>SUM(K$10:K10)</f>
         <v>0</v>
       </c>
-      <c r="L11" s="50">
+      <c r="L11" s="63">
         <f>AVERAGE(L$10:L10)</f>
         <v>0</v>
       </c>
-      <c r="M11" s="50">
+      <c r="M11" s="63">
         <f>AVERAGE(M$10:M10)</f>
         <v>0</v>
       </c>
-      <c r="N11" s="50">
+      <c r="N11" s="63">
         <f>AVERAGE(N$10:N10)</f>
         <v>0</v>
       </c>
-      <c r="O11" s="50">
+      <c r="O11" s="63">
         <f>AVERAGE(O$10:O10)</f>
         <v>0</v>
       </c>
-      <c r="P11" s="51">
+      <c r="P11" s="64">
         <f>SUM(P$10:P10)</f>
         <v>0</v>
       </c>
-      <c r="Q11" s="51">
+      <c r="Q11" s="64">
         <f>SUM(Q$10:Q10)</f>
         <v>0</v>
       </c>
-      <c r="R11" s="51">
+      <c r="R11" s="64">
         <f>SUM(R$10:R10)</f>
         <v>0</v>
       </c>
-      <c r="S11" s="50">
+      <c r="S11" s="63">
         <f>AVERAGE(S$10:S10)</f>
         <v>0</v>
       </c>
-      <c r="T11" s="50" t="e">
+      <c r="T11" s="63" t="e">
         <f>AVERAGE(T$10:T10)</f>
         <v>#DIV/0!</v>
       </c>
-      <c r="U11" s="51">
+      <c r="U11" s="64">
         <f>SUM(U$10:U10)</f>
         <v>0</v>
       </c>
-      <c r="V11" s="51">
+      <c r="V11" s="64">
         <f>SUM(V$10:V10)</f>
         <v>0</v>
       </c>
-      <c r="W11" s="51">
+      <c r="W11" s="64">
         <f>SUM(W$10:W10)</f>
         <v>0</v>
       </c>
-      <c r="X11" s="51">
+      <c r="X11" s="64">
         <f>SUM(X$10:X10)</f>
         <v>0</v>
       </c>
-      <c r="Y11" s="51">
+      <c r="Y11" s="64">
         <f>SUM(Y$10:Y10)</f>
         <v>0</v>
       </c>
-      <c r="Z11" s="51">
+      <c r="Z11" s="64">
         <f>SUM(Z$10:Z10)</f>
         <v>0</v>
       </c>
-      <c r="AA11" s="51">
+      <c r="AA11" s="64">
         <f>SUM(AA$10:AA10)</f>
         <v>0</v>
       </c>
-      <c r="AB11" s="51">
+      <c r="AB11" s="64">
         <f>SUM(AB$10:AB10)</f>
         <v>0</v>
       </c>
-      <c r="AC11" s="51">
+      <c r="AC11" s="64">
         <f>SUM(AC$10:AC10)</f>
         <v>0</v>
       </c>
-      <c r="AD11" s="51">
+      <c r="AD11" s="64">
         <f>SUM(AD$10:AD10)</f>
         <v>0</v>
       </c>
-      <c r="AE11" s="51">
+      <c r="AE11" s="64">
         <f>SUM(AE$10:AE10)</f>
         <v>0</v>
       </c>
-      <c r="AF11" s="53">
+      <c r="AF11" s="65">
         <f>SUM(AF$10:AF10)</f>
         <v>0</v>
       </c>
@@ -11100,6 +11143,21 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="A8:A9"/>
+    <mergeCell ref="B8:B9"/>
+    <mergeCell ref="C8:C9"/>
+    <mergeCell ref="D8:D9"/>
+    <mergeCell ref="E8:E9"/>
+    <mergeCell ref="F8:F9"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="H8:H9"/>
+    <mergeCell ref="I8:I9"/>
+    <mergeCell ref="J8:J9"/>
+    <mergeCell ref="K8:K9"/>
+    <mergeCell ref="L8:L9"/>
+    <mergeCell ref="M8:M9"/>
+    <mergeCell ref="N8:N9"/>
+    <mergeCell ref="AD8:AD9"/>
     <mergeCell ref="AE8:AE9"/>
     <mergeCell ref="AF8:AF9"/>
     <mergeCell ref="O8:O9"/>
@@ -11109,21 +11167,6 @@
     <mergeCell ref="S8:S9"/>
     <mergeCell ref="T8:T9"/>
     <mergeCell ref="U8:AC8"/>
-    <mergeCell ref="K8:K9"/>
-    <mergeCell ref="L8:L9"/>
-    <mergeCell ref="M8:M9"/>
-    <mergeCell ref="N8:N9"/>
-    <mergeCell ref="AD8:AD9"/>
-    <mergeCell ref="F8:F9"/>
-    <mergeCell ref="G8:G9"/>
-    <mergeCell ref="H8:H9"/>
-    <mergeCell ref="I8:I9"/>
-    <mergeCell ref="J8:J9"/>
-    <mergeCell ref="A8:A9"/>
-    <mergeCell ref="B8:B9"/>
-    <mergeCell ref="C8:C9"/>
-    <mergeCell ref="D8:D9"/>
-    <mergeCell ref="E8:E9"/>
   </mergeCells>
   <conditionalFormatting sqref="H10">
     <cfRule type="notContainsBlanks" dxfId="2" priority="1">
@@ -11267,29 +11310,29 @@
       <c r="L7" s="2"/>
     </row>
     <row r="8" spans="1:12" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="64" t="s">
+      <c r="A8" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="61" t="s">
+      <c r="B8" s="49" t="s">
         <v>86</v>
       </c>
-      <c r="C8" s="62"/>
-      <c r="D8" s="62"/>
-      <c r="E8" s="62"/>
-      <c r="F8" s="62"/>
-      <c r="G8" s="62"/>
-      <c r="H8" s="62"/>
-      <c r="I8" s="62"/>
-      <c r="J8" s="63"/>
-      <c r="K8" s="65" t="s">
+      <c r="C8" s="50"/>
+      <c r="D8" s="50"/>
+      <c r="E8" s="50"/>
+      <c r="F8" s="50"/>
+      <c r="G8" s="50"/>
+      <c r="H8" s="50"/>
+      <c r="I8" s="50"/>
+      <c r="J8" s="51"/>
+      <c r="K8" s="53" t="s">
         <v>114</v>
       </c>
-      <c r="L8" s="65" t="s">
+      <c r="L8" s="53" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:12" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="59"/>
+      <c r="A9" s="47"/>
       <c r="B9" s="13">
         <v>5011</v>
       </c>
@@ -11317,93 +11360,93 @@
       <c r="J9" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
+      <c r="K9" s="47"/>
+      <c r="L9" s="47"/>
     </row>
     <row r="10" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="36" t="s">
+      <c r="A10" s="34" t="s">
         <v>91</v>
       </c>
-      <c r="B10" s="37" t="s">
+      <c r="B10" s="35" t="s">
         <v>102</v>
       </c>
-      <c r="C10" s="37" t="s">
+      <c r="C10" s="35" t="s">
         <v>103</v>
       </c>
-      <c r="D10" s="37" t="s">
+      <c r="D10" s="35" t="s">
         <v>104</v>
       </c>
-      <c r="E10" s="37" t="s">
+      <c r="E10" s="35" t="s">
         <v>105</v>
       </c>
-      <c r="F10" s="37" t="s">
+      <c r="F10" s="35" t="s">
         <v>106</v>
       </c>
-      <c r="G10" s="37" t="s">
+      <c r="G10" s="35" t="s">
         <v>107</v>
       </c>
-      <c r="H10" s="37" t="s">
+      <c r="H10" s="35" t="s">
         <v>108</v>
       </c>
-      <c r="I10" s="37" t="s">
+      <c r="I10" s="35" t="s">
         <v>109</v>
       </c>
-      <c r="J10" s="37" t="s">
+      <c r="J10" s="35" t="s">
         <v>110</v>
       </c>
-      <c r="K10" s="37" t="s">
+      <c r="K10" s="35" t="s">
         <v>111</v>
       </c>
-      <c r="L10" s="37" t="e">
+      <c r="L10" s="35" t="e">
         <f>B10+C10+D10+E10+F10+G10+H10+I10+J10+K10</f>
         <v>#VALUE!</v>
       </c>
     </row>
     <row r="11" spans="1:12" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="40" t="s">
+      <c r="A11" s="61" t="s">
         <v>151</v>
       </c>
-      <c r="B11" s="38">
+      <c r="B11" s="62">
         <f>SUM(B$10:B10)</f>
         <v>0</v>
       </c>
-      <c r="C11" s="38">
+      <c r="C11" s="62">
         <f>SUM(C$10:C10)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="38">
+      <c r="D11" s="62">
         <f>SUM(D$10:D10)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="38">
+      <c r="E11" s="62">
         <f>SUM(E$10:E10)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="38">
+      <c r="F11" s="62">
         <f>SUM(F$10:F10)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="38">
+      <c r="G11" s="62">
         <f>SUM(G$10:G10)</f>
         <v>0</v>
       </c>
-      <c r="H11" s="38">
+      <c r="H11" s="62">
         <f>SUM(H$10:H10)</f>
         <v>0</v>
       </c>
-      <c r="I11" s="38">
+      <c r="I11" s="62">
         <f>SUM(I$10:I10)</f>
         <v>0</v>
       </c>
-      <c r="J11" s="38">
+      <c r="J11" s="62">
         <f>SUM(J$10:J10)</f>
         <v>0</v>
       </c>
-      <c r="K11" s="38">
+      <c r="K11" s="62">
         <f>SUM(K$10:K10)</f>
         <v>0</v>
       </c>
-      <c r="L11" s="39" t="e">
+      <c r="L11" s="66" t="e">
         <f>SUM(L$10:L10)</f>
         <v>#VALUE!</v>
       </c>

</xml_diff>